<commit_message>
fix: align workbook status contract
</commit_message>
<xml_diff>
--- a/skills/cross-market-product-selection/assets/通用选品数据库模板.xlsx
+++ b/skills/cross-market-product-selection/assets/通用选品数据库模板.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务说明" sheetId="1" r:id="R8cb07507d02f42cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="亚马逊候选" sheetId="2" r:id="R33f9c3a136aa47f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1688候选" sheetId="3" r:id="R0696c0f4f9fa4aea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="货源匹配" sheetId="4" r:id="R0a3dc8c0eb554dcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="严格结果" sheetId="5" r:id="Ra76c4347cc514d2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待核验" sheetId="6" r:id="Rf682de7e699b4bb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="7" r:id="R7eb4dcbeb419483f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务说明" sheetId="1" r:id="R9cdd62639868445b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="亚马逊候选" sheetId="2" r:id="R8c4a20e8d8904ea1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1688候选" sheetId="3" r:id="Rafda571c307b4bfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="货源匹配" sheetId="4" r:id="R87290987b1514d9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="严格结果" sheetId="5" r:id="Rdc1caca4ce4d4d36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待核验" sheetId="6" r:id="R063a361ef0654cdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="7" r:id="Rc789b94d494f46c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1272,7 +1272,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R847e18d178834951"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R302810121ffa455a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1563,18 +1563,18 @@
     <x:mergeCell ref="A2:AJ2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:A103">
-    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="严格"/>
+    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="严格合格"/>
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="待核验"/>
-    <x:cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="淘汰"/>
+    <x:cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="已淘汰"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="A4:A103">
-      <x:formula1>"严格,待核验,淘汰"</x:formula1>
+      <x:formula1>"严格合格,待核验,已淘汰"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd7b55099b9b4550"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb267765dabef4a28"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1900,18 +1900,18 @@
     <x:mergeCell ref="A2:AO2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:A103">
-    <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="严格"/>
+    <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="严格合格"/>
     <x:cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="待核验"/>
-    <x:cfRule type="containsText" dxfId="7" priority="3" operator="containsText" text="淘汰"/>
+    <x:cfRule type="containsText" dxfId="7" priority="3" operator="containsText" text="已淘汰"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="A4:A103">
-      <x:formula1>"严格,待核验,淘汰"</x:formula1>
+      <x:formula1>"严格合格,待核验,已淘汰"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2162b0560fa240cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R508cab8a9f3f4655"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2258,18 +2258,18 @@
     <x:mergeCell ref="A2:AR2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:A103">
-    <x:cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="严格"/>
+    <x:cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="严格合格"/>
     <x:cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="待核验"/>
-    <x:cfRule type="containsText" dxfId="10" priority="3" operator="containsText" text="淘汰"/>
+    <x:cfRule type="containsText" dxfId="10" priority="3" operator="containsText" text="已淘汰"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="A4:A103">
-      <x:formula1>"严格,待核验,淘汰"</x:formula1>
+      <x:formula1>"严格合格,待核验,已淘汰"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c3ee1ffe75b4520"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ac71bf7a6c94769"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2609,18 +2609,18 @@
     <x:mergeCell ref="A2:AQ2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:A103">
-    <x:cfRule type="containsText" dxfId="11" priority="1" operator="containsText" text="严格"/>
+    <x:cfRule type="containsText" dxfId="11" priority="1" operator="containsText" text="严格合格"/>
     <x:cfRule type="containsText" dxfId="12" priority="2" operator="containsText" text="待核验"/>
-    <x:cfRule type="containsText" dxfId="13" priority="3" operator="containsText" text="淘汰"/>
+    <x:cfRule type="containsText" dxfId="13" priority="3" operator="containsText" text="已淘汰"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="A4:A103">
-      <x:formula1>"严格,待核验,淘汰"</x:formula1>
+      <x:formula1>"严格合格,待核验,已淘汰"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fbaef412f734278"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1be8661258943df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2775,18 +2775,18 @@
     <x:mergeCell ref="A2:R2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:A103">
-    <x:cfRule type="containsText" dxfId="14" priority="1" operator="containsText" text="严格"/>
+    <x:cfRule type="containsText" dxfId="14" priority="1" operator="containsText" text="严格合格"/>
     <x:cfRule type="containsText" dxfId="15" priority="2" operator="containsText" text="待核验"/>
-    <x:cfRule type="containsText" dxfId="16" priority="3" operator="containsText" text="淘汰"/>
+    <x:cfRule type="containsText" dxfId="16" priority="3" operator="containsText" text="已淘汰"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="A4:A103">
-      <x:formula1>"严格,待核验,淘汰"</x:formula1>
+      <x:formula1>"严格合格,待核验,已淘汰"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf59e94767ade410b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00a395b9b686499a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2920,18 +2920,18 @@
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:A103">
-    <x:cfRule type="containsText" dxfId="17" priority="1" operator="containsText" text="严格"/>
+    <x:cfRule type="containsText" dxfId="17" priority="1" operator="containsText" text="严格合格"/>
     <x:cfRule type="containsText" dxfId="18" priority="2" operator="containsText" text="待核验"/>
-    <x:cfRule type="containsText" dxfId="19" priority="3" operator="containsText" text="淘汰"/>
+    <x:cfRule type="containsText" dxfId="19" priority="3" operator="containsText" text="已淘汰"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="A4:A103">
-      <x:formula1>"严格,待核验,淘汰"</x:formula1>
+      <x:formula1>"严格合格,待核验,已淘汰"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf185c7eabeb4155"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8cc880b360840c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: harden product and price identity checks
</commit_message>
<xml_diff>
--- a/skills/cross-market-product-selection/assets/通用选品数据库模板.xlsx
+++ b/skills/cross-market-product-selection/assets/通用选品数据库模板.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务说明" sheetId="1" r:id="R933399172898494f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目标产品" sheetId="2" r:id="Rc5bb22af6c59488b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="价格基准" sheetId="3" r:id="Rd90a633098ee4fad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="亚马逊候选" sheetId="4" r:id="R26a7e9dd50cc4c52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1688候选" sheetId="5" r:id="R7ac0af3b8bca442b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="货源匹配" sheetId="6" r:id="R5441cc55c5044abf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="严格结果" sheetId="7" r:id="Rcbc297c5fa8a43c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待核验" sheetId="8" r:id="R5e4b8466199c4500"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="9" r:id="R4bc0279e04db46d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务说明" sheetId="1" r:id="R970c4048668544a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目标产品" sheetId="2" r:id="R0a796489e12a4468"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="价格基准" sheetId="3" r:id="Rdf9e9a186d394aae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="亚马逊候选" sheetId="4" r:id="R86727b9705334f8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1688候选" sheetId="5" r:id="Raf98f3a3f0a24573"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="货源匹配" sheetId="6" r:id="Ra87d0c801a324add"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="严格结果" sheetId="7" r:id="R453561ab9ad242da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待核验" sheetId="8" r:id="Ree2cbd2e1cd442c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="9" r:id="R436cc4400f96422b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -415,9 +415,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TargetProductsTable" displayName="TargetProductsTable" ref="A3:W4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A3:W4"/>
-  <x:tableColumns count="23">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TargetProductsTable" displayName="TargetProductsTable" ref="A3:X4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:X4"/>
+  <x:tableColumns count="24">
     <x:tableColumn id="1" name="目标产品ID"/>
     <x:tableColumn id="2" name="目标产品名称"/>
     <x:tableColumn id="3" name="用户确认状态"/>
@@ -435,12 +435,13 @@
     <x:tableColumn id="15" name="Amazon价格允许偏差"/>
     <x:tableColumn id="16" name="Amazon同类均价"/>
     <x:tableColumn id="17" name="Amazon同类均价最低样本数"/>
-    <x:tableColumn id="18" name="1688目标成本"/>
-    <x:tableColumn id="19" name="1688价格允许偏差"/>
-    <x:tableColumn id="20" name="采购数量档位"/>
-    <x:tableColumn id="21" name="目标严格合格数量"/>
-    <x:tableColumn id="22" name="Amazon目标币种"/>
-    <x:tableColumn id="23" name="1688成本币种"/>
+    <x:tableColumn id="18" name="Amazon目标站点"/>
+    <x:tableColumn id="19" name="1688目标成本"/>
+    <x:tableColumn id="20" name="1688价格允许偏差"/>
+    <x:tableColumn id="21" name="采购数量档位"/>
+    <x:tableColumn id="22" name="目标严格合格数量"/>
+    <x:tableColumn id="23" name="Amazon目标币种"/>
+    <x:tableColumn id="24" name="1688成本币种"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -582,9 +583,9 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="SourceMatchesTable" displayName="SourceMatchesTable" ref="A3:BF4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A3:BF4"/>
-  <x:tableColumns count="58">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="SourceMatchesTable" displayName="SourceMatchesTable" ref="A3:BI4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:BI4"/>
+  <x:tableColumns count="61">
     <x:tableColumn id="1" name="状态"/>
     <x:tableColumn id="2" name="模式"/>
     <x:tableColumn id="3" name="目标产品ID"/>
@@ -613,36 +614,39 @@
     <x:tableColumn id="26" name="外观门槛"/>
     <x:tableColumn id="27" name="功能门槛"/>
     <x:tableColumn id="28" name="价格/MOQ门槛"/>
-    <x:tableColumn id="29" name="采购数量档位"/>
-    <x:tableColumn id="30" name="MOQ"/>
-    <x:tableColumn id="31" name="阶梯价"/>
-    <x:tableColumn id="32" name="详情身份门槛"/>
-    <x:tableColumn id="33" name="供应商门槛"/>
-    <x:tableColumn id="34" name="生产能力门槛"/>
-    <x:tableColumn id="35" name="ODM/OEM/定制门槛"/>
-    <x:tableColumn id="36" name="证据一致性门槛"/>
-    <x:tableColumn id="37" name="外观逐项核验"/>
-    <x:tableColumn id="38" name="功能逐项核验"/>
-    <x:tableColumn id="39" name="市场机会得分"/>
-    <x:tableColumn id="40" name="市场机会结论"/>
-    <x:tableColumn id="41" name="市场机会证据"/>
-    <x:tableColumn id="42" name="供应能力得分"/>
-    <x:tableColumn id="43" name="供应能力结论"/>
-    <x:tableColumn id="44" name="供应能力证据"/>
-    <x:tableColumn id="45" name="匹配质量得分"/>
-    <x:tableColumn id="46" name="匹配质量结论"/>
-    <x:tableColumn id="47" name="匹配质量证据"/>
-    <x:tableColumn id="48" name="最终配对得分"/>
-    <x:tableColumn id="49" name="生产能力证据"/>
-    <x:tableColumn id="50" name="ODM/OEM/定制证据"/>
-    <x:tableColumn id="51" name="主要限制"/>
-    <x:tableColumn id="52" name="来源类型"/>
-    <x:tableColumn id="53" name="来源链接"/>
-    <x:tableColumn id="54" name="检索路径"/>
-    <x:tableColumn id="55" name="获取时间"/>
-    <x:tableColumn id="56" name="置信度"/>
-    <x:tableColumn id="57" name="冲突说明"/>
-    <x:tableColumn id="58" name="决策日志引用"/>
+    <x:tableColumn id="29" name="目标成本"/>
+    <x:tableColumn id="30" name="实际单价"/>
+    <x:tableColumn id="31" name="成本币种"/>
+    <x:tableColumn id="32" name="采购数量档位"/>
+    <x:tableColumn id="33" name="MOQ"/>
+    <x:tableColumn id="34" name="阶梯价"/>
+    <x:tableColumn id="35" name="详情身份门槛"/>
+    <x:tableColumn id="36" name="供应商门槛"/>
+    <x:tableColumn id="37" name="生产能力门槛"/>
+    <x:tableColumn id="38" name="ODM/OEM/定制门槛"/>
+    <x:tableColumn id="39" name="证据一致性门槛"/>
+    <x:tableColumn id="40" name="外观逐项核验"/>
+    <x:tableColumn id="41" name="功能逐项核验"/>
+    <x:tableColumn id="42" name="市场机会得分"/>
+    <x:tableColumn id="43" name="市场机会结论"/>
+    <x:tableColumn id="44" name="市场机会证据"/>
+    <x:tableColumn id="45" name="供应能力得分"/>
+    <x:tableColumn id="46" name="供应能力结论"/>
+    <x:tableColumn id="47" name="供应能力证据"/>
+    <x:tableColumn id="48" name="匹配质量得分"/>
+    <x:tableColumn id="49" name="匹配质量结论"/>
+    <x:tableColumn id="50" name="匹配质量证据"/>
+    <x:tableColumn id="51" name="最终配对得分"/>
+    <x:tableColumn id="52" name="生产能力证据"/>
+    <x:tableColumn id="53" name="ODM/OEM/定制证据"/>
+    <x:tableColumn id="54" name="主要限制"/>
+    <x:tableColumn id="55" name="来源类型"/>
+    <x:tableColumn id="56" name="来源链接"/>
+    <x:tableColumn id="57" name="检索路径"/>
+    <x:tableColumn id="58" name="获取时间"/>
+    <x:tableColumn id="59" name="置信度"/>
+    <x:tableColumn id="60" name="冲突说明"/>
+    <x:tableColumn id="61" name="决策日志引用"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1280,7 +1284,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3944b479a25d4833"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R973be06183c74496"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1312,6 +1316,7 @@
     <x:col min="21" max="21" width="16" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="16" hidden="0" customWidth="1"/>
     <x:col min="23" max="23" width="16" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1340,10 +1345,11 @@
       <x:c r="U1" s="4"/>
       <x:c r="V1" s="4"/>
       <x:c r="W1" s="4"/>
+      <x:c r="X1" s="4"/>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>每个目标产品独立冻结参考图、必需视图、外观/功能门槛、目标价格与 Top-N；一行一产品。</x:v>
+        <x:v>每个目标产品独立冻结参考图、必需视图、外观/功能门槛、Amazon目标站点、目标价格与 Top-N；一行一产品。</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -1367,6 +1373,7 @@
       <x:c r="U2" s="8"/>
       <x:c r="V2" s="8"/>
       <x:c r="W2" s="8"/>
+      <x:c r="X2" s="8"/>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="14" t="str">
@@ -1421,21 +1428,24 @@
         <x:v>Amazon同类均价最低样本数</x:v>
       </x:c>
       <x:c r="R3" s="14" t="str">
+        <x:v>Amazon目标站点</x:v>
+      </x:c>
+      <x:c r="S3" s="14" t="str">
         <x:v>1688目标成本</x:v>
       </x:c>
-      <x:c r="S3" s="14" t="str">
+      <x:c r="T3" s="14" t="str">
         <x:v>1688价格允许偏差</x:v>
       </x:c>
-      <x:c r="T3" s="14" t="str">
+      <x:c r="U3" s="14" t="str">
         <x:v>采购数量档位</x:v>
       </x:c>
-      <x:c r="U3" s="14" t="str">
+      <x:c r="V3" s="14" t="str">
         <x:v>目标严格合格数量</x:v>
       </x:c>
-      <x:c r="V3" s="14" t="str">
+      <x:c r="W3" s="14" t="str">
         <x:v>Amazon目标币种</x:v>
       </x:c>
-      <x:c r="W3" s="14" t="str">
+      <x:c r="X3" s="14" t="str">
         <x:v>1688成本币种</x:v>
       </x:c>
     </x:row>
@@ -1457,1007 +1467,1008 @@
       <x:c r="O4" s="31"/>
       <x:c r="P4" s="19"/>
       <x:c r="Q4" s="19"/>
-      <x:c r="R4" s="29"/>
-      <x:c r="S4" s="31"/>
-      <x:c r="T4" s="33"/>
+      <x:c r="R4" s="19"/>
+      <x:c r="S4" s="29"/>
+      <x:c r="T4" s="31"/>
       <x:c r="U4" s="33"/>
-      <x:c r="V4" s="19"/>
-      <x:c r="W4" s="29"/>
+      <x:c r="V4" s="33"/>
+      <x:c r="W4" s="19"/>
+      <x:c r="X4" s="29"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="28"/>
       <x:c r="N5" s="30"/>
       <x:c r="O5" s="32"/>
-      <x:c r="R5" s="30"/>
-      <x:c r="S5" s="32"/>
-      <x:c r="T5" s="34"/>
+      <x:c r="S5" s="30"/>
+      <x:c r="T5" s="32"/>
       <x:c r="U5" s="34"/>
-      <x:c r="W5" s="30"/>
+      <x:c r="V5" s="34"/>
+      <x:c r="X5" s="30"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="28"/>
       <x:c r="N6" s="30"/>
       <x:c r="O6" s="32"/>
-      <x:c r="R6" s="30"/>
-      <x:c r="S6" s="32"/>
-      <x:c r="T6" s="34"/>
+      <x:c r="S6" s="30"/>
+      <x:c r="T6" s="32"/>
       <x:c r="U6" s="34"/>
-      <x:c r="W6" s="30"/>
+      <x:c r="V6" s="34"/>
+      <x:c r="X6" s="30"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="28"/>
       <x:c r="N7" s="30"/>
       <x:c r="O7" s="32"/>
-      <x:c r="R7" s="30"/>
-      <x:c r="S7" s="32"/>
-      <x:c r="T7" s="34"/>
+      <x:c r="S7" s="30"/>
+      <x:c r="T7" s="32"/>
       <x:c r="U7" s="34"/>
-      <x:c r="W7" s="30"/>
+      <x:c r="V7" s="34"/>
+      <x:c r="X7" s="30"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="28"/>
       <x:c r="N8" s="30"/>
       <x:c r="O8" s="32"/>
-      <x:c r="R8" s="30"/>
-      <x:c r="S8" s="32"/>
-      <x:c r="T8" s="34"/>
+      <x:c r="S8" s="30"/>
+      <x:c r="T8" s="32"/>
       <x:c r="U8" s="34"/>
-      <x:c r="W8" s="30"/>
+      <x:c r="V8" s="34"/>
+      <x:c r="X8" s="30"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="28"/>
       <x:c r="N9" s="30"/>
       <x:c r="O9" s="32"/>
-      <x:c r="R9" s="30"/>
-      <x:c r="S9" s="32"/>
-      <x:c r="T9" s="34"/>
+      <x:c r="S9" s="30"/>
+      <x:c r="T9" s="32"/>
       <x:c r="U9" s="34"/>
-      <x:c r="W9" s="30"/>
+      <x:c r="V9" s="34"/>
+      <x:c r="X9" s="30"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="28"/>
       <x:c r="N10" s="30"/>
       <x:c r="O10" s="32"/>
-      <x:c r="R10" s="30"/>
-      <x:c r="S10" s="32"/>
-      <x:c r="T10" s="34"/>
+      <x:c r="S10" s="30"/>
+      <x:c r="T10" s="32"/>
       <x:c r="U10" s="34"/>
-      <x:c r="W10" s="30"/>
+      <x:c r="V10" s="34"/>
+      <x:c r="X10" s="30"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="28"/>
       <x:c r="N11" s="30"/>
       <x:c r="O11" s="32"/>
-      <x:c r="R11" s="30"/>
-      <x:c r="S11" s="32"/>
-      <x:c r="T11" s="34"/>
+      <x:c r="S11" s="30"/>
+      <x:c r="T11" s="32"/>
       <x:c r="U11" s="34"/>
-      <x:c r="W11" s="30"/>
+      <x:c r="V11" s="34"/>
+      <x:c r="X11" s="30"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="28"/>
       <x:c r="N12" s="30"/>
       <x:c r="O12" s="32"/>
-      <x:c r="R12" s="30"/>
-      <x:c r="S12" s="32"/>
-      <x:c r="T12" s="34"/>
+      <x:c r="S12" s="30"/>
+      <x:c r="T12" s="32"/>
       <x:c r="U12" s="34"/>
-      <x:c r="W12" s="30"/>
+      <x:c r="V12" s="34"/>
+      <x:c r="X12" s="30"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="28"/>
       <x:c r="N13" s="30"/>
       <x:c r="O13" s="32"/>
-      <x:c r="R13" s="30"/>
-      <x:c r="S13" s="32"/>
-      <x:c r="T13" s="34"/>
+      <x:c r="S13" s="30"/>
+      <x:c r="T13" s="32"/>
       <x:c r="U13" s="34"/>
-      <x:c r="W13" s="30"/>
+      <x:c r="V13" s="34"/>
+      <x:c r="X13" s="30"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="28"/>
       <x:c r="N14" s="30"/>
       <x:c r="O14" s="32"/>
-      <x:c r="R14" s="30"/>
-      <x:c r="S14" s="32"/>
-      <x:c r="T14" s="34"/>
+      <x:c r="S14" s="30"/>
+      <x:c r="T14" s="32"/>
       <x:c r="U14" s="34"/>
-      <x:c r="W14" s="30"/>
+      <x:c r="V14" s="34"/>
+      <x:c r="X14" s="30"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="28"/>
       <x:c r="N15" s="30"/>
       <x:c r="O15" s="32"/>
-      <x:c r="R15" s="30"/>
-      <x:c r="S15" s="32"/>
-      <x:c r="T15" s="34"/>
+      <x:c r="S15" s="30"/>
+      <x:c r="T15" s="32"/>
       <x:c r="U15" s="34"/>
-      <x:c r="W15" s="30"/>
+      <x:c r="V15" s="34"/>
+      <x:c r="X15" s="30"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="28"/>
       <x:c r="N16" s="30"/>
       <x:c r="O16" s="32"/>
-      <x:c r="R16" s="30"/>
-      <x:c r="S16" s="32"/>
-      <x:c r="T16" s="34"/>
+      <x:c r="S16" s="30"/>
+      <x:c r="T16" s="32"/>
       <x:c r="U16" s="34"/>
-      <x:c r="W16" s="30"/>
+      <x:c r="V16" s="34"/>
+      <x:c r="X16" s="30"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="28"/>
       <x:c r="N17" s="30"/>
       <x:c r="O17" s="32"/>
-      <x:c r="R17" s="30"/>
-      <x:c r="S17" s="32"/>
-      <x:c r="T17" s="34"/>
+      <x:c r="S17" s="30"/>
+      <x:c r="T17" s="32"/>
       <x:c r="U17" s="34"/>
-      <x:c r="W17" s="30"/>
+      <x:c r="V17" s="34"/>
+      <x:c r="X17" s="30"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="28"/>
       <x:c r="N18" s="30"/>
       <x:c r="O18" s="32"/>
-      <x:c r="R18" s="30"/>
-      <x:c r="S18" s="32"/>
-      <x:c r="T18" s="34"/>
+      <x:c r="S18" s="30"/>
+      <x:c r="T18" s="32"/>
       <x:c r="U18" s="34"/>
-      <x:c r="W18" s="30"/>
+      <x:c r="V18" s="34"/>
+      <x:c r="X18" s="30"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="28"/>
       <x:c r="N19" s="30"/>
       <x:c r="O19" s="32"/>
-      <x:c r="R19" s="30"/>
-      <x:c r="S19" s="32"/>
-      <x:c r="T19" s="34"/>
+      <x:c r="S19" s="30"/>
+      <x:c r="T19" s="32"/>
       <x:c r="U19" s="34"/>
-      <x:c r="W19" s="30"/>
+      <x:c r="V19" s="34"/>
+      <x:c r="X19" s="30"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="28"/>
       <x:c r="N20" s="30"/>
       <x:c r="O20" s="32"/>
-      <x:c r="R20" s="30"/>
-      <x:c r="S20" s="32"/>
-      <x:c r="T20" s="34"/>
+      <x:c r="S20" s="30"/>
+      <x:c r="T20" s="32"/>
       <x:c r="U20" s="34"/>
-      <x:c r="W20" s="30"/>
+      <x:c r="V20" s="34"/>
+      <x:c r="X20" s="30"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="28"/>
       <x:c r="N21" s="30"/>
       <x:c r="O21" s="32"/>
-      <x:c r="R21" s="30"/>
-      <x:c r="S21" s="32"/>
-      <x:c r="T21" s="34"/>
+      <x:c r="S21" s="30"/>
+      <x:c r="T21" s="32"/>
       <x:c r="U21" s="34"/>
-      <x:c r="W21" s="30"/>
+      <x:c r="V21" s="34"/>
+      <x:c r="X21" s="30"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="28"/>
       <x:c r="N22" s="30"/>
       <x:c r="O22" s="32"/>
-      <x:c r="R22" s="30"/>
-      <x:c r="S22" s="32"/>
-      <x:c r="T22" s="34"/>
+      <x:c r="S22" s="30"/>
+      <x:c r="T22" s="32"/>
       <x:c r="U22" s="34"/>
-      <x:c r="W22" s="30"/>
+      <x:c r="V22" s="34"/>
+      <x:c r="X22" s="30"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="28"/>
       <x:c r="N23" s="30"/>
       <x:c r="O23" s="32"/>
-      <x:c r="R23" s="30"/>
-      <x:c r="S23" s="32"/>
-      <x:c r="T23" s="34"/>
+      <x:c r="S23" s="30"/>
+      <x:c r="T23" s="32"/>
       <x:c r="U23" s="34"/>
-      <x:c r="W23" s="30"/>
+      <x:c r="V23" s="34"/>
+      <x:c r="X23" s="30"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="28"/>
       <x:c r="N24" s="30"/>
       <x:c r="O24" s="32"/>
-      <x:c r="R24" s="30"/>
-      <x:c r="S24" s="32"/>
-      <x:c r="T24" s="34"/>
+      <x:c r="S24" s="30"/>
+      <x:c r="T24" s="32"/>
       <x:c r="U24" s="34"/>
-      <x:c r="W24" s="30"/>
+      <x:c r="V24" s="34"/>
+      <x:c r="X24" s="30"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="28"/>
       <x:c r="N25" s="30"/>
       <x:c r="O25" s="32"/>
-      <x:c r="R25" s="30"/>
-      <x:c r="S25" s="32"/>
-      <x:c r="T25" s="34"/>
+      <x:c r="S25" s="30"/>
+      <x:c r="T25" s="32"/>
       <x:c r="U25" s="34"/>
-      <x:c r="W25" s="30"/>
+      <x:c r="V25" s="34"/>
+      <x:c r="X25" s="30"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="28"/>
       <x:c r="N26" s="30"/>
       <x:c r="O26" s="32"/>
-      <x:c r="R26" s="30"/>
-      <x:c r="S26" s="32"/>
-      <x:c r="T26" s="34"/>
+      <x:c r="S26" s="30"/>
+      <x:c r="T26" s="32"/>
       <x:c r="U26" s="34"/>
-      <x:c r="W26" s="30"/>
+      <x:c r="V26" s="34"/>
+      <x:c r="X26" s="30"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="28"/>
       <x:c r="N27" s="30"/>
       <x:c r="O27" s="32"/>
-      <x:c r="R27" s="30"/>
-      <x:c r="S27" s="32"/>
-      <x:c r="T27" s="34"/>
+      <x:c r="S27" s="30"/>
+      <x:c r="T27" s="32"/>
       <x:c r="U27" s="34"/>
-      <x:c r="W27" s="30"/>
+      <x:c r="V27" s="34"/>
+      <x:c r="X27" s="30"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="28"/>
       <x:c r="N28" s="30"/>
       <x:c r="O28" s="32"/>
-      <x:c r="R28" s="30"/>
-      <x:c r="S28" s="32"/>
-      <x:c r="T28" s="34"/>
+      <x:c r="S28" s="30"/>
+      <x:c r="T28" s="32"/>
       <x:c r="U28" s="34"/>
-      <x:c r="W28" s="30"/>
+      <x:c r="V28" s="34"/>
+      <x:c r="X28" s="30"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="28"/>
       <x:c r="N29" s="30"/>
       <x:c r="O29" s="32"/>
-      <x:c r="R29" s="30"/>
-      <x:c r="S29" s="32"/>
-      <x:c r="T29" s="34"/>
+      <x:c r="S29" s="30"/>
+      <x:c r="T29" s="32"/>
       <x:c r="U29" s="34"/>
-      <x:c r="W29" s="30"/>
+      <x:c r="V29" s="34"/>
+      <x:c r="X29" s="30"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="28"/>
       <x:c r="N30" s="30"/>
       <x:c r="O30" s="32"/>
-      <x:c r="R30" s="30"/>
-      <x:c r="S30" s="32"/>
-      <x:c r="T30" s="34"/>
+      <x:c r="S30" s="30"/>
+      <x:c r="T30" s="32"/>
       <x:c r="U30" s="34"/>
-      <x:c r="W30" s="30"/>
+      <x:c r="V30" s="34"/>
+      <x:c r="X30" s="30"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="28"/>
       <x:c r="N31" s="30"/>
       <x:c r="O31" s="32"/>
-      <x:c r="R31" s="30"/>
-      <x:c r="S31" s="32"/>
-      <x:c r="T31" s="34"/>
+      <x:c r="S31" s="30"/>
+      <x:c r="T31" s="32"/>
       <x:c r="U31" s="34"/>
-      <x:c r="W31" s="30"/>
+      <x:c r="V31" s="34"/>
+      <x:c r="X31" s="30"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="28"/>
       <x:c r="N32" s="30"/>
       <x:c r="O32" s="32"/>
-      <x:c r="R32" s="30"/>
-      <x:c r="S32" s="32"/>
-      <x:c r="T32" s="34"/>
+      <x:c r="S32" s="30"/>
+      <x:c r="T32" s="32"/>
       <x:c r="U32" s="34"/>
-      <x:c r="W32" s="30"/>
+      <x:c r="V32" s="34"/>
+      <x:c r="X32" s="30"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="28"/>
       <x:c r="N33" s="30"/>
       <x:c r="O33" s="32"/>
-      <x:c r="R33" s="30"/>
-      <x:c r="S33" s="32"/>
-      <x:c r="T33" s="34"/>
+      <x:c r="S33" s="30"/>
+      <x:c r="T33" s="32"/>
       <x:c r="U33" s="34"/>
-      <x:c r="W33" s="30"/>
+      <x:c r="V33" s="34"/>
+      <x:c r="X33" s="30"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="28"/>
       <x:c r="N34" s="30"/>
       <x:c r="O34" s="32"/>
-      <x:c r="R34" s="30"/>
-      <x:c r="S34" s="32"/>
-      <x:c r="T34" s="34"/>
+      <x:c r="S34" s="30"/>
+      <x:c r="T34" s="32"/>
       <x:c r="U34" s="34"/>
-      <x:c r="W34" s="30"/>
+      <x:c r="V34" s="34"/>
+      <x:c r="X34" s="30"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="28"/>
       <x:c r="N35" s="30"/>
       <x:c r="O35" s="32"/>
-      <x:c r="R35" s="30"/>
-      <x:c r="S35" s="32"/>
-      <x:c r="T35" s="34"/>
+      <x:c r="S35" s="30"/>
+      <x:c r="T35" s="32"/>
       <x:c r="U35" s="34"/>
-      <x:c r="W35" s="30"/>
+      <x:c r="V35" s="34"/>
+      <x:c r="X35" s="30"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="28"/>
       <x:c r="N36" s="30"/>
       <x:c r="O36" s="32"/>
-      <x:c r="R36" s="30"/>
-      <x:c r="S36" s="32"/>
-      <x:c r="T36" s="34"/>
+      <x:c r="S36" s="30"/>
+      <x:c r="T36" s="32"/>
       <x:c r="U36" s="34"/>
-      <x:c r="W36" s="30"/>
+      <x:c r="V36" s="34"/>
+      <x:c r="X36" s="30"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="28"/>
       <x:c r="N37" s="30"/>
       <x:c r="O37" s="32"/>
-      <x:c r="R37" s="30"/>
-      <x:c r="S37" s="32"/>
-      <x:c r="T37" s="34"/>
+      <x:c r="S37" s="30"/>
+      <x:c r="T37" s="32"/>
       <x:c r="U37" s="34"/>
-      <x:c r="W37" s="30"/>
+      <x:c r="V37" s="34"/>
+      <x:c r="X37" s="30"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="28"/>
       <x:c r="N38" s="30"/>
       <x:c r="O38" s="32"/>
-      <x:c r="R38" s="30"/>
-      <x:c r="S38" s="32"/>
-      <x:c r="T38" s="34"/>
+      <x:c r="S38" s="30"/>
+      <x:c r="T38" s="32"/>
       <x:c r="U38" s="34"/>
-      <x:c r="W38" s="30"/>
+      <x:c r="V38" s="34"/>
+      <x:c r="X38" s="30"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="28"/>
       <x:c r="N39" s="30"/>
       <x:c r="O39" s="32"/>
-      <x:c r="R39" s="30"/>
-      <x:c r="S39" s="32"/>
-      <x:c r="T39" s="34"/>
+      <x:c r="S39" s="30"/>
+      <x:c r="T39" s="32"/>
       <x:c r="U39" s="34"/>
-      <x:c r="W39" s="30"/>
+      <x:c r="V39" s="34"/>
+      <x:c r="X39" s="30"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="28"/>
       <x:c r="N40" s="30"/>
       <x:c r="O40" s="32"/>
-      <x:c r="R40" s="30"/>
-      <x:c r="S40" s="32"/>
-      <x:c r="T40" s="34"/>
+      <x:c r="S40" s="30"/>
+      <x:c r="T40" s="32"/>
       <x:c r="U40" s="34"/>
-      <x:c r="W40" s="30"/>
+      <x:c r="V40" s="34"/>
+      <x:c r="X40" s="30"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="28"/>
       <x:c r="N41" s="30"/>
       <x:c r="O41" s="32"/>
-      <x:c r="R41" s="30"/>
-      <x:c r="S41" s="32"/>
-      <x:c r="T41" s="34"/>
+      <x:c r="S41" s="30"/>
+      <x:c r="T41" s="32"/>
       <x:c r="U41" s="34"/>
-      <x:c r="W41" s="30"/>
+      <x:c r="V41" s="34"/>
+      <x:c r="X41" s="30"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="28"/>
       <x:c r="N42" s="30"/>
       <x:c r="O42" s="32"/>
-      <x:c r="R42" s="30"/>
-      <x:c r="S42" s="32"/>
-      <x:c r="T42" s="34"/>
+      <x:c r="S42" s="30"/>
+      <x:c r="T42" s="32"/>
       <x:c r="U42" s="34"/>
-      <x:c r="W42" s="30"/>
+      <x:c r="V42" s="34"/>
+      <x:c r="X42" s="30"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="28"/>
       <x:c r="N43" s="30"/>
       <x:c r="O43" s="32"/>
-      <x:c r="R43" s="30"/>
-      <x:c r="S43" s="32"/>
-      <x:c r="T43" s="34"/>
+      <x:c r="S43" s="30"/>
+      <x:c r="T43" s="32"/>
       <x:c r="U43" s="34"/>
-      <x:c r="W43" s="30"/>
+      <x:c r="V43" s="34"/>
+      <x:c r="X43" s="30"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="28"/>
       <x:c r="N44" s="30"/>
       <x:c r="O44" s="32"/>
-      <x:c r="R44" s="30"/>
-      <x:c r="S44" s="32"/>
-      <x:c r="T44" s="34"/>
+      <x:c r="S44" s="30"/>
+      <x:c r="T44" s="32"/>
       <x:c r="U44" s="34"/>
-      <x:c r="W44" s="30"/>
+      <x:c r="V44" s="34"/>
+      <x:c r="X44" s="30"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="28"/>
       <x:c r="N45" s="30"/>
       <x:c r="O45" s="32"/>
-      <x:c r="R45" s="30"/>
-      <x:c r="S45" s="32"/>
-      <x:c r="T45" s="34"/>
+      <x:c r="S45" s="30"/>
+      <x:c r="T45" s="32"/>
       <x:c r="U45" s="34"/>
-      <x:c r="W45" s="30"/>
+      <x:c r="V45" s="34"/>
+      <x:c r="X45" s="30"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="28"/>
       <x:c r="N46" s="30"/>
       <x:c r="O46" s="32"/>
-      <x:c r="R46" s="30"/>
-      <x:c r="S46" s="32"/>
-      <x:c r="T46" s="34"/>
+      <x:c r="S46" s="30"/>
+      <x:c r="T46" s="32"/>
       <x:c r="U46" s="34"/>
-      <x:c r="W46" s="30"/>
+      <x:c r="V46" s="34"/>
+      <x:c r="X46" s="30"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="28"/>
       <x:c r="N47" s="30"/>
       <x:c r="O47" s="32"/>
-      <x:c r="R47" s="30"/>
-      <x:c r="S47" s="32"/>
-      <x:c r="T47" s="34"/>
+      <x:c r="S47" s="30"/>
+      <x:c r="T47" s="32"/>
       <x:c r="U47" s="34"/>
-      <x:c r="W47" s="30"/>
+      <x:c r="V47" s="34"/>
+      <x:c r="X47" s="30"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="28"/>
       <x:c r="N48" s="30"/>
       <x:c r="O48" s="32"/>
-      <x:c r="R48" s="30"/>
-      <x:c r="S48" s="32"/>
-      <x:c r="T48" s="34"/>
+      <x:c r="S48" s="30"/>
+      <x:c r="T48" s="32"/>
       <x:c r="U48" s="34"/>
-      <x:c r="W48" s="30"/>
+      <x:c r="V48" s="34"/>
+      <x:c r="X48" s="30"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="28"/>
       <x:c r="N49" s="30"/>
       <x:c r="O49" s="32"/>
-      <x:c r="R49" s="30"/>
-      <x:c r="S49" s="32"/>
-      <x:c r="T49" s="34"/>
+      <x:c r="S49" s="30"/>
+      <x:c r="T49" s="32"/>
       <x:c r="U49" s="34"/>
-      <x:c r="W49" s="30"/>
+      <x:c r="V49" s="34"/>
+      <x:c r="X49" s="30"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="28"/>
       <x:c r="N50" s="30"/>
       <x:c r="O50" s="32"/>
-      <x:c r="R50" s="30"/>
-      <x:c r="S50" s="32"/>
-      <x:c r="T50" s="34"/>
+      <x:c r="S50" s="30"/>
+      <x:c r="T50" s="32"/>
       <x:c r="U50" s="34"/>
-      <x:c r="W50" s="30"/>
+      <x:c r="V50" s="34"/>
+      <x:c r="X50" s="30"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="28"/>
       <x:c r="N51" s="30"/>
       <x:c r="O51" s="32"/>
-      <x:c r="R51" s="30"/>
-      <x:c r="S51" s="32"/>
-      <x:c r="T51" s="34"/>
+      <x:c r="S51" s="30"/>
+      <x:c r="T51" s="32"/>
       <x:c r="U51" s="34"/>
-      <x:c r="W51" s="30"/>
+      <x:c r="V51" s="34"/>
+      <x:c r="X51" s="30"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="28"/>
       <x:c r="N52" s="30"/>
       <x:c r="O52" s="32"/>
-      <x:c r="R52" s="30"/>
-      <x:c r="S52" s="32"/>
-      <x:c r="T52" s="34"/>
+      <x:c r="S52" s="30"/>
+      <x:c r="T52" s="32"/>
       <x:c r="U52" s="34"/>
-      <x:c r="W52" s="30"/>
+      <x:c r="V52" s="34"/>
+      <x:c r="X52" s="30"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="28"/>
       <x:c r="N53" s="30"/>
       <x:c r="O53" s="32"/>
-      <x:c r="R53" s="30"/>
-      <x:c r="S53" s="32"/>
-      <x:c r="T53" s="34"/>
+      <x:c r="S53" s="30"/>
+      <x:c r="T53" s="32"/>
       <x:c r="U53" s="34"/>
-      <x:c r="W53" s="30"/>
+      <x:c r="V53" s="34"/>
+      <x:c r="X53" s="30"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="28"/>
       <x:c r="N54" s="30"/>
       <x:c r="O54" s="32"/>
-      <x:c r="R54" s="30"/>
-      <x:c r="S54" s="32"/>
-      <x:c r="T54" s="34"/>
+      <x:c r="S54" s="30"/>
+      <x:c r="T54" s="32"/>
       <x:c r="U54" s="34"/>
-      <x:c r="W54" s="30"/>
+      <x:c r="V54" s="34"/>
+      <x:c r="X54" s="30"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="28"/>
       <x:c r="N55" s="30"/>
       <x:c r="O55" s="32"/>
-      <x:c r="R55" s="30"/>
-      <x:c r="S55" s="32"/>
-      <x:c r="T55" s="34"/>
+      <x:c r="S55" s="30"/>
+      <x:c r="T55" s="32"/>
       <x:c r="U55" s="34"/>
-      <x:c r="W55" s="30"/>
+      <x:c r="V55" s="34"/>
+      <x:c r="X55" s="30"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="28"/>
       <x:c r="N56" s="30"/>
       <x:c r="O56" s="32"/>
-      <x:c r="R56" s="30"/>
-      <x:c r="S56" s="32"/>
-      <x:c r="T56" s="34"/>
+      <x:c r="S56" s="30"/>
+      <x:c r="T56" s="32"/>
       <x:c r="U56" s="34"/>
-      <x:c r="W56" s="30"/>
+      <x:c r="V56" s="34"/>
+      <x:c r="X56" s="30"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="28"/>
       <x:c r="N57" s="30"/>
       <x:c r="O57" s="32"/>
-      <x:c r="R57" s="30"/>
-      <x:c r="S57" s="32"/>
-      <x:c r="T57" s="34"/>
+      <x:c r="S57" s="30"/>
+      <x:c r="T57" s="32"/>
       <x:c r="U57" s="34"/>
-      <x:c r="W57" s="30"/>
+      <x:c r="V57" s="34"/>
+      <x:c r="X57" s="30"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="28"/>
       <x:c r="N58" s="30"/>
       <x:c r="O58" s="32"/>
-      <x:c r="R58" s="30"/>
-      <x:c r="S58" s="32"/>
-      <x:c r="T58" s="34"/>
+      <x:c r="S58" s="30"/>
+      <x:c r="T58" s="32"/>
       <x:c r="U58" s="34"/>
-      <x:c r="W58" s="30"/>
+      <x:c r="V58" s="34"/>
+      <x:c r="X58" s="30"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="28"/>
       <x:c r="N59" s="30"/>
       <x:c r="O59" s="32"/>
-      <x:c r="R59" s="30"/>
-      <x:c r="S59" s="32"/>
-      <x:c r="T59" s="34"/>
+      <x:c r="S59" s="30"/>
+      <x:c r="T59" s="32"/>
       <x:c r="U59" s="34"/>
-      <x:c r="W59" s="30"/>
+      <x:c r="V59" s="34"/>
+      <x:c r="X59" s="30"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="28"/>
       <x:c r="N60" s="30"/>
       <x:c r="O60" s="32"/>
-      <x:c r="R60" s="30"/>
-      <x:c r="S60" s="32"/>
-      <x:c r="T60" s="34"/>
+      <x:c r="S60" s="30"/>
+      <x:c r="T60" s="32"/>
       <x:c r="U60" s="34"/>
-      <x:c r="W60" s="30"/>
+      <x:c r="V60" s="34"/>
+      <x:c r="X60" s="30"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="28"/>
       <x:c r="N61" s="30"/>
       <x:c r="O61" s="32"/>
-      <x:c r="R61" s="30"/>
-      <x:c r="S61" s="32"/>
-      <x:c r="T61" s="34"/>
+      <x:c r="S61" s="30"/>
+      <x:c r="T61" s="32"/>
       <x:c r="U61" s="34"/>
-      <x:c r="W61" s="30"/>
+      <x:c r="V61" s="34"/>
+      <x:c r="X61" s="30"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="28"/>
       <x:c r="N62" s="30"/>
       <x:c r="O62" s="32"/>
-      <x:c r="R62" s="30"/>
-      <x:c r="S62" s="32"/>
-      <x:c r="T62" s="34"/>
+      <x:c r="S62" s="30"/>
+      <x:c r="T62" s="32"/>
       <x:c r="U62" s="34"/>
-      <x:c r="W62" s="30"/>
+      <x:c r="V62" s="34"/>
+      <x:c r="X62" s="30"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="28"/>
       <x:c r="N63" s="30"/>
       <x:c r="O63" s="32"/>
-      <x:c r="R63" s="30"/>
-      <x:c r="S63" s="32"/>
-      <x:c r="T63" s="34"/>
+      <x:c r="S63" s="30"/>
+      <x:c r="T63" s="32"/>
       <x:c r="U63" s="34"/>
-      <x:c r="W63" s="30"/>
+      <x:c r="V63" s="34"/>
+      <x:c r="X63" s="30"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="28"/>
       <x:c r="N64" s="30"/>
       <x:c r="O64" s="32"/>
-      <x:c r="R64" s="30"/>
-      <x:c r="S64" s="32"/>
-      <x:c r="T64" s="34"/>
+      <x:c r="S64" s="30"/>
+      <x:c r="T64" s="32"/>
       <x:c r="U64" s="34"/>
-      <x:c r="W64" s="30"/>
+      <x:c r="V64" s="34"/>
+      <x:c r="X64" s="30"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="28"/>
       <x:c r="N65" s="30"/>
       <x:c r="O65" s="32"/>
-      <x:c r="R65" s="30"/>
-      <x:c r="S65" s="32"/>
-      <x:c r="T65" s="34"/>
+      <x:c r="S65" s="30"/>
+      <x:c r="T65" s="32"/>
       <x:c r="U65" s="34"/>
-      <x:c r="W65" s="30"/>
+      <x:c r="V65" s="34"/>
+      <x:c r="X65" s="30"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="28"/>
       <x:c r="N66" s="30"/>
       <x:c r="O66" s="32"/>
-      <x:c r="R66" s="30"/>
-      <x:c r="S66" s="32"/>
-      <x:c r="T66" s="34"/>
+      <x:c r="S66" s="30"/>
+      <x:c r="T66" s="32"/>
       <x:c r="U66" s="34"/>
-      <x:c r="W66" s="30"/>
+      <x:c r="V66" s="34"/>
+      <x:c r="X66" s="30"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="28"/>
       <x:c r="N67" s="30"/>
       <x:c r="O67" s="32"/>
-      <x:c r="R67" s="30"/>
-      <x:c r="S67" s="32"/>
-      <x:c r="T67" s="34"/>
+      <x:c r="S67" s="30"/>
+      <x:c r="T67" s="32"/>
       <x:c r="U67" s="34"/>
-      <x:c r="W67" s="30"/>
+      <x:c r="V67" s="34"/>
+      <x:c r="X67" s="30"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="28"/>
       <x:c r="N68" s="30"/>
       <x:c r="O68" s="32"/>
-      <x:c r="R68" s="30"/>
-      <x:c r="S68" s="32"/>
-      <x:c r="T68" s="34"/>
+      <x:c r="S68" s="30"/>
+      <x:c r="T68" s="32"/>
       <x:c r="U68" s="34"/>
-      <x:c r="W68" s="30"/>
+      <x:c r="V68" s="34"/>
+      <x:c r="X68" s="30"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="28"/>
       <x:c r="N69" s="30"/>
       <x:c r="O69" s="32"/>
-      <x:c r="R69" s="30"/>
-      <x:c r="S69" s="32"/>
-      <x:c r="T69" s="34"/>
+      <x:c r="S69" s="30"/>
+      <x:c r="T69" s="32"/>
       <x:c r="U69" s="34"/>
-      <x:c r="W69" s="30"/>
+      <x:c r="V69" s="34"/>
+      <x:c r="X69" s="30"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="28"/>
       <x:c r="N70" s="30"/>
       <x:c r="O70" s="32"/>
-      <x:c r="R70" s="30"/>
-      <x:c r="S70" s="32"/>
-      <x:c r="T70" s="34"/>
+      <x:c r="S70" s="30"/>
+      <x:c r="T70" s="32"/>
       <x:c r="U70" s="34"/>
-      <x:c r="W70" s="30"/>
+      <x:c r="V70" s="34"/>
+      <x:c r="X70" s="30"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="28"/>
       <x:c r="N71" s="30"/>
       <x:c r="O71" s="32"/>
-      <x:c r="R71" s="30"/>
-      <x:c r="S71" s="32"/>
-      <x:c r="T71" s="34"/>
+      <x:c r="S71" s="30"/>
+      <x:c r="T71" s="32"/>
       <x:c r="U71" s="34"/>
-      <x:c r="W71" s="30"/>
+      <x:c r="V71" s="34"/>
+      <x:c r="X71" s="30"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="28"/>
       <x:c r="N72" s="30"/>
       <x:c r="O72" s="32"/>
-      <x:c r="R72" s="30"/>
-      <x:c r="S72" s="32"/>
-      <x:c r="T72" s="34"/>
+      <x:c r="S72" s="30"/>
+      <x:c r="T72" s="32"/>
       <x:c r="U72" s="34"/>
-      <x:c r="W72" s="30"/>
+      <x:c r="V72" s="34"/>
+      <x:c r="X72" s="30"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="28"/>
       <x:c r="N73" s="30"/>
       <x:c r="O73" s="32"/>
-      <x:c r="R73" s="30"/>
-      <x:c r="S73" s="32"/>
-      <x:c r="T73" s="34"/>
+      <x:c r="S73" s="30"/>
+      <x:c r="T73" s="32"/>
       <x:c r="U73" s="34"/>
-      <x:c r="W73" s="30"/>
+      <x:c r="V73" s="34"/>
+      <x:c r="X73" s="30"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="28"/>
       <x:c r="N74" s="30"/>
       <x:c r="O74" s="32"/>
-      <x:c r="R74" s="30"/>
-      <x:c r="S74" s="32"/>
-      <x:c r="T74" s="34"/>
+      <x:c r="S74" s="30"/>
+      <x:c r="T74" s="32"/>
       <x:c r="U74" s="34"/>
-      <x:c r="W74" s="30"/>
+      <x:c r="V74" s="34"/>
+      <x:c r="X74" s="30"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="28"/>
       <x:c r="N75" s="30"/>
       <x:c r="O75" s="32"/>
-      <x:c r="R75" s="30"/>
-      <x:c r="S75" s="32"/>
-      <x:c r="T75" s="34"/>
+      <x:c r="S75" s="30"/>
+      <x:c r="T75" s="32"/>
       <x:c r="U75" s="34"/>
-      <x:c r="W75" s="30"/>
+      <x:c r="V75" s="34"/>
+      <x:c r="X75" s="30"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="28"/>
       <x:c r="N76" s="30"/>
       <x:c r="O76" s="32"/>
-      <x:c r="R76" s="30"/>
-      <x:c r="S76" s="32"/>
-      <x:c r="T76" s="34"/>
+      <x:c r="S76" s="30"/>
+      <x:c r="T76" s="32"/>
       <x:c r="U76" s="34"/>
-      <x:c r="W76" s="30"/>
+      <x:c r="V76" s="34"/>
+      <x:c r="X76" s="30"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="28"/>
       <x:c r="N77" s="30"/>
       <x:c r="O77" s="32"/>
-      <x:c r="R77" s="30"/>
-      <x:c r="S77" s="32"/>
-      <x:c r="T77" s="34"/>
+      <x:c r="S77" s="30"/>
+      <x:c r="T77" s="32"/>
       <x:c r="U77" s="34"/>
-      <x:c r="W77" s="30"/>
+      <x:c r="V77" s="34"/>
+      <x:c r="X77" s="30"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="28"/>
       <x:c r="N78" s="30"/>
       <x:c r="O78" s="32"/>
-      <x:c r="R78" s="30"/>
-      <x:c r="S78" s="32"/>
-      <x:c r="T78" s="34"/>
+      <x:c r="S78" s="30"/>
+      <x:c r="T78" s="32"/>
       <x:c r="U78" s="34"/>
-      <x:c r="W78" s="30"/>
+      <x:c r="V78" s="34"/>
+      <x:c r="X78" s="30"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="28"/>
       <x:c r="N79" s="30"/>
       <x:c r="O79" s="32"/>
-      <x:c r="R79" s="30"/>
-      <x:c r="S79" s="32"/>
-      <x:c r="T79" s="34"/>
+      <x:c r="S79" s="30"/>
+      <x:c r="T79" s="32"/>
       <x:c r="U79" s="34"/>
-      <x:c r="W79" s="30"/>
+      <x:c r="V79" s="34"/>
+      <x:c r="X79" s="30"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="28"/>
       <x:c r="N80" s="30"/>
       <x:c r="O80" s="32"/>
-      <x:c r="R80" s="30"/>
-      <x:c r="S80" s="32"/>
-      <x:c r="T80" s="34"/>
+      <x:c r="S80" s="30"/>
+      <x:c r="T80" s="32"/>
       <x:c r="U80" s="34"/>
-      <x:c r="W80" s="30"/>
+      <x:c r="V80" s="34"/>
+      <x:c r="X80" s="30"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="28"/>
       <x:c r="N81" s="30"/>
       <x:c r="O81" s="32"/>
-      <x:c r="R81" s="30"/>
-      <x:c r="S81" s="32"/>
-      <x:c r="T81" s="34"/>
+      <x:c r="S81" s="30"/>
+      <x:c r="T81" s="32"/>
       <x:c r="U81" s="34"/>
-      <x:c r="W81" s="30"/>
+      <x:c r="V81" s="34"/>
+      <x:c r="X81" s="30"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="28"/>
       <x:c r="N82" s="30"/>
       <x:c r="O82" s="32"/>
-      <x:c r="R82" s="30"/>
-      <x:c r="S82" s="32"/>
-      <x:c r="T82" s="34"/>
+      <x:c r="S82" s="30"/>
+      <x:c r="T82" s="32"/>
       <x:c r="U82" s="34"/>
-      <x:c r="W82" s="30"/>
+      <x:c r="V82" s="34"/>
+      <x:c r="X82" s="30"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="28"/>
       <x:c r="N83" s="30"/>
       <x:c r="O83" s="32"/>
-      <x:c r="R83" s="30"/>
-      <x:c r="S83" s="32"/>
-      <x:c r="T83" s="34"/>
+      <x:c r="S83" s="30"/>
+      <x:c r="T83" s="32"/>
       <x:c r="U83" s="34"/>
-      <x:c r="W83" s="30"/>
+      <x:c r="V83" s="34"/>
+      <x:c r="X83" s="30"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="28"/>
       <x:c r="N84" s="30"/>
       <x:c r="O84" s="32"/>
-      <x:c r="R84" s="30"/>
-      <x:c r="S84" s="32"/>
-      <x:c r="T84" s="34"/>
+      <x:c r="S84" s="30"/>
+      <x:c r="T84" s="32"/>
       <x:c r="U84" s="34"/>
-      <x:c r="W84" s="30"/>
+      <x:c r="V84" s="34"/>
+      <x:c r="X84" s="30"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="28"/>
       <x:c r="N85" s="30"/>
       <x:c r="O85" s="32"/>
-      <x:c r="R85" s="30"/>
-      <x:c r="S85" s="32"/>
-      <x:c r="T85" s="34"/>
+      <x:c r="S85" s="30"/>
+      <x:c r="T85" s="32"/>
       <x:c r="U85" s="34"/>
-      <x:c r="W85" s="30"/>
+      <x:c r="V85" s="34"/>
+      <x:c r="X85" s="30"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="28"/>
       <x:c r="N86" s="30"/>
       <x:c r="O86" s="32"/>
-      <x:c r="R86" s="30"/>
-      <x:c r="S86" s="32"/>
-      <x:c r="T86" s="34"/>
+      <x:c r="S86" s="30"/>
+      <x:c r="T86" s="32"/>
       <x:c r="U86" s="34"/>
-      <x:c r="W86" s="30"/>
+      <x:c r="V86" s="34"/>
+      <x:c r="X86" s="30"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="28"/>
       <x:c r="N87" s="30"/>
       <x:c r="O87" s="32"/>
-      <x:c r="R87" s="30"/>
-      <x:c r="S87" s="32"/>
-      <x:c r="T87" s="34"/>
+      <x:c r="S87" s="30"/>
+      <x:c r="T87" s="32"/>
       <x:c r="U87" s="34"/>
-      <x:c r="W87" s="30"/>
+      <x:c r="V87" s="34"/>
+      <x:c r="X87" s="30"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="28"/>
       <x:c r="N88" s="30"/>
       <x:c r="O88" s="32"/>
-      <x:c r="R88" s="30"/>
-      <x:c r="S88" s="32"/>
-      <x:c r="T88" s="34"/>
+      <x:c r="S88" s="30"/>
+      <x:c r="T88" s="32"/>
       <x:c r="U88" s="34"/>
-      <x:c r="W88" s="30"/>
+      <x:c r="V88" s="34"/>
+      <x:c r="X88" s="30"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="28"/>
       <x:c r="N89" s="30"/>
       <x:c r="O89" s="32"/>
-      <x:c r="R89" s="30"/>
-      <x:c r="S89" s="32"/>
-      <x:c r="T89" s="34"/>
+      <x:c r="S89" s="30"/>
+      <x:c r="T89" s="32"/>
       <x:c r="U89" s="34"/>
-      <x:c r="W89" s="30"/>
+      <x:c r="V89" s="34"/>
+      <x:c r="X89" s="30"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="28"/>
       <x:c r="N90" s="30"/>
       <x:c r="O90" s="32"/>
-      <x:c r="R90" s="30"/>
-      <x:c r="S90" s="32"/>
-      <x:c r="T90" s="34"/>
+      <x:c r="S90" s="30"/>
+      <x:c r="T90" s="32"/>
       <x:c r="U90" s="34"/>
-      <x:c r="W90" s="30"/>
+      <x:c r="V90" s="34"/>
+      <x:c r="X90" s="30"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="28"/>
       <x:c r="N91" s="30"/>
       <x:c r="O91" s="32"/>
-      <x:c r="R91" s="30"/>
-      <x:c r="S91" s="32"/>
-      <x:c r="T91" s="34"/>
+      <x:c r="S91" s="30"/>
+      <x:c r="T91" s="32"/>
       <x:c r="U91" s="34"/>
-      <x:c r="W91" s="30"/>
+      <x:c r="V91" s="34"/>
+      <x:c r="X91" s="30"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="28"/>
       <x:c r="N92" s="30"/>
       <x:c r="O92" s="32"/>
-      <x:c r="R92" s="30"/>
-      <x:c r="S92" s="32"/>
-      <x:c r="T92" s="34"/>
+      <x:c r="S92" s="30"/>
+      <x:c r="T92" s="32"/>
       <x:c r="U92" s="34"/>
-      <x:c r="W92" s="30"/>
+      <x:c r="V92" s="34"/>
+      <x:c r="X92" s="30"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="28"/>
       <x:c r="N93" s="30"/>
       <x:c r="O93" s="32"/>
-      <x:c r="R93" s="30"/>
-      <x:c r="S93" s="32"/>
-      <x:c r="T93" s="34"/>
+      <x:c r="S93" s="30"/>
+      <x:c r="T93" s="32"/>
       <x:c r="U93" s="34"/>
-      <x:c r="W93" s="30"/>
+      <x:c r="V93" s="34"/>
+      <x:c r="X93" s="30"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="28"/>
       <x:c r="N94" s="30"/>
       <x:c r="O94" s="32"/>
-      <x:c r="R94" s="30"/>
-      <x:c r="S94" s="32"/>
-      <x:c r="T94" s="34"/>
+      <x:c r="S94" s="30"/>
+      <x:c r="T94" s="32"/>
       <x:c r="U94" s="34"/>
-      <x:c r="W94" s="30"/>
+      <x:c r="V94" s="34"/>
+      <x:c r="X94" s="30"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="28"/>
       <x:c r="N95" s="30"/>
       <x:c r="O95" s="32"/>
-      <x:c r="R95" s="30"/>
-      <x:c r="S95" s="32"/>
-      <x:c r="T95" s="34"/>
+      <x:c r="S95" s="30"/>
+      <x:c r="T95" s="32"/>
       <x:c r="U95" s="34"/>
-      <x:c r="W95" s="30"/>
+      <x:c r="V95" s="34"/>
+      <x:c r="X95" s="30"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="28"/>
       <x:c r="N96" s="30"/>
       <x:c r="O96" s="32"/>
-      <x:c r="R96" s="30"/>
-      <x:c r="S96" s="32"/>
-      <x:c r="T96" s="34"/>
+      <x:c r="S96" s="30"/>
+      <x:c r="T96" s="32"/>
       <x:c r="U96" s="34"/>
-      <x:c r="W96" s="30"/>
+      <x:c r="V96" s="34"/>
+      <x:c r="X96" s="30"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="28"/>
       <x:c r="N97" s="30"/>
       <x:c r="O97" s="32"/>
-      <x:c r="R97" s="30"/>
-      <x:c r="S97" s="32"/>
-      <x:c r="T97" s="34"/>
+      <x:c r="S97" s="30"/>
+      <x:c r="T97" s="32"/>
       <x:c r="U97" s="34"/>
-      <x:c r="W97" s="30"/>
+      <x:c r="V97" s="34"/>
+      <x:c r="X97" s="30"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="28"/>
       <x:c r="N98" s="30"/>
       <x:c r="O98" s="32"/>
-      <x:c r="R98" s="30"/>
-      <x:c r="S98" s="32"/>
-      <x:c r="T98" s="34"/>
+      <x:c r="S98" s="30"/>
+      <x:c r="T98" s="32"/>
       <x:c r="U98" s="34"/>
-      <x:c r="W98" s="30"/>
+      <x:c r="V98" s="34"/>
+      <x:c r="X98" s="30"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="28"/>
       <x:c r="N99" s="30"/>
       <x:c r="O99" s="32"/>
-      <x:c r="R99" s="30"/>
-      <x:c r="S99" s="32"/>
-      <x:c r="T99" s="34"/>
+      <x:c r="S99" s="30"/>
+      <x:c r="T99" s="32"/>
       <x:c r="U99" s="34"/>
-      <x:c r="W99" s="30"/>
+      <x:c r="V99" s="34"/>
+      <x:c r="X99" s="30"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="28"/>
       <x:c r="N100" s="30"/>
       <x:c r="O100" s="32"/>
-      <x:c r="R100" s="30"/>
-      <x:c r="S100" s="32"/>
-      <x:c r="T100" s="34"/>
+      <x:c r="S100" s="30"/>
+      <x:c r="T100" s="32"/>
       <x:c r="U100" s="34"/>
-      <x:c r="W100" s="30"/>
+      <x:c r="V100" s="34"/>
+      <x:c r="X100" s="30"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="28"/>
       <x:c r="N101" s="30"/>
       <x:c r="O101" s="32"/>
-      <x:c r="R101" s="30"/>
-      <x:c r="S101" s="32"/>
-      <x:c r="T101" s="34"/>
+      <x:c r="S101" s="30"/>
+      <x:c r="T101" s="32"/>
       <x:c r="U101" s="34"/>
-      <x:c r="W101" s="30"/>
+      <x:c r="V101" s="34"/>
+      <x:c r="X101" s="30"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="28"/>
       <x:c r="N102" s="30"/>
       <x:c r="O102" s="32"/>
-      <x:c r="R102" s="30"/>
-      <x:c r="S102" s="32"/>
-      <x:c r="T102" s="34"/>
+      <x:c r="S102" s="30"/>
+      <x:c r="T102" s="32"/>
       <x:c r="U102" s="34"/>
-      <x:c r="W102" s="30"/>
+      <x:c r="V102" s="34"/>
+      <x:c r="X102" s="30"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="28"/>
       <x:c r="N103" s="30"/>
       <x:c r="O103" s="32"/>
-      <x:c r="R103" s="30"/>
-      <x:c r="S103" s="32"/>
-      <x:c r="T103" s="34"/>
+      <x:c r="S103" s="30"/>
+      <x:c r="T103" s="32"/>
       <x:c r="U103" s="34"/>
-      <x:c r="W103" s="30"/>
+      <x:c r="V103" s="34"/>
+      <x:c r="X103" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:W1"/>
-    <x:mergeCell ref="A2:W2"/>
+    <x:mergeCell ref="A1:X1"/>
+    <x:mergeCell ref="A2:X2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="C4:C103">
@@ -2469,7 +2480,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4690efdf8cd44ef8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ad32d240e914e85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2514,7 +2525,7 @@
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>只有产品本体、外观和功能都通过的可追溯样本才能纳入；同一跨站产品组在每个目标内只计一次。</x:v>
+        <x:v>只有目标站点内且产品本体、外观和功能都通过的可追溯样本才能纳入；同一商品和跨站产品组在每个目标内各只计一次。</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -3298,7 +3309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf553b322b0974a29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b253179c58a461c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5528,7 +5539,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb644ced4316e454c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1813d6434fdc4cb8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8210,7 +8221,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30ce819891a64d53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3de49f1eeeb14ff5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8254,12 +8265,12 @@
     <x:col min="33" max="33" width="16" hidden="0" customWidth="1"/>
     <x:col min="34" max="34" width="16" hidden="0" customWidth="1"/>
     <x:col min="35" max="35" width="16" hidden="0" customWidth="1"/>
-    <x:col min="36" max="36" width="30" hidden="0" customWidth="1"/>
+    <x:col min="36" max="36" width="16" hidden="0" customWidth="1"/>
     <x:col min="37" max="37" width="16" hidden="0" customWidth="1"/>
     <x:col min="38" max="38" width="16" hidden="0" customWidth="1"/>
-    <x:col min="39" max="39" width="16" hidden="0" customWidth="1"/>
-    <x:col min="40" max="40" width="30" hidden="0" customWidth="1"/>
-    <x:col min="41" max="41" width="30" hidden="0" customWidth="1"/>
+    <x:col min="39" max="39" width="30" hidden="0" customWidth="1"/>
+    <x:col min="40" max="40" width="16" hidden="0" customWidth="1"/>
+    <x:col min="41" max="41" width="16" hidden="0" customWidth="1"/>
     <x:col min="42" max="42" width="16" hidden="0" customWidth="1"/>
     <x:col min="43" max="43" width="30" hidden="0" customWidth="1"/>
     <x:col min="44" max="44" width="30" hidden="0" customWidth="1"/>
@@ -8269,14 +8280,17 @@
     <x:col min="48" max="48" width="16" hidden="0" customWidth="1"/>
     <x:col min="49" max="49" width="30" hidden="0" customWidth="1"/>
     <x:col min="50" max="50" width="30" hidden="0" customWidth="1"/>
-    <x:col min="51" max="51" width="30" hidden="0" customWidth="1"/>
-    <x:col min="52" max="52" width="16" hidden="0" customWidth="1"/>
-    <x:col min="53" max="53" width="28" hidden="0" customWidth="1"/>
-    <x:col min="54" max="54" width="28" hidden="0" customWidth="1"/>
-    <x:col min="55" max="55" width="20" hidden="0" customWidth="1"/>
-    <x:col min="56" max="56" width="12" hidden="0" customWidth="1"/>
-    <x:col min="57" max="57" width="30" hidden="0" customWidth="1"/>
-    <x:col min="58" max="58" width="16" hidden="0" customWidth="1"/>
+    <x:col min="51" max="51" width="16" hidden="0" customWidth="1"/>
+    <x:col min="52" max="52" width="30" hidden="0" customWidth="1"/>
+    <x:col min="53" max="53" width="30" hidden="0" customWidth="1"/>
+    <x:col min="54" max="54" width="30" hidden="0" customWidth="1"/>
+    <x:col min="55" max="55" width="16" hidden="0" customWidth="1"/>
+    <x:col min="56" max="56" width="28" hidden="0" customWidth="1"/>
+    <x:col min="57" max="57" width="28" hidden="0" customWidth="1"/>
+    <x:col min="58" max="58" width="20" hidden="0" customWidth="1"/>
+    <x:col min="59" max="59" width="12" hidden="0" customWidth="1"/>
+    <x:col min="60" max="60" width="30" hidden="0" customWidth="1"/>
+    <x:col min="61" max="61" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -8340,6 +8354,9 @@
       <x:c r="BD1" s="4"/>
       <x:c r="BE1" s="4"/>
       <x:c r="BF1" s="4"/>
+      <x:c r="BG1" s="4"/>
+      <x:c r="BH1" s="4"/>
+      <x:c r="BI1" s="4"/>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="8" t="str">
@@ -8402,6 +8419,9 @@
       <x:c r="BD2" s="8"/>
       <x:c r="BE2" s="8"/>
       <x:c r="BF2" s="8"/>
+      <x:c r="BG2" s="8"/>
+      <x:c r="BH2" s="8"/>
+      <x:c r="BI2" s="8"/>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="14" t="str">
@@ -8489,93 +8509,102 @@
         <x:v>价格/MOQ门槛</x:v>
       </x:c>
       <x:c r="AC3" s="14" t="str">
+        <x:v>目标成本</x:v>
+      </x:c>
+      <x:c r="AD3" s="14" t="str">
+        <x:v>实际单价</x:v>
+      </x:c>
+      <x:c r="AE3" s="14" t="str">
+        <x:v>成本币种</x:v>
+      </x:c>
+      <x:c r="AF3" s="14" t="str">
         <x:v>采购数量档位</x:v>
       </x:c>
-      <x:c r="AD3" s="14" t="str">
+      <x:c r="AG3" s="14" t="str">
         <x:v>MOQ</x:v>
       </x:c>
-      <x:c r="AE3" s="14" t="str">
+      <x:c r="AH3" s="14" t="str">
         <x:v>阶梯价</x:v>
       </x:c>
-      <x:c r="AF3" s="14" t="str">
+      <x:c r="AI3" s="14" t="str">
         <x:v>详情身份门槛</x:v>
       </x:c>
-      <x:c r="AG3" s="14" t="str">
+      <x:c r="AJ3" s="14" t="str">
         <x:v>供应商门槛</x:v>
       </x:c>
-      <x:c r="AH3" s="14" t="str">
+      <x:c r="AK3" s="14" t="str">
         <x:v>生产能力门槛</x:v>
       </x:c>
-      <x:c r="AI3" s="14" t="str">
+      <x:c r="AL3" s="14" t="str">
         <x:v>ODM/OEM/定制门槛</x:v>
       </x:c>
-      <x:c r="AJ3" s="14" t="str">
+      <x:c r="AM3" s="14" t="str">
         <x:v>证据一致性门槛</x:v>
       </x:c>
-      <x:c r="AK3" s="14" t="str">
+      <x:c r="AN3" s="14" t="str">
         <x:v>外观逐项核验</x:v>
       </x:c>
-      <x:c r="AL3" s="14" t="str">
+      <x:c r="AO3" s="14" t="str">
         <x:v>功能逐项核验</x:v>
       </x:c>
-      <x:c r="AM3" s="14" t="str">
+      <x:c r="AP3" s="14" t="str">
         <x:v>市场机会得分</x:v>
       </x:c>
-      <x:c r="AN3" s="14" t="str">
+      <x:c r="AQ3" s="14" t="str">
         <x:v>市场机会结论</x:v>
       </x:c>
-      <x:c r="AO3" s="14" t="str">
+      <x:c r="AR3" s="14" t="str">
         <x:v>市场机会证据</x:v>
       </x:c>
-      <x:c r="AP3" s="14" t="str">
+      <x:c r="AS3" s="14" t="str">
         <x:v>供应能力得分</x:v>
       </x:c>
-      <x:c r="AQ3" s="14" t="str">
+      <x:c r="AT3" s="14" t="str">
         <x:v>供应能力结论</x:v>
       </x:c>
-      <x:c r="AR3" s="14" t="str">
+      <x:c r="AU3" s="14" t="str">
         <x:v>供应能力证据</x:v>
       </x:c>
-      <x:c r="AS3" s="14" t="str">
+      <x:c r="AV3" s="14" t="str">
         <x:v>匹配质量得分</x:v>
       </x:c>
-      <x:c r="AT3" s="14" t="str">
+      <x:c r="AW3" s="14" t="str">
         <x:v>匹配质量结论</x:v>
       </x:c>
-      <x:c r="AU3" s="14" t="str">
+      <x:c r="AX3" s="14" t="str">
         <x:v>匹配质量证据</x:v>
       </x:c>
-      <x:c r="AV3" s="14" t="str">
+      <x:c r="AY3" s="14" t="str">
         <x:v>最终配对得分</x:v>
       </x:c>
-      <x:c r="AW3" s="14" t="str">
+      <x:c r="AZ3" s="14" t="str">
         <x:v>生产能力证据</x:v>
       </x:c>
-      <x:c r="AX3" s="14" t="str">
+      <x:c r="BA3" s="14" t="str">
         <x:v>ODM/OEM/定制证据</x:v>
       </x:c>
-      <x:c r="AY3" s="14" t="str">
+      <x:c r="BB3" s="14" t="str">
         <x:v>主要限制</x:v>
       </x:c>
-      <x:c r="AZ3" s="14" t="str">
+      <x:c r="BC3" s="14" t="str">
         <x:v>来源类型</x:v>
       </x:c>
-      <x:c r="BA3" s="14" t="str">
+      <x:c r="BD3" s="14" t="str">
         <x:v>来源链接</x:v>
       </x:c>
-      <x:c r="BB3" s="14" t="str">
+      <x:c r="BE3" s="14" t="str">
         <x:v>检索路径</x:v>
       </x:c>
-      <x:c r="BC3" s="14" t="str">
+      <x:c r="BF3" s="14" t="str">
         <x:v>获取时间</x:v>
       </x:c>
-      <x:c r="BD3" s="14" t="str">
+      <x:c r="BG3" s="14" t="str">
         <x:v>置信度</x:v>
       </x:c>
-      <x:c r="BE3" s="14" t="str">
+      <x:c r="BH3" s="14" t="str">
         <x:v>冲突说明</x:v>
       </x:c>
-      <x:c r="BF3" s="14" t="str">
+      <x:c r="BI3" s="14" t="str">
         <x:v>决策日志引用</x:v>
       </x:c>
     </x:row>
@@ -8608,17 +8637,17 @@
       <x:c r="Z4" s="19"/>
       <x:c r="AA4" s="19"/>
       <x:c r="AB4" s="29"/>
-      <x:c r="AC4" s="33"/>
-      <x:c r="AD4" s="33"/>
-      <x:c r="AE4" s="19"/>
-      <x:c r="AF4" s="19"/>
-      <x:c r="AG4" s="19"/>
+      <x:c r="AC4" s="29"/>
+      <x:c r="AD4" s="29"/>
+      <x:c r="AE4" s="29"/>
+      <x:c r="AF4" s="33"/>
+      <x:c r="AG4" s="33"/>
       <x:c r="AH4" s="19"/>
       <x:c r="AI4" s="19"/>
       <x:c r="AJ4" s="19"/>
       <x:c r="AK4" s="19"/>
       <x:c r="AL4" s="19"/>
-      <x:c r="AM4" s="37"/>
+      <x:c r="AM4" s="19"/>
       <x:c r="AN4" s="19"/>
       <x:c r="AO4" s="19"/>
       <x:c r="AP4" s="37"/>
@@ -8630,14 +8659,17 @@
       <x:c r="AV4" s="37"/>
       <x:c r="AW4" s="19"/>
       <x:c r="AX4" s="19"/>
-      <x:c r="AY4" s="19"/>
+      <x:c r="AY4" s="37"/>
       <x:c r="AZ4" s="19"/>
       <x:c r="BA4" s="19"/>
       <x:c r="BB4" s="19"/>
-      <x:c r="BC4" s="35"/>
+      <x:c r="BC4" s="19"/>
       <x:c r="BD4" s="19"/>
       <x:c r="BE4" s="19"/>
-      <x:c r="BF4" s="19"/>
+      <x:c r="BF4" s="35"/>
+      <x:c r="BG4" s="19"/>
+      <x:c r="BH4" s="19"/>
+      <x:c r="BI4" s="19"/>
     </x:row>
     <x:row r="5">
       <x:c r="C5" s="28"/>
@@ -8649,13 +8681,16 @@
       <x:c r="N5" s="28"/>
       <x:c r="O5" s="28"/>
       <x:c r="AB5" s="30"/>
-      <x:c r="AC5" s="34"/>
-      <x:c r="AD5" s="34"/>
-      <x:c r="AM5" s="38"/>
+      <x:c r="AC5" s="30"/>
+      <x:c r="AD5" s="30"/>
+      <x:c r="AE5" s="30"/>
+      <x:c r="AF5" s="34"/>
+      <x:c r="AG5" s="34"/>
       <x:c r="AP5" s="38"/>
       <x:c r="AS5" s="38"/>
       <x:c r="AV5" s="38"/>
-      <x:c r="BC5" s="36"/>
+      <x:c r="AY5" s="38"/>
+      <x:c r="BF5" s="36"/>
     </x:row>
     <x:row r="6">
       <x:c r="C6" s="28"/>
@@ -8667,13 +8702,16 @@
       <x:c r="N6" s="28"/>
       <x:c r="O6" s="28"/>
       <x:c r="AB6" s="30"/>
-      <x:c r="AC6" s="34"/>
-      <x:c r="AD6" s="34"/>
-      <x:c r="AM6" s="38"/>
+      <x:c r="AC6" s="30"/>
+      <x:c r="AD6" s="30"/>
+      <x:c r="AE6" s="30"/>
+      <x:c r="AF6" s="34"/>
+      <x:c r="AG6" s="34"/>
       <x:c r="AP6" s="38"/>
       <x:c r="AS6" s="38"/>
       <x:c r="AV6" s="38"/>
-      <x:c r="BC6" s="36"/>
+      <x:c r="AY6" s="38"/>
+      <x:c r="BF6" s="36"/>
     </x:row>
     <x:row r="7">
       <x:c r="C7" s="28"/>
@@ -8685,13 +8723,16 @@
       <x:c r="N7" s="28"/>
       <x:c r="O7" s="28"/>
       <x:c r="AB7" s="30"/>
-      <x:c r="AC7" s="34"/>
-      <x:c r="AD7" s="34"/>
-      <x:c r="AM7" s="38"/>
+      <x:c r="AC7" s="30"/>
+      <x:c r="AD7" s="30"/>
+      <x:c r="AE7" s="30"/>
+      <x:c r="AF7" s="34"/>
+      <x:c r="AG7" s="34"/>
       <x:c r="AP7" s="38"/>
       <x:c r="AS7" s="38"/>
       <x:c r="AV7" s="38"/>
-      <x:c r="BC7" s="36"/>
+      <x:c r="AY7" s="38"/>
+      <x:c r="BF7" s="36"/>
     </x:row>
     <x:row r="8">
       <x:c r="C8" s="28"/>
@@ -8703,13 +8744,16 @@
       <x:c r="N8" s="28"/>
       <x:c r="O8" s="28"/>
       <x:c r="AB8" s="30"/>
-      <x:c r="AC8" s="34"/>
-      <x:c r="AD8" s="34"/>
-      <x:c r="AM8" s="38"/>
+      <x:c r="AC8" s="30"/>
+      <x:c r="AD8" s="30"/>
+      <x:c r="AE8" s="30"/>
+      <x:c r="AF8" s="34"/>
+      <x:c r="AG8" s="34"/>
       <x:c r="AP8" s="38"/>
       <x:c r="AS8" s="38"/>
       <x:c r="AV8" s="38"/>
-      <x:c r="BC8" s="36"/>
+      <x:c r="AY8" s="38"/>
+      <x:c r="BF8" s="36"/>
     </x:row>
     <x:row r="9">
       <x:c r="C9" s="28"/>
@@ -8721,13 +8765,16 @@
       <x:c r="N9" s="28"/>
       <x:c r="O9" s="28"/>
       <x:c r="AB9" s="30"/>
-      <x:c r="AC9" s="34"/>
-      <x:c r="AD9" s="34"/>
-      <x:c r="AM9" s="38"/>
+      <x:c r="AC9" s="30"/>
+      <x:c r="AD9" s="30"/>
+      <x:c r="AE9" s="30"/>
+      <x:c r="AF9" s="34"/>
+      <x:c r="AG9" s="34"/>
       <x:c r="AP9" s="38"/>
       <x:c r="AS9" s="38"/>
       <x:c r="AV9" s="38"/>
-      <x:c r="BC9" s="36"/>
+      <x:c r="AY9" s="38"/>
+      <x:c r="BF9" s="36"/>
     </x:row>
     <x:row r="10">
       <x:c r="C10" s="28"/>
@@ -8739,13 +8786,16 @@
       <x:c r="N10" s="28"/>
       <x:c r="O10" s="28"/>
       <x:c r="AB10" s="30"/>
-      <x:c r="AC10" s="34"/>
-      <x:c r="AD10" s="34"/>
-      <x:c r="AM10" s="38"/>
+      <x:c r="AC10" s="30"/>
+      <x:c r="AD10" s="30"/>
+      <x:c r="AE10" s="30"/>
+      <x:c r="AF10" s="34"/>
+      <x:c r="AG10" s="34"/>
       <x:c r="AP10" s="38"/>
       <x:c r="AS10" s="38"/>
       <x:c r="AV10" s="38"/>
-      <x:c r="BC10" s="36"/>
+      <x:c r="AY10" s="38"/>
+      <x:c r="BF10" s="36"/>
     </x:row>
     <x:row r="11">
       <x:c r="C11" s="28"/>
@@ -8757,13 +8807,16 @@
       <x:c r="N11" s="28"/>
       <x:c r="O11" s="28"/>
       <x:c r="AB11" s="30"/>
-      <x:c r="AC11" s="34"/>
-      <x:c r="AD11" s="34"/>
-      <x:c r="AM11" s="38"/>
+      <x:c r="AC11" s="30"/>
+      <x:c r="AD11" s="30"/>
+      <x:c r="AE11" s="30"/>
+      <x:c r="AF11" s="34"/>
+      <x:c r="AG11" s="34"/>
       <x:c r="AP11" s="38"/>
       <x:c r="AS11" s="38"/>
       <x:c r="AV11" s="38"/>
-      <x:c r="BC11" s="36"/>
+      <x:c r="AY11" s="38"/>
+      <x:c r="BF11" s="36"/>
     </x:row>
     <x:row r="12">
       <x:c r="C12" s="28"/>
@@ -8775,13 +8828,16 @@
       <x:c r="N12" s="28"/>
       <x:c r="O12" s="28"/>
       <x:c r="AB12" s="30"/>
-      <x:c r="AC12" s="34"/>
-      <x:c r="AD12" s="34"/>
-      <x:c r="AM12" s="38"/>
+      <x:c r="AC12" s="30"/>
+      <x:c r="AD12" s="30"/>
+      <x:c r="AE12" s="30"/>
+      <x:c r="AF12" s="34"/>
+      <x:c r="AG12" s="34"/>
       <x:c r="AP12" s="38"/>
       <x:c r="AS12" s="38"/>
       <x:c r="AV12" s="38"/>
-      <x:c r="BC12" s="36"/>
+      <x:c r="AY12" s="38"/>
+      <x:c r="BF12" s="36"/>
     </x:row>
     <x:row r="13">
       <x:c r="C13" s="28"/>
@@ -8793,13 +8849,16 @@
       <x:c r="N13" s="28"/>
       <x:c r="O13" s="28"/>
       <x:c r="AB13" s="30"/>
-      <x:c r="AC13" s="34"/>
-      <x:c r="AD13" s="34"/>
-      <x:c r="AM13" s="38"/>
+      <x:c r="AC13" s="30"/>
+      <x:c r="AD13" s="30"/>
+      <x:c r="AE13" s="30"/>
+      <x:c r="AF13" s="34"/>
+      <x:c r="AG13" s="34"/>
       <x:c r="AP13" s="38"/>
       <x:c r="AS13" s="38"/>
       <x:c r="AV13" s="38"/>
-      <x:c r="BC13" s="36"/>
+      <x:c r="AY13" s="38"/>
+      <x:c r="BF13" s="36"/>
     </x:row>
     <x:row r="14">
       <x:c r="C14" s="28"/>
@@ -8811,13 +8870,16 @@
       <x:c r="N14" s="28"/>
       <x:c r="O14" s="28"/>
       <x:c r="AB14" s="30"/>
-      <x:c r="AC14" s="34"/>
-      <x:c r="AD14" s="34"/>
-      <x:c r="AM14" s="38"/>
+      <x:c r="AC14" s="30"/>
+      <x:c r="AD14" s="30"/>
+      <x:c r="AE14" s="30"/>
+      <x:c r="AF14" s="34"/>
+      <x:c r="AG14" s="34"/>
       <x:c r="AP14" s="38"/>
       <x:c r="AS14" s="38"/>
       <x:c r="AV14" s="38"/>
-      <x:c r="BC14" s="36"/>
+      <x:c r="AY14" s="38"/>
+      <x:c r="BF14" s="36"/>
     </x:row>
     <x:row r="15">
       <x:c r="C15" s="28"/>
@@ -8829,13 +8891,16 @@
       <x:c r="N15" s="28"/>
       <x:c r="O15" s="28"/>
       <x:c r="AB15" s="30"/>
-      <x:c r="AC15" s="34"/>
-      <x:c r="AD15" s="34"/>
-      <x:c r="AM15" s="38"/>
+      <x:c r="AC15" s="30"/>
+      <x:c r="AD15" s="30"/>
+      <x:c r="AE15" s="30"/>
+      <x:c r="AF15" s="34"/>
+      <x:c r="AG15" s="34"/>
       <x:c r="AP15" s="38"/>
       <x:c r="AS15" s="38"/>
       <x:c r="AV15" s="38"/>
-      <x:c r="BC15" s="36"/>
+      <x:c r="AY15" s="38"/>
+      <x:c r="BF15" s="36"/>
     </x:row>
     <x:row r="16">
       <x:c r="C16" s="28"/>
@@ -8847,13 +8912,16 @@
       <x:c r="N16" s="28"/>
       <x:c r="O16" s="28"/>
       <x:c r="AB16" s="30"/>
-      <x:c r="AC16" s="34"/>
-      <x:c r="AD16" s="34"/>
-      <x:c r="AM16" s="38"/>
+      <x:c r="AC16" s="30"/>
+      <x:c r="AD16" s="30"/>
+      <x:c r="AE16" s="30"/>
+      <x:c r="AF16" s="34"/>
+      <x:c r="AG16" s="34"/>
       <x:c r="AP16" s="38"/>
       <x:c r="AS16" s="38"/>
       <x:c r="AV16" s="38"/>
-      <x:c r="BC16" s="36"/>
+      <x:c r="AY16" s="38"/>
+      <x:c r="BF16" s="36"/>
     </x:row>
     <x:row r="17">
       <x:c r="C17" s="28"/>
@@ -8865,13 +8933,16 @@
       <x:c r="N17" s="28"/>
       <x:c r="O17" s="28"/>
       <x:c r="AB17" s="30"/>
-      <x:c r="AC17" s="34"/>
-      <x:c r="AD17" s="34"/>
-      <x:c r="AM17" s="38"/>
+      <x:c r="AC17" s="30"/>
+      <x:c r="AD17" s="30"/>
+      <x:c r="AE17" s="30"/>
+      <x:c r="AF17" s="34"/>
+      <x:c r="AG17" s="34"/>
       <x:c r="AP17" s="38"/>
       <x:c r="AS17" s="38"/>
       <x:c r="AV17" s="38"/>
-      <x:c r="BC17" s="36"/>
+      <x:c r="AY17" s="38"/>
+      <x:c r="BF17" s="36"/>
     </x:row>
     <x:row r="18">
       <x:c r="C18" s="28"/>
@@ -8883,13 +8954,16 @@
       <x:c r="N18" s="28"/>
       <x:c r="O18" s="28"/>
       <x:c r="AB18" s="30"/>
-      <x:c r="AC18" s="34"/>
-      <x:c r="AD18" s="34"/>
-      <x:c r="AM18" s="38"/>
+      <x:c r="AC18" s="30"/>
+      <x:c r="AD18" s="30"/>
+      <x:c r="AE18" s="30"/>
+      <x:c r="AF18" s="34"/>
+      <x:c r="AG18" s="34"/>
       <x:c r="AP18" s="38"/>
       <x:c r="AS18" s="38"/>
       <x:c r="AV18" s="38"/>
-      <x:c r="BC18" s="36"/>
+      <x:c r="AY18" s="38"/>
+      <x:c r="BF18" s="36"/>
     </x:row>
     <x:row r="19">
       <x:c r="C19" s="28"/>
@@ -8901,13 +8975,16 @@
       <x:c r="N19" s="28"/>
       <x:c r="O19" s="28"/>
       <x:c r="AB19" s="30"/>
-      <x:c r="AC19" s="34"/>
-      <x:c r="AD19" s="34"/>
-      <x:c r="AM19" s="38"/>
+      <x:c r="AC19" s="30"/>
+      <x:c r="AD19" s="30"/>
+      <x:c r="AE19" s="30"/>
+      <x:c r="AF19" s="34"/>
+      <x:c r="AG19" s="34"/>
       <x:c r="AP19" s="38"/>
       <x:c r="AS19" s="38"/>
       <x:c r="AV19" s="38"/>
-      <x:c r="BC19" s="36"/>
+      <x:c r="AY19" s="38"/>
+      <x:c r="BF19" s="36"/>
     </x:row>
     <x:row r="20">
       <x:c r="C20" s="28"/>
@@ -8919,13 +8996,16 @@
       <x:c r="N20" s="28"/>
       <x:c r="O20" s="28"/>
       <x:c r="AB20" s="30"/>
-      <x:c r="AC20" s="34"/>
-      <x:c r="AD20" s="34"/>
-      <x:c r="AM20" s="38"/>
+      <x:c r="AC20" s="30"/>
+      <x:c r="AD20" s="30"/>
+      <x:c r="AE20" s="30"/>
+      <x:c r="AF20" s="34"/>
+      <x:c r="AG20" s="34"/>
       <x:c r="AP20" s="38"/>
       <x:c r="AS20" s="38"/>
       <x:c r="AV20" s="38"/>
-      <x:c r="BC20" s="36"/>
+      <x:c r="AY20" s="38"/>
+      <x:c r="BF20" s="36"/>
     </x:row>
     <x:row r="21">
       <x:c r="C21" s="28"/>
@@ -8937,13 +9017,16 @@
       <x:c r="N21" s="28"/>
       <x:c r="O21" s="28"/>
       <x:c r="AB21" s="30"/>
-      <x:c r="AC21" s="34"/>
-      <x:c r="AD21" s="34"/>
-      <x:c r="AM21" s="38"/>
+      <x:c r="AC21" s="30"/>
+      <x:c r="AD21" s="30"/>
+      <x:c r="AE21" s="30"/>
+      <x:c r="AF21" s="34"/>
+      <x:c r="AG21" s="34"/>
       <x:c r="AP21" s="38"/>
       <x:c r="AS21" s="38"/>
       <x:c r="AV21" s="38"/>
-      <x:c r="BC21" s="36"/>
+      <x:c r="AY21" s="38"/>
+      <x:c r="BF21" s="36"/>
     </x:row>
     <x:row r="22">
       <x:c r="C22" s="28"/>
@@ -8955,13 +9038,16 @@
       <x:c r="N22" s="28"/>
       <x:c r="O22" s="28"/>
       <x:c r="AB22" s="30"/>
-      <x:c r="AC22" s="34"/>
-      <x:c r="AD22" s="34"/>
-      <x:c r="AM22" s="38"/>
+      <x:c r="AC22" s="30"/>
+      <x:c r="AD22" s="30"/>
+      <x:c r="AE22" s="30"/>
+      <x:c r="AF22" s="34"/>
+      <x:c r="AG22" s="34"/>
       <x:c r="AP22" s="38"/>
       <x:c r="AS22" s="38"/>
       <x:c r="AV22" s="38"/>
-      <x:c r="BC22" s="36"/>
+      <x:c r="AY22" s="38"/>
+      <x:c r="BF22" s="36"/>
     </x:row>
     <x:row r="23">
       <x:c r="C23" s="28"/>
@@ -8973,13 +9059,16 @@
       <x:c r="N23" s="28"/>
       <x:c r="O23" s="28"/>
       <x:c r="AB23" s="30"/>
-      <x:c r="AC23" s="34"/>
-      <x:c r="AD23" s="34"/>
-      <x:c r="AM23" s="38"/>
+      <x:c r="AC23" s="30"/>
+      <x:c r="AD23" s="30"/>
+      <x:c r="AE23" s="30"/>
+      <x:c r="AF23" s="34"/>
+      <x:c r="AG23" s="34"/>
       <x:c r="AP23" s="38"/>
       <x:c r="AS23" s="38"/>
       <x:c r="AV23" s="38"/>
-      <x:c r="BC23" s="36"/>
+      <x:c r="AY23" s="38"/>
+      <x:c r="BF23" s="36"/>
     </x:row>
     <x:row r="24">
       <x:c r="C24" s="28"/>
@@ -8991,13 +9080,16 @@
       <x:c r="N24" s="28"/>
       <x:c r="O24" s="28"/>
       <x:c r="AB24" s="30"/>
-      <x:c r="AC24" s="34"/>
-      <x:c r="AD24" s="34"/>
-      <x:c r="AM24" s="38"/>
+      <x:c r="AC24" s="30"/>
+      <x:c r="AD24" s="30"/>
+      <x:c r="AE24" s="30"/>
+      <x:c r="AF24" s="34"/>
+      <x:c r="AG24" s="34"/>
       <x:c r="AP24" s="38"/>
       <x:c r="AS24" s="38"/>
       <x:c r="AV24" s="38"/>
-      <x:c r="BC24" s="36"/>
+      <x:c r="AY24" s="38"/>
+      <x:c r="BF24" s="36"/>
     </x:row>
     <x:row r="25">
       <x:c r="C25" s="28"/>
@@ -9009,13 +9101,16 @@
       <x:c r="N25" s="28"/>
       <x:c r="O25" s="28"/>
       <x:c r="AB25" s="30"/>
-      <x:c r="AC25" s="34"/>
-      <x:c r="AD25" s="34"/>
-      <x:c r="AM25" s="38"/>
+      <x:c r="AC25" s="30"/>
+      <x:c r="AD25" s="30"/>
+      <x:c r="AE25" s="30"/>
+      <x:c r="AF25" s="34"/>
+      <x:c r="AG25" s="34"/>
       <x:c r="AP25" s="38"/>
       <x:c r="AS25" s="38"/>
       <x:c r="AV25" s="38"/>
-      <x:c r="BC25" s="36"/>
+      <x:c r="AY25" s="38"/>
+      <x:c r="BF25" s="36"/>
     </x:row>
     <x:row r="26">
       <x:c r="C26" s="28"/>
@@ -9027,13 +9122,16 @@
       <x:c r="N26" s="28"/>
       <x:c r="O26" s="28"/>
       <x:c r="AB26" s="30"/>
-      <x:c r="AC26" s="34"/>
-      <x:c r="AD26" s="34"/>
-      <x:c r="AM26" s="38"/>
+      <x:c r="AC26" s="30"/>
+      <x:c r="AD26" s="30"/>
+      <x:c r="AE26" s="30"/>
+      <x:c r="AF26" s="34"/>
+      <x:c r="AG26" s="34"/>
       <x:c r="AP26" s="38"/>
       <x:c r="AS26" s="38"/>
       <x:c r="AV26" s="38"/>
-      <x:c r="BC26" s="36"/>
+      <x:c r="AY26" s="38"/>
+      <x:c r="BF26" s="36"/>
     </x:row>
     <x:row r="27">
       <x:c r="C27" s="28"/>
@@ -9045,13 +9143,16 @@
       <x:c r="N27" s="28"/>
       <x:c r="O27" s="28"/>
       <x:c r="AB27" s="30"/>
-      <x:c r="AC27" s="34"/>
-      <x:c r="AD27" s="34"/>
-      <x:c r="AM27" s="38"/>
+      <x:c r="AC27" s="30"/>
+      <x:c r="AD27" s="30"/>
+      <x:c r="AE27" s="30"/>
+      <x:c r="AF27" s="34"/>
+      <x:c r="AG27" s="34"/>
       <x:c r="AP27" s="38"/>
       <x:c r="AS27" s="38"/>
       <x:c r="AV27" s="38"/>
-      <x:c r="BC27" s="36"/>
+      <x:c r="AY27" s="38"/>
+      <x:c r="BF27" s="36"/>
     </x:row>
     <x:row r="28">
       <x:c r="C28" s="28"/>
@@ -9063,13 +9164,16 @@
       <x:c r="N28" s="28"/>
       <x:c r="O28" s="28"/>
       <x:c r="AB28" s="30"/>
-      <x:c r="AC28" s="34"/>
-      <x:c r="AD28" s="34"/>
-      <x:c r="AM28" s="38"/>
+      <x:c r="AC28" s="30"/>
+      <x:c r="AD28" s="30"/>
+      <x:c r="AE28" s="30"/>
+      <x:c r="AF28" s="34"/>
+      <x:c r="AG28" s="34"/>
       <x:c r="AP28" s="38"/>
       <x:c r="AS28" s="38"/>
       <x:c r="AV28" s="38"/>
-      <x:c r="BC28" s="36"/>
+      <x:c r="AY28" s="38"/>
+      <x:c r="BF28" s="36"/>
     </x:row>
     <x:row r="29">
       <x:c r="C29" s="28"/>
@@ -9081,13 +9185,16 @@
       <x:c r="N29" s="28"/>
       <x:c r="O29" s="28"/>
       <x:c r="AB29" s="30"/>
-      <x:c r="AC29" s="34"/>
-      <x:c r="AD29" s="34"/>
-      <x:c r="AM29" s="38"/>
+      <x:c r="AC29" s="30"/>
+      <x:c r="AD29" s="30"/>
+      <x:c r="AE29" s="30"/>
+      <x:c r="AF29" s="34"/>
+      <x:c r="AG29" s="34"/>
       <x:c r="AP29" s="38"/>
       <x:c r="AS29" s="38"/>
       <x:c r="AV29" s="38"/>
-      <x:c r="BC29" s="36"/>
+      <x:c r="AY29" s="38"/>
+      <x:c r="BF29" s="36"/>
     </x:row>
     <x:row r="30">
       <x:c r="C30" s="28"/>
@@ -9099,13 +9206,16 @@
       <x:c r="N30" s="28"/>
       <x:c r="O30" s="28"/>
       <x:c r="AB30" s="30"/>
-      <x:c r="AC30" s="34"/>
-      <x:c r="AD30" s="34"/>
-      <x:c r="AM30" s="38"/>
+      <x:c r="AC30" s="30"/>
+      <x:c r="AD30" s="30"/>
+      <x:c r="AE30" s="30"/>
+      <x:c r="AF30" s="34"/>
+      <x:c r="AG30" s="34"/>
       <x:c r="AP30" s="38"/>
       <x:c r="AS30" s="38"/>
       <x:c r="AV30" s="38"/>
-      <x:c r="BC30" s="36"/>
+      <x:c r="AY30" s="38"/>
+      <x:c r="BF30" s="36"/>
     </x:row>
     <x:row r="31">
       <x:c r="C31" s="28"/>
@@ -9117,13 +9227,16 @@
       <x:c r="N31" s="28"/>
       <x:c r="O31" s="28"/>
       <x:c r="AB31" s="30"/>
-      <x:c r="AC31" s="34"/>
-      <x:c r="AD31" s="34"/>
-      <x:c r="AM31" s="38"/>
+      <x:c r="AC31" s="30"/>
+      <x:c r="AD31" s="30"/>
+      <x:c r="AE31" s="30"/>
+      <x:c r="AF31" s="34"/>
+      <x:c r="AG31" s="34"/>
       <x:c r="AP31" s="38"/>
       <x:c r="AS31" s="38"/>
       <x:c r="AV31" s="38"/>
-      <x:c r="BC31" s="36"/>
+      <x:c r="AY31" s="38"/>
+      <x:c r="BF31" s="36"/>
     </x:row>
     <x:row r="32">
       <x:c r="C32" s="28"/>
@@ -9135,13 +9248,16 @@
       <x:c r="N32" s="28"/>
       <x:c r="O32" s="28"/>
       <x:c r="AB32" s="30"/>
-      <x:c r="AC32" s="34"/>
-      <x:c r="AD32" s="34"/>
-      <x:c r="AM32" s="38"/>
+      <x:c r="AC32" s="30"/>
+      <x:c r="AD32" s="30"/>
+      <x:c r="AE32" s="30"/>
+      <x:c r="AF32" s="34"/>
+      <x:c r="AG32" s="34"/>
       <x:c r="AP32" s="38"/>
       <x:c r="AS32" s="38"/>
       <x:c r="AV32" s="38"/>
-      <x:c r="BC32" s="36"/>
+      <x:c r="AY32" s="38"/>
+      <x:c r="BF32" s="36"/>
     </x:row>
     <x:row r="33">
       <x:c r="C33" s="28"/>
@@ -9153,13 +9269,16 @@
       <x:c r="N33" s="28"/>
       <x:c r="O33" s="28"/>
       <x:c r="AB33" s="30"/>
-      <x:c r="AC33" s="34"/>
-      <x:c r="AD33" s="34"/>
-      <x:c r="AM33" s="38"/>
+      <x:c r="AC33" s="30"/>
+      <x:c r="AD33" s="30"/>
+      <x:c r="AE33" s="30"/>
+      <x:c r="AF33" s="34"/>
+      <x:c r="AG33" s="34"/>
       <x:c r="AP33" s="38"/>
       <x:c r="AS33" s="38"/>
       <x:c r="AV33" s="38"/>
-      <x:c r="BC33" s="36"/>
+      <x:c r="AY33" s="38"/>
+      <x:c r="BF33" s="36"/>
     </x:row>
     <x:row r="34">
       <x:c r="C34" s="28"/>
@@ -9171,13 +9290,16 @@
       <x:c r="N34" s="28"/>
       <x:c r="O34" s="28"/>
       <x:c r="AB34" s="30"/>
-      <x:c r="AC34" s="34"/>
-      <x:c r="AD34" s="34"/>
-      <x:c r="AM34" s="38"/>
+      <x:c r="AC34" s="30"/>
+      <x:c r="AD34" s="30"/>
+      <x:c r="AE34" s="30"/>
+      <x:c r="AF34" s="34"/>
+      <x:c r="AG34" s="34"/>
       <x:c r="AP34" s="38"/>
       <x:c r="AS34" s="38"/>
       <x:c r="AV34" s="38"/>
-      <x:c r="BC34" s="36"/>
+      <x:c r="AY34" s="38"/>
+      <x:c r="BF34" s="36"/>
     </x:row>
     <x:row r="35">
       <x:c r="C35" s="28"/>
@@ -9189,13 +9311,16 @@
       <x:c r="N35" s="28"/>
       <x:c r="O35" s="28"/>
       <x:c r="AB35" s="30"/>
-      <x:c r="AC35" s="34"/>
-      <x:c r="AD35" s="34"/>
-      <x:c r="AM35" s="38"/>
+      <x:c r="AC35" s="30"/>
+      <x:c r="AD35" s="30"/>
+      <x:c r="AE35" s="30"/>
+      <x:c r="AF35" s="34"/>
+      <x:c r="AG35" s="34"/>
       <x:c r="AP35" s="38"/>
       <x:c r="AS35" s="38"/>
       <x:c r="AV35" s="38"/>
-      <x:c r="BC35" s="36"/>
+      <x:c r="AY35" s="38"/>
+      <x:c r="BF35" s="36"/>
     </x:row>
     <x:row r="36">
       <x:c r="C36" s="28"/>
@@ -9207,13 +9332,16 @@
       <x:c r="N36" s="28"/>
       <x:c r="O36" s="28"/>
       <x:c r="AB36" s="30"/>
-      <x:c r="AC36" s="34"/>
-      <x:c r="AD36" s="34"/>
-      <x:c r="AM36" s="38"/>
+      <x:c r="AC36" s="30"/>
+      <x:c r="AD36" s="30"/>
+      <x:c r="AE36" s="30"/>
+      <x:c r="AF36" s="34"/>
+      <x:c r="AG36" s="34"/>
       <x:c r="AP36" s="38"/>
       <x:c r="AS36" s="38"/>
       <x:c r="AV36" s="38"/>
-      <x:c r="BC36" s="36"/>
+      <x:c r="AY36" s="38"/>
+      <x:c r="BF36" s="36"/>
     </x:row>
     <x:row r="37">
       <x:c r="C37" s="28"/>
@@ -9225,13 +9353,16 @@
       <x:c r="N37" s="28"/>
       <x:c r="O37" s="28"/>
       <x:c r="AB37" s="30"/>
-      <x:c r="AC37" s="34"/>
-      <x:c r="AD37" s="34"/>
-      <x:c r="AM37" s="38"/>
+      <x:c r="AC37" s="30"/>
+      <x:c r="AD37" s="30"/>
+      <x:c r="AE37" s="30"/>
+      <x:c r="AF37" s="34"/>
+      <x:c r="AG37" s="34"/>
       <x:c r="AP37" s="38"/>
       <x:c r="AS37" s="38"/>
       <x:c r="AV37" s="38"/>
-      <x:c r="BC37" s="36"/>
+      <x:c r="AY37" s="38"/>
+      <x:c r="BF37" s="36"/>
     </x:row>
     <x:row r="38">
       <x:c r="C38" s="28"/>
@@ -9243,13 +9374,16 @@
       <x:c r="N38" s="28"/>
       <x:c r="O38" s="28"/>
       <x:c r="AB38" s="30"/>
-      <x:c r="AC38" s="34"/>
-      <x:c r="AD38" s="34"/>
-      <x:c r="AM38" s="38"/>
+      <x:c r="AC38" s="30"/>
+      <x:c r="AD38" s="30"/>
+      <x:c r="AE38" s="30"/>
+      <x:c r="AF38" s="34"/>
+      <x:c r="AG38" s="34"/>
       <x:c r="AP38" s="38"/>
       <x:c r="AS38" s="38"/>
       <x:c r="AV38" s="38"/>
-      <x:c r="BC38" s="36"/>
+      <x:c r="AY38" s="38"/>
+      <x:c r="BF38" s="36"/>
     </x:row>
     <x:row r="39">
       <x:c r="C39" s="28"/>
@@ -9261,13 +9395,16 @@
       <x:c r="N39" s="28"/>
       <x:c r="O39" s="28"/>
       <x:c r="AB39" s="30"/>
-      <x:c r="AC39" s="34"/>
-      <x:c r="AD39" s="34"/>
-      <x:c r="AM39" s="38"/>
+      <x:c r="AC39" s="30"/>
+      <x:c r="AD39" s="30"/>
+      <x:c r="AE39" s="30"/>
+      <x:c r="AF39" s="34"/>
+      <x:c r="AG39" s="34"/>
       <x:c r="AP39" s="38"/>
       <x:c r="AS39" s="38"/>
       <x:c r="AV39" s="38"/>
-      <x:c r="BC39" s="36"/>
+      <x:c r="AY39" s="38"/>
+      <x:c r="BF39" s="36"/>
     </x:row>
     <x:row r="40">
       <x:c r="C40" s="28"/>
@@ -9279,13 +9416,16 @@
       <x:c r="N40" s="28"/>
       <x:c r="O40" s="28"/>
       <x:c r="AB40" s="30"/>
-      <x:c r="AC40" s="34"/>
-      <x:c r="AD40" s="34"/>
-      <x:c r="AM40" s="38"/>
+      <x:c r="AC40" s="30"/>
+      <x:c r="AD40" s="30"/>
+      <x:c r="AE40" s="30"/>
+      <x:c r="AF40" s="34"/>
+      <x:c r="AG40" s="34"/>
       <x:c r="AP40" s="38"/>
       <x:c r="AS40" s="38"/>
       <x:c r="AV40" s="38"/>
-      <x:c r="BC40" s="36"/>
+      <x:c r="AY40" s="38"/>
+      <x:c r="BF40" s="36"/>
     </x:row>
     <x:row r="41">
       <x:c r="C41" s="28"/>
@@ -9297,13 +9437,16 @@
       <x:c r="N41" s="28"/>
       <x:c r="O41" s="28"/>
       <x:c r="AB41" s="30"/>
-      <x:c r="AC41" s="34"/>
-      <x:c r="AD41" s="34"/>
-      <x:c r="AM41" s="38"/>
+      <x:c r="AC41" s="30"/>
+      <x:c r="AD41" s="30"/>
+      <x:c r="AE41" s="30"/>
+      <x:c r="AF41" s="34"/>
+      <x:c r="AG41" s="34"/>
       <x:c r="AP41" s="38"/>
       <x:c r="AS41" s="38"/>
       <x:c r="AV41" s="38"/>
-      <x:c r="BC41" s="36"/>
+      <x:c r="AY41" s="38"/>
+      <x:c r="BF41" s="36"/>
     </x:row>
     <x:row r="42">
       <x:c r="C42" s="28"/>
@@ -9315,13 +9458,16 @@
       <x:c r="N42" s="28"/>
       <x:c r="O42" s="28"/>
       <x:c r="AB42" s="30"/>
-      <x:c r="AC42" s="34"/>
-      <x:c r="AD42" s="34"/>
-      <x:c r="AM42" s="38"/>
+      <x:c r="AC42" s="30"/>
+      <x:c r="AD42" s="30"/>
+      <x:c r="AE42" s="30"/>
+      <x:c r="AF42" s="34"/>
+      <x:c r="AG42" s="34"/>
       <x:c r="AP42" s="38"/>
       <x:c r="AS42" s="38"/>
       <x:c r="AV42" s="38"/>
-      <x:c r="BC42" s="36"/>
+      <x:c r="AY42" s="38"/>
+      <x:c r="BF42" s="36"/>
     </x:row>
     <x:row r="43">
       <x:c r="C43" s="28"/>
@@ -9333,13 +9479,16 @@
       <x:c r="N43" s="28"/>
       <x:c r="O43" s="28"/>
       <x:c r="AB43" s="30"/>
-      <x:c r="AC43" s="34"/>
-      <x:c r="AD43" s="34"/>
-      <x:c r="AM43" s="38"/>
+      <x:c r="AC43" s="30"/>
+      <x:c r="AD43" s="30"/>
+      <x:c r="AE43" s="30"/>
+      <x:c r="AF43" s="34"/>
+      <x:c r="AG43" s="34"/>
       <x:c r="AP43" s="38"/>
       <x:c r="AS43" s="38"/>
       <x:c r="AV43" s="38"/>
-      <x:c r="BC43" s="36"/>
+      <x:c r="AY43" s="38"/>
+      <x:c r="BF43" s="36"/>
     </x:row>
     <x:row r="44">
       <x:c r="C44" s="28"/>
@@ -9351,13 +9500,16 @@
       <x:c r="N44" s="28"/>
       <x:c r="O44" s="28"/>
       <x:c r="AB44" s="30"/>
-      <x:c r="AC44" s="34"/>
-      <x:c r="AD44" s="34"/>
-      <x:c r="AM44" s="38"/>
+      <x:c r="AC44" s="30"/>
+      <x:c r="AD44" s="30"/>
+      <x:c r="AE44" s="30"/>
+      <x:c r="AF44" s="34"/>
+      <x:c r="AG44" s="34"/>
       <x:c r="AP44" s="38"/>
       <x:c r="AS44" s="38"/>
       <x:c r="AV44" s="38"/>
-      <x:c r="BC44" s="36"/>
+      <x:c r="AY44" s="38"/>
+      <x:c r="BF44" s="36"/>
     </x:row>
     <x:row r="45">
       <x:c r="C45" s="28"/>
@@ -9369,13 +9521,16 @@
       <x:c r="N45" s="28"/>
       <x:c r="O45" s="28"/>
       <x:c r="AB45" s="30"/>
-      <x:c r="AC45" s="34"/>
-      <x:c r="AD45" s="34"/>
-      <x:c r="AM45" s="38"/>
+      <x:c r="AC45" s="30"/>
+      <x:c r="AD45" s="30"/>
+      <x:c r="AE45" s="30"/>
+      <x:c r="AF45" s="34"/>
+      <x:c r="AG45" s="34"/>
       <x:c r="AP45" s="38"/>
       <x:c r="AS45" s="38"/>
       <x:c r="AV45" s="38"/>
-      <x:c r="BC45" s="36"/>
+      <x:c r="AY45" s="38"/>
+      <x:c r="BF45" s="36"/>
     </x:row>
     <x:row r="46">
       <x:c r="C46" s="28"/>
@@ -9387,13 +9542,16 @@
       <x:c r="N46" s="28"/>
       <x:c r="O46" s="28"/>
       <x:c r="AB46" s="30"/>
-      <x:c r="AC46" s="34"/>
-      <x:c r="AD46" s="34"/>
-      <x:c r="AM46" s="38"/>
+      <x:c r="AC46" s="30"/>
+      <x:c r="AD46" s="30"/>
+      <x:c r="AE46" s="30"/>
+      <x:c r="AF46" s="34"/>
+      <x:c r="AG46" s="34"/>
       <x:c r="AP46" s="38"/>
       <x:c r="AS46" s="38"/>
       <x:c r="AV46" s="38"/>
-      <x:c r="BC46" s="36"/>
+      <x:c r="AY46" s="38"/>
+      <x:c r="BF46" s="36"/>
     </x:row>
     <x:row r="47">
       <x:c r="C47" s="28"/>
@@ -9405,13 +9563,16 @@
       <x:c r="N47" s="28"/>
       <x:c r="O47" s="28"/>
       <x:c r="AB47" s="30"/>
-      <x:c r="AC47" s="34"/>
-      <x:c r="AD47" s="34"/>
-      <x:c r="AM47" s="38"/>
+      <x:c r="AC47" s="30"/>
+      <x:c r="AD47" s="30"/>
+      <x:c r="AE47" s="30"/>
+      <x:c r="AF47" s="34"/>
+      <x:c r="AG47" s="34"/>
       <x:c r="AP47" s="38"/>
       <x:c r="AS47" s="38"/>
       <x:c r="AV47" s="38"/>
-      <x:c r="BC47" s="36"/>
+      <x:c r="AY47" s="38"/>
+      <x:c r="BF47" s="36"/>
     </x:row>
     <x:row r="48">
       <x:c r="C48" s="28"/>
@@ -9423,13 +9584,16 @@
       <x:c r="N48" s="28"/>
       <x:c r="O48" s="28"/>
       <x:c r="AB48" s="30"/>
-      <x:c r="AC48" s="34"/>
-      <x:c r="AD48" s="34"/>
-      <x:c r="AM48" s="38"/>
+      <x:c r="AC48" s="30"/>
+      <x:c r="AD48" s="30"/>
+      <x:c r="AE48" s="30"/>
+      <x:c r="AF48" s="34"/>
+      <x:c r="AG48" s="34"/>
       <x:c r="AP48" s="38"/>
       <x:c r="AS48" s="38"/>
       <x:c r="AV48" s="38"/>
-      <x:c r="BC48" s="36"/>
+      <x:c r="AY48" s="38"/>
+      <x:c r="BF48" s="36"/>
     </x:row>
     <x:row r="49">
       <x:c r="C49" s="28"/>
@@ -9441,13 +9605,16 @@
       <x:c r="N49" s="28"/>
       <x:c r="O49" s="28"/>
       <x:c r="AB49" s="30"/>
-      <x:c r="AC49" s="34"/>
-      <x:c r="AD49" s="34"/>
-      <x:c r="AM49" s="38"/>
+      <x:c r="AC49" s="30"/>
+      <x:c r="AD49" s="30"/>
+      <x:c r="AE49" s="30"/>
+      <x:c r="AF49" s="34"/>
+      <x:c r="AG49" s="34"/>
       <x:c r="AP49" s="38"/>
       <x:c r="AS49" s="38"/>
       <x:c r="AV49" s="38"/>
-      <x:c r="BC49" s="36"/>
+      <x:c r="AY49" s="38"/>
+      <x:c r="BF49" s="36"/>
     </x:row>
     <x:row r="50">
       <x:c r="C50" s="28"/>
@@ -9459,13 +9626,16 @@
       <x:c r="N50" s="28"/>
       <x:c r="O50" s="28"/>
       <x:c r="AB50" s="30"/>
-      <x:c r="AC50" s="34"/>
-      <x:c r="AD50" s="34"/>
-      <x:c r="AM50" s="38"/>
+      <x:c r="AC50" s="30"/>
+      <x:c r="AD50" s="30"/>
+      <x:c r="AE50" s="30"/>
+      <x:c r="AF50" s="34"/>
+      <x:c r="AG50" s="34"/>
       <x:c r="AP50" s="38"/>
       <x:c r="AS50" s="38"/>
       <x:c r="AV50" s="38"/>
-      <x:c r="BC50" s="36"/>
+      <x:c r="AY50" s="38"/>
+      <x:c r="BF50" s="36"/>
     </x:row>
     <x:row r="51">
       <x:c r="C51" s="28"/>
@@ -9477,13 +9647,16 @@
       <x:c r="N51" s="28"/>
       <x:c r="O51" s="28"/>
       <x:c r="AB51" s="30"/>
-      <x:c r="AC51" s="34"/>
-      <x:c r="AD51" s="34"/>
-      <x:c r="AM51" s="38"/>
+      <x:c r="AC51" s="30"/>
+      <x:c r="AD51" s="30"/>
+      <x:c r="AE51" s="30"/>
+      <x:c r="AF51" s="34"/>
+      <x:c r="AG51" s="34"/>
       <x:c r="AP51" s="38"/>
       <x:c r="AS51" s="38"/>
       <x:c r="AV51" s="38"/>
-      <x:c r="BC51" s="36"/>
+      <x:c r="AY51" s="38"/>
+      <x:c r="BF51" s="36"/>
     </x:row>
     <x:row r="52">
       <x:c r="C52" s="28"/>
@@ -9495,13 +9668,16 @@
       <x:c r="N52" s="28"/>
       <x:c r="O52" s="28"/>
       <x:c r="AB52" s="30"/>
-      <x:c r="AC52" s="34"/>
-      <x:c r="AD52" s="34"/>
-      <x:c r="AM52" s="38"/>
+      <x:c r="AC52" s="30"/>
+      <x:c r="AD52" s="30"/>
+      <x:c r="AE52" s="30"/>
+      <x:c r="AF52" s="34"/>
+      <x:c r="AG52" s="34"/>
       <x:c r="AP52" s="38"/>
       <x:c r="AS52" s="38"/>
       <x:c r="AV52" s="38"/>
-      <x:c r="BC52" s="36"/>
+      <x:c r="AY52" s="38"/>
+      <x:c r="BF52" s="36"/>
     </x:row>
     <x:row r="53">
       <x:c r="C53" s="28"/>
@@ -9513,13 +9689,16 @@
       <x:c r="N53" s="28"/>
       <x:c r="O53" s="28"/>
       <x:c r="AB53" s="30"/>
-      <x:c r="AC53" s="34"/>
-      <x:c r="AD53" s="34"/>
-      <x:c r="AM53" s="38"/>
+      <x:c r="AC53" s="30"/>
+      <x:c r="AD53" s="30"/>
+      <x:c r="AE53" s="30"/>
+      <x:c r="AF53" s="34"/>
+      <x:c r="AG53" s="34"/>
       <x:c r="AP53" s="38"/>
       <x:c r="AS53" s="38"/>
       <x:c r="AV53" s="38"/>
-      <x:c r="BC53" s="36"/>
+      <x:c r="AY53" s="38"/>
+      <x:c r="BF53" s="36"/>
     </x:row>
     <x:row r="54">
       <x:c r="C54" s="28"/>
@@ -9531,13 +9710,16 @@
       <x:c r="N54" s="28"/>
       <x:c r="O54" s="28"/>
       <x:c r="AB54" s="30"/>
-      <x:c r="AC54" s="34"/>
-      <x:c r="AD54" s="34"/>
-      <x:c r="AM54" s="38"/>
+      <x:c r="AC54" s="30"/>
+      <x:c r="AD54" s="30"/>
+      <x:c r="AE54" s="30"/>
+      <x:c r="AF54" s="34"/>
+      <x:c r="AG54" s="34"/>
       <x:c r="AP54" s="38"/>
       <x:c r="AS54" s="38"/>
       <x:c r="AV54" s="38"/>
-      <x:c r="BC54" s="36"/>
+      <x:c r="AY54" s="38"/>
+      <x:c r="BF54" s="36"/>
     </x:row>
     <x:row r="55">
       <x:c r="C55" s="28"/>
@@ -9549,13 +9731,16 @@
       <x:c r="N55" s="28"/>
       <x:c r="O55" s="28"/>
       <x:c r="AB55" s="30"/>
-      <x:c r="AC55" s="34"/>
-      <x:c r="AD55" s="34"/>
-      <x:c r="AM55" s="38"/>
+      <x:c r="AC55" s="30"/>
+      <x:c r="AD55" s="30"/>
+      <x:c r="AE55" s="30"/>
+      <x:c r="AF55" s="34"/>
+      <x:c r="AG55" s="34"/>
       <x:c r="AP55" s="38"/>
       <x:c r="AS55" s="38"/>
       <x:c r="AV55" s="38"/>
-      <x:c r="BC55" s="36"/>
+      <x:c r="AY55" s="38"/>
+      <x:c r="BF55" s="36"/>
     </x:row>
     <x:row r="56">
       <x:c r="C56" s="28"/>
@@ -9567,13 +9752,16 @@
       <x:c r="N56" s="28"/>
       <x:c r="O56" s="28"/>
       <x:c r="AB56" s="30"/>
-      <x:c r="AC56" s="34"/>
-      <x:c r="AD56" s="34"/>
-      <x:c r="AM56" s="38"/>
+      <x:c r="AC56" s="30"/>
+      <x:c r="AD56" s="30"/>
+      <x:c r="AE56" s="30"/>
+      <x:c r="AF56" s="34"/>
+      <x:c r="AG56" s="34"/>
       <x:c r="AP56" s="38"/>
       <x:c r="AS56" s="38"/>
       <x:c r="AV56" s="38"/>
-      <x:c r="BC56" s="36"/>
+      <x:c r="AY56" s="38"/>
+      <x:c r="BF56" s="36"/>
     </x:row>
     <x:row r="57">
       <x:c r="C57" s="28"/>
@@ -9585,13 +9773,16 @@
       <x:c r="N57" s="28"/>
       <x:c r="O57" s="28"/>
       <x:c r="AB57" s="30"/>
-      <x:c r="AC57" s="34"/>
-      <x:c r="AD57" s="34"/>
-      <x:c r="AM57" s="38"/>
+      <x:c r="AC57" s="30"/>
+      <x:c r="AD57" s="30"/>
+      <x:c r="AE57" s="30"/>
+      <x:c r="AF57" s="34"/>
+      <x:c r="AG57" s="34"/>
       <x:c r="AP57" s="38"/>
       <x:c r="AS57" s="38"/>
       <x:c r="AV57" s="38"/>
-      <x:c r="BC57" s="36"/>
+      <x:c r="AY57" s="38"/>
+      <x:c r="BF57" s="36"/>
     </x:row>
     <x:row r="58">
       <x:c r="C58" s="28"/>
@@ -9603,13 +9794,16 @@
       <x:c r="N58" s="28"/>
       <x:c r="O58" s="28"/>
       <x:c r="AB58" s="30"/>
-      <x:c r="AC58" s="34"/>
-      <x:c r="AD58" s="34"/>
-      <x:c r="AM58" s="38"/>
+      <x:c r="AC58" s="30"/>
+      <x:c r="AD58" s="30"/>
+      <x:c r="AE58" s="30"/>
+      <x:c r="AF58" s="34"/>
+      <x:c r="AG58" s="34"/>
       <x:c r="AP58" s="38"/>
       <x:c r="AS58" s="38"/>
       <x:c r="AV58" s="38"/>
-      <x:c r="BC58" s="36"/>
+      <x:c r="AY58" s="38"/>
+      <x:c r="BF58" s="36"/>
     </x:row>
     <x:row r="59">
       <x:c r="C59" s="28"/>
@@ -9621,13 +9815,16 @@
       <x:c r="N59" s="28"/>
       <x:c r="O59" s="28"/>
       <x:c r="AB59" s="30"/>
-      <x:c r="AC59" s="34"/>
-      <x:c r="AD59" s="34"/>
-      <x:c r="AM59" s="38"/>
+      <x:c r="AC59" s="30"/>
+      <x:c r="AD59" s="30"/>
+      <x:c r="AE59" s="30"/>
+      <x:c r="AF59" s="34"/>
+      <x:c r="AG59" s="34"/>
       <x:c r="AP59" s="38"/>
       <x:c r="AS59" s="38"/>
       <x:c r="AV59" s="38"/>
-      <x:c r="BC59" s="36"/>
+      <x:c r="AY59" s="38"/>
+      <x:c r="BF59" s="36"/>
     </x:row>
     <x:row r="60">
       <x:c r="C60" s="28"/>
@@ -9639,13 +9836,16 @@
       <x:c r="N60" s="28"/>
       <x:c r="O60" s="28"/>
       <x:c r="AB60" s="30"/>
-      <x:c r="AC60" s="34"/>
-      <x:c r="AD60" s="34"/>
-      <x:c r="AM60" s="38"/>
+      <x:c r="AC60" s="30"/>
+      <x:c r="AD60" s="30"/>
+      <x:c r="AE60" s="30"/>
+      <x:c r="AF60" s="34"/>
+      <x:c r="AG60" s="34"/>
       <x:c r="AP60" s="38"/>
       <x:c r="AS60" s="38"/>
       <x:c r="AV60" s="38"/>
-      <x:c r="BC60" s="36"/>
+      <x:c r="AY60" s="38"/>
+      <x:c r="BF60" s="36"/>
     </x:row>
     <x:row r="61">
       <x:c r="C61" s="28"/>
@@ -9657,13 +9857,16 @@
       <x:c r="N61" s="28"/>
       <x:c r="O61" s="28"/>
       <x:c r="AB61" s="30"/>
-      <x:c r="AC61" s="34"/>
-      <x:c r="AD61" s="34"/>
-      <x:c r="AM61" s="38"/>
+      <x:c r="AC61" s="30"/>
+      <x:c r="AD61" s="30"/>
+      <x:c r="AE61" s="30"/>
+      <x:c r="AF61" s="34"/>
+      <x:c r="AG61" s="34"/>
       <x:c r="AP61" s="38"/>
       <x:c r="AS61" s="38"/>
       <x:c r="AV61" s="38"/>
-      <x:c r="BC61" s="36"/>
+      <x:c r="AY61" s="38"/>
+      <x:c r="BF61" s="36"/>
     </x:row>
     <x:row r="62">
       <x:c r="C62" s="28"/>
@@ -9675,13 +9878,16 @@
       <x:c r="N62" s="28"/>
       <x:c r="O62" s="28"/>
       <x:c r="AB62" s="30"/>
-      <x:c r="AC62" s="34"/>
-      <x:c r="AD62" s="34"/>
-      <x:c r="AM62" s="38"/>
+      <x:c r="AC62" s="30"/>
+      <x:c r="AD62" s="30"/>
+      <x:c r="AE62" s="30"/>
+      <x:c r="AF62" s="34"/>
+      <x:c r="AG62" s="34"/>
       <x:c r="AP62" s="38"/>
       <x:c r="AS62" s="38"/>
       <x:c r="AV62" s="38"/>
-      <x:c r="BC62" s="36"/>
+      <x:c r="AY62" s="38"/>
+      <x:c r="BF62" s="36"/>
     </x:row>
     <x:row r="63">
       <x:c r="C63" s="28"/>
@@ -9693,13 +9899,16 @@
       <x:c r="N63" s="28"/>
       <x:c r="O63" s="28"/>
       <x:c r="AB63" s="30"/>
-      <x:c r="AC63" s="34"/>
-      <x:c r="AD63" s="34"/>
-      <x:c r="AM63" s="38"/>
+      <x:c r="AC63" s="30"/>
+      <x:c r="AD63" s="30"/>
+      <x:c r="AE63" s="30"/>
+      <x:c r="AF63" s="34"/>
+      <x:c r="AG63" s="34"/>
       <x:c r="AP63" s="38"/>
       <x:c r="AS63" s="38"/>
       <x:c r="AV63" s="38"/>
-      <x:c r="BC63" s="36"/>
+      <x:c r="AY63" s="38"/>
+      <x:c r="BF63" s="36"/>
     </x:row>
     <x:row r="64">
       <x:c r="C64" s="28"/>
@@ -9711,13 +9920,16 @@
       <x:c r="N64" s="28"/>
       <x:c r="O64" s="28"/>
       <x:c r="AB64" s="30"/>
-      <x:c r="AC64" s="34"/>
-      <x:c r="AD64" s="34"/>
-      <x:c r="AM64" s="38"/>
+      <x:c r="AC64" s="30"/>
+      <x:c r="AD64" s="30"/>
+      <x:c r="AE64" s="30"/>
+      <x:c r="AF64" s="34"/>
+      <x:c r="AG64" s="34"/>
       <x:c r="AP64" s="38"/>
       <x:c r="AS64" s="38"/>
       <x:c r="AV64" s="38"/>
-      <x:c r="BC64" s="36"/>
+      <x:c r="AY64" s="38"/>
+      <x:c r="BF64" s="36"/>
     </x:row>
     <x:row r="65">
       <x:c r="C65" s="28"/>
@@ -9729,13 +9941,16 @@
       <x:c r="N65" s="28"/>
       <x:c r="O65" s="28"/>
       <x:c r="AB65" s="30"/>
-      <x:c r="AC65" s="34"/>
-      <x:c r="AD65" s="34"/>
-      <x:c r="AM65" s="38"/>
+      <x:c r="AC65" s="30"/>
+      <x:c r="AD65" s="30"/>
+      <x:c r="AE65" s="30"/>
+      <x:c r="AF65" s="34"/>
+      <x:c r="AG65" s="34"/>
       <x:c r="AP65" s="38"/>
       <x:c r="AS65" s="38"/>
       <x:c r="AV65" s="38"/>
-      <x:c r="BC65" s="36"/>
+      <x:c r="AY65" s="38"/>
+      <x:c r="BF65" s="36"/>
     </x:row>
     <x:row r="66">
       <x:c r="C66" s="28"/>
@@ -9747,13 +9962,16 @@
       <x:c r="N66" s="28"/>
       <x:c r="O66" s="28"/>
       <x:c r="AB66" s="30"/>
-      <x:c r="AC66" s="34"/>
-      <x:c r="AD66" s="34"/>
-      <x:c r="AM66" s="38"/>
+      <x:c r="AC66" s="30"/>
+      <x:c r="AD66" s="30"/>
+      <x:c r="AE66" s="30"/>
+      <x:c r="AF66" s="34"/>
+      <x:c r="AG66" s="34"/>
       <x:c r="AP66" s="38"/>
       <x:c r="AS66" s="38"/>
       <x:c r="AV66" s="38"/>
-      <x:c r="BC66" s="36"/>
+      <x:c r="AY66" s="38"/>
+      <x:c r="BF66" s="36"/>
     </x:row>
     <x:row r="67">
       <x:c r="C67" s="28"/>
@@ -9765,13 +9983,16 @@
       <x:c r="N67" s="28"/>
       <x:c r="O67" s="28"/>
       <x:c r="AB67" s="30"/>
-      <x:c r="AC67" s="34"/>
-      <x:c r="AD67" s="34"/>
-      <x:c r="AM67" s="38"/>
+      <x:c r="AC67" s="30"/>
+      <x:c r="AD67" s="30"/>
+      <x:c r="AE67" s="30"/>
+      <x:c r="AF67" s="34"/>
+      <x:c r="AG67" s="34"/>
       <x:c r="AP67" s="38"/>
       <x:c r="AS67" s="38"/>
       <x:c r="AV67" s="38"/>
-      <x:c r="BC67" s="36"/>
+      <x:c r="AY67" s="38"/>
+      <x:c r="BF67" s="36"/>
     </x:row>
     <x:row r="68">
       <x:c r="C68" s="28"/>
@@ -9783,13 +10004,16 @@
       <x:c r="N68" s="28"/>
       <x:c r="O68" s="28"/>
       <x:c r="AB68" s="30"/>
-      <x:c r="AC68" s="34"/>
-      <x:c r="AD68" s="34"/>
-      <x:c r="AM68" s="38"/>
+      <x:c r="AC68" s="30"/>
+      <x:c r="AD68" s="30"/>
+      <x:c r="AE68" s="30"/>
+      <x:c r="AF68" s="34"/>
+      <x:c r="AG68" s="34"/>
       <x:c r="AP68" s="38"/>
       <x:c r="AS68" s="38"/>
       <x:c r="AV68" s="38"/>
-      <x:c r="BC68" s="36"/>
+      <x:c r="AY68" s="38"/>
+      <x:c r="BF68" s="36"/>
     </x:row>
     <x:row r="69">
       <x:c r="C69" s="28"/>
@@ -9801,13 +10025,16 @@
       <x:c r="N69" s="28"/>
       <x:c r="O69" s="28"/>
       <x:c r="AB69" s="30"/>
-      <x:c r="AC69" s="34"/>
-      <x:c r="AD69" s="34"/>
-      <x:c r="AM69" s="38"/>
+      <x:c r="AC69" s="30"/>
+      <x:c r="AD69" s="30"/>
+      <x:c r="AE69" s="30"/>
+      <x:c r="AF69" s="34"/>
+      <x:c r="AG69" s="34"/>
       <x:c r="AP69" s="38"/>
       <x:c r="AS69" s="38"/>
       <x:c r="AV69" s="38"/>
-      <x:c r="BC69" s="36"/>
+      <x:c r="AY69" s="38"/>
+      <x:c r="BF69" s="36"/>
     </x:row>
     <x:row r="70">
       <x:c r="C70" s="28"/>
@@ -9819,13 +10046,16 @@
       <x:c r="N70" s="28"/>
       <x:c r="O70" s="28"/>
       <x:c r="AB70" s="30"/>
-      <x:c r="AC70" s="34"/>
-      <x:c r="AD70" s="34"/>
-      <x:c r="AM70" s="38"/>
+      <x:c r="AC70" s="30"/>
+      <x:c r="AD70" s="30"/>
+      <x:c r="AE70" s="30"/>
+      <x:c r="AF70" s="34"/>
+      <x:c r="AG70" s="34"/>
       <x:c r="AP70" s="38"/>
       <x:c r="AS70" s="38"/>
       <x:c r="AV70" s="38"/>
-      <x:c r="BC70" s="36"/>
+      <x:c r="AY70" s="38"/>
+      <x:c r="BF70" s="36"/>
     </x:row>
     <x:row r="71">
       <x:c r="C71" s="28"/>
@@ -9837,13 +10067,16 @@
       <x:c r="N71" s="28"/>
       <x:c r="O71" s="28"/>
       <x:c r="AB71" s="30"/>
-      <x:c r="AC71" s="34"/>
-      <x:c r="AD71" s="34"/>
-      <x:c r="AM71" s="38"/>
+      <x:c r="AC71" s="30"/>
+      <x:c r="AD71" s="30"/>
+      <x:c r="AE71" s="30"/>
+      <x:c r="AF71" s="34"/>
+      <x:c r="AG71" s="34"/>
       <x:c r="AP71" s="38"/>
       <x:c r="AS71" s="38"/>
       <x:c r="AV71" s="38"/>
-      <x:c r="BC71" s="36"/>
+      <x:c r="AY71" s="38"/>
+      <x:c r="BF71" s="36"/>
     </x:row>
     <x:row r="72">
       <x:c r="C72" s="28"/>
@@ -9855,13 +10088,16 @@
       <x:c r="N72" s="28"/>
       <x:c r="O72" s="28"/>
       <x:c r="AB72" s="30"/>
-      <x:c r="AC72" s="34"/>
-      <x:c r="AD72" s="34"/>
-      <x:c r="AM72" s="38"/>
+      <x:c r="AC72" s="30"/>
+      <x:c r="AD72" s="30"/>
+      <x:c r="AE72" s="30"/>
+      <x:c r="AF72" s="34"/>
+      <x:c r="AG72" s="34"/>
       <x:c r="AP72" s="38"/>
       <x:c r="AS72" s="38"/>
       <x:c r="AV72" s="38"/>
-      <x:c r="BC72" s="36"/>
+      <x:c r="AY72" s="38"/>
+      <x:c r="BF72" s="36"/>
     </x:row>
     <x:row r="73">
       <x:c r="C73" s="28"/>
@@ -9873,13 +10109,16 @@
       <x:c r="N73" s="28"/>
       <x:c r="O73" s="28"/>
       <x:c r="AB73" s="30"/>
-      <x:c r="AC73" s="34"/>
-      <x:c r="AD73" s="34"/>
-      <x:c r="AM73" s="38"/>
+      <x:c r="AC73" s="30"/>
+      <x:c r="AD73" s="30"/>
+      <x:c r="AE73" s="30"/>
+      <x:c r="AF73" s="34"/>
+      <x:c r="AG73" s="34"/>
       <x:c r="AP73" s="38"/>
       <x:c r="AS73" s="38"/>
       <x:c r="AV73" s="38"/>
-      <x:c r="BC73" s="36"/>
+      <x:c r="AY73" s="38"/>
+      <x:c r="BF73" s="36"/>
     </x:row>
     <x:row r="74">
       <x:c r="C74" s="28"/>
@@ -9891,13 +10130,16 @@
       <x:c r="N74" s="28"/>
       <x:c r="O74" s="28"/>
       <x:c r="AB74" s="30"/>
-      <x:c r="AC74" s="34"/>
-      <x:c r="AD74" s="34"/>
-      <x:c r="AM74" s="38"/>
+      <x:c r="AC74" s="30"/>
+      <x:c r="AD74" s="30"/>
+      <x:c r="AE74" s="30"/>
+      <x:c r="AF74" s="34"/>
+      <x:c r="AG74" s="34"/>
       <x:c r="AP74" s="38"/>
       <x:c r="AS74" s="38"/>
       <x:c r="AV74" s="38"/>
-      <x:c r="BC74" s="36"/>
+      <x:c r="AY74" s="38"/>
+      <x:c r="BF74" s="36"/>
     </x:row>
     <x:row r="75">
       <x:c r="C75" s="28"/>
@@ -9909,13 +10151,16 @@
       <x:c r="N75" s="28"/>
       <x:c r="O75" s="28"/>
       <x:c r="AB75" s="30"/>
-      <x:c r="AC75" s="34"/>
-      <x:c r="AD75" s="34"/>
-      <x:c r="AM75" s="38"/>
+      <x:c r="AC75" s="30"/>
+      <x:c r="AD75" s="30"/>
+      <x:c r="AE75" s="30"/>
+      <x:c r="AF75" s="34"/>
+      <x:c r="AG75" s="34"/>
       <x:c r="AP75" s="38"/>
       <x:c r="AS75" s="38"/>
       <x:c r="AV75" s="38"/>
-      <x:c r="BC75" s="36"/>
+      <x:c r="AY75" s="38"/>
+      <x:c r="BF75" s="36"/>
     </x:row>
     <x:row r="76">
       <x:c r="C76" s="28"/>
@@ -9927,13 +10172,16 @@
       <x:c r="N76" s="28"/>
       <x:c r="O76" s="28"/>
       <x:c r="AB76" s="30"/>
-      <x:c r="AC76" s="34"/>
-      <x:c r="AD76" s="34"/>
-      <x:c r="AM76" s="38"/>
+      <x:c r="AC76" s="30"/>
+      <x:c r="AD76" s="30"/>
+      <x:c r="AE76" s="30"/>
+      <x:c r="AF76" s="34"/>
+      <x:c r="AG76" s="34"/>
       <x:c r="AP76" s="38"/>
       <x:c r="AS76" s="38"/>
       <x:c r="AV76" s="38"/>
-      <x:c r="BC76" s="36"/>
+      <x:c r="AY76" s="38"/>
+      <x:c r="BF76" s="36"/>
     </x:row>
     <x:row r="77">
       <x:c r="C77" s="28"/>
@@ -9945,13 +10193,16 @@
       <x:c r="N77" s="28"/>
       <x:c r="O77" s="28"/>
       <x:c r="AB77" s="30"/>
-      <x:c r="AC77" s="34"/>
-      <x:c r="AD77" s="34"/>
-      <x:c r="AM77" s="38"/>
+      <x:c r="AC77" s="30"/>
+      <x:c r="AD77" s="30"/>
+      <x:c r="AE77" s="30"/>
+      <x:c r="AF77" s="34"/>
+      <x:c r="AG77" s="34"/>
       <x:c r="AP77" s="38"/>
       <x:c r="AS77" s="38"/>
       <x:c r="AV77" s="38"/>
-      <x:c r="BC77" s="36"/>
+      <x:c r="AY77" s="38"/>
+      <x:c r="BF77" s="36"/>
     </x:row>
     <x:row r="78">
       <x:c r="C78" s="28"/>
@@ -9963,13 +10214,16 @@
       <x:c r="N78" s="28"/>
       <x:c r="O78" s="28"/>
       <x:c r="AB78" s="30"/>
-      <x:c r="AC78" s="34"/>
-      <x:c r="AD78" s="34"/>
-      <x:c r="AM78" s="38"/>
+      <x:c r="AC78" s="30"/>
+      <x:c r="AD78" s="30"/>
+      <x:c r="AE78" s="30"/>
+      <x:c r="AF78" s="34"/>
+      <x:c r="AG78" s="34"/>
       <x:c r="AP78" s="38"/>
       <x:c r="AS78" s="38"/>
       <x:c r="AV78" s="38"/>
-      <x:c r="BC78" s="36"/>
+      <x:c r="AY78" s="38"/>
+      <x:c r="BF78" s="36"/>
     </x:row>
     <x:row r="79">
       <x:c r="C79" s="28"/>
@@ -9981,13 +10235,16 @@
       <x:c r="N79" s="28"/>
       <x:c r="O79" s="28"/>
       <x:c r="AB79" s="30"/>
-      <x:c r="AC79" s="34"/>
-      <x:c r="AD79" s="34"/>
-      <x:c r="AM79" s="38"/>
+      <x:c r="AC79" s="30"/>
+      <x:c r="AD79" s="30"/>
+      <x:c r="AE79" s="30"/>
+      <x:c r="AF79" s="34"/>
+      <x:c r="AG79" s="34"/>
       <x:c r="AP79" s="38"/>
       <x:c r="AS79" s="38"/>
       <x:c r="AV79" s="38"/>
-      <x:c r="BC79" s="36"/>
+      <x:c r="AY79" s="38"/>
+      <x:c r="BF79" s="36"/>
     </x:row>
     <x:row r="80">
       <x:c r="C80" s="28"/>
@@ -9999,13 +10256,16 @@
       <x:c r="N80" s="28"/>
       <x:c r="O80" s="28"/>
       <x:c r="AB80" s="30"/>
-      <x:c r="AC80" s="34"/>
-      <x:c r="AD80" s="34"/>
-      <x:c r="AM80" s="38"/>
+      <x:c r="AC80" s="30"/>
+      <x:c r="AD80" s="30"/>
+      <x:c r="AE80" s="30"/>
+      <x:c r="AF80" s="34"/>
+      <x:c r="AG80" s="34"/>
       <x:c r="AP80" s="38"/>
       <x:c r="AS80" s="38"/>
       <x:c r="AV80" s="38"/>
-      <x:c r="BC80" s="36"/>
+      <x:c r="AY80" s="38"/>
+      <x:c r="BF80" s="36"/>
     </x:row>
     <x:row r="81">
       <x:c r="C81" s="28"/>
@@ -10017,13 +10277,16 @@
       <x:c r="N81" s="28"/>
       <x:c r="O81" s="28"/>
       <x:c r="AB81" s="30"/>
-      <x:c r="AC81" s="34"/>
-      <x:c r="AD81" s="34"/>
-      <x:c r="AM81" s="38"/>
+      <x:c r="AC81" s="30"/>
+      <x:c r="AD81" s="30"/>
+      <x:c r="AE81" s="30"/>
+      <x:c r="AF81" s="34"/>
+      <x:c r="AG81" s="34"/>
       <x:c r="AP81" s="38"/>
       <x:c r="AS81" s="38"/>
       <x:c r="AV81" s="38"/>
-      <x:c r="BC81" s="36"/>
+      <x:c r="AY81" s="38"/>
+      <x:c r="BF81" s="36"/>
     </x:row>
     <x:row r="82">
       <x:c r="C82" s="28"/>
@@ -10035,13 +10298,16 @@
       <x:c r="N82" s="28"/>
       <x:c r="O82" s="28"/>
       <x:c r="AB82" s="30"/>
-      <x:c r="AC82" s="34"/>
-      <x:c r="AD82" s="34"/>
-      <x:c r="AM82" s="38"/>
+      <x:c r="AC82" s="30"/>
+      <x:c r="AD82" s="30"/>
+      <x:c r="AE82" s="30"/>
+      <x:c r="AF82" s="34"/>
+      <x:c r="AG82" s="34"/>
       <x:c r="AP82" s="38"/>
       <x:c r="AS82" s="38"/>
       <x:c r="AV82" s="38"/>
-      <x:c r="BC82" s="36"/>
+      <x:c r="AY82" s="38"/>
+      <x:c r="BF82" s="36"/>
     </x:row>
     <x:row r="83">
       <x:c r="C83" s="28"/>
@@ -10053,13 +10319,16 @@
       <x:c r="N83" s="28"/>
       <x:c r="O83" s="28"/>
       <x:c r="AB83" s="30"/>
-      <x:c r="AC83" s="34"/>
-      <x:c r="AD83" s="34"/>
-      <x:c r="AM83" s="38"/>
+      <x:c r="AC83" s="30"/>
+      <x:c r="AD83" s="30"/>
+      <x:c r="AE83" s="30"/>
+      <x:c r="AF83" s="34"/>
+      <x:c r="AG83" s="34"/>
       <x:c r="AP83" s="38"/>
       <x:c r="AS83" s="38"/>
       <x:c r="AV83" s="38"/>
-      <x:c r="BC83" s="36"/>
+      <x:c r="AY83" s="38"/>
+      <x:c r="BF83" s="36"/>
     </x:row>
     <x:row r="84">
       <x:c r="C84" s="28"/>
@@ -10071,13 +10340,16 @@
       <x:c r="N84" s="28"/>
       <x:c r="O84" s="28"/>
       <x:c r="AB84" s="30"/>
-      <x:c r="AC84" s="34"/>
-      <x:c r="AD84" s="34"/>
-      <x:c r="AM84" s="38"/>
+      <x:c r="AC84" s="30"/>
+      <x:c r="AD84" s="30"/>
+      <x:c r="AE84" s="30"/>
+      <x:c r="AF84" s="34"/>
+      <x:c r="AG84" s="34"/>
       <x:c r="AP84" s="38"/>
       <x:c r="AS84" s="38"/>
       <x:c r="AV84" s="38"/>
-      <x:c r="BC84" s="36"/>
+      <x:c r="AY84" s="38"/>
+      <x:c r="BF84" s="36"/>
     </x:row>
     <x:row r="85">
       <x:c r="C85" s="28"/>
@@ -10089,13 +10361,16 @@
       <x:c r="N85" s="28"/>
       <x:c r="O85" s="28"/>
       <x:c r="AB85" s="30"/>
-      <x:c r="AC85" s="34"/>
-      <x:c r="AD85" s="34"/>
-      <x:c r="AM85" s="38"/>
+      <x:c r="AC85" s="30"/>
+      <x:c r="AD85" s="30"/>
+      <x:c r="AE85" s="30"/>
+      <x:c r="AF85" s="34"/>
+      <x:c r="AG85" s="34"/>
       <x:c r="AP85" s="38"/>
       <x:c r="AS85" s="38"/>
       <x:c r="AV85" s="38"/>
-      <x:c r="BC85" s="36"/>
+      <x:c r="AY85" s="38"/>
+      <x:c r="BF85" s="36"/>
     </x:row>
     <x:row r="86">
       <x:c r="C86" s="28"/>
@@ -10107,13 +10382,16 @@
       <x:c r="N86" s="28"/>
       <x:c r="O86" s="28"/>
       <x:c r="AB86" s="30"/>
-      <x:c r="AC86" s="34"/>
-      <x:c r="AD86" s="34"/>
-      <x:c r="AM86" s="38"/>
+      <x:c r="AC86" s="30"/>
+      <x:c r="AD86" s="30"/>
+      <x:c r="AE86" s="30"/>
+      <x:c r="AF86" s="34"/>
+      <x:c r="AG86" s="34"/>
       <x:c r="AP86" s="38"/>
       <x:c r="AS86" s="38"/>
       <x:c r="AV86" s="38"/>
-      <x:c r="BC86" s="36"/>
+      <x:c r="AY86" s="38"/>
+      <x:c r="BF86" s="36"/>
     </x:row>
     <x:row r="87">
       <x:c r="C87" s="28"/>
@@ -10125,13 +10403,16 @@
       <x:c r="N87" s="28"/>
       <x:c r="O87" s="28"/>
       <x:c r="AB87" s="30"/>
-      <x:c r="AC87" s="34"/>
-      <x:c r="AD87" s="34"/>
-      <x:c r="AM87" s="38"/>
+      <x:c r="AC87" s="30"/>
+      <x:c r="AD87" s="30"/>
+      <x:c r="AE87" s="30"/>
+      <x:c r="AF87" s="34"/>
+      <x:c r="AG87" s="34"/>
       <x:c r="AP87" s="38"/>
       <x:c r="AS87" s="38"/>
       <x:c r="AV87" s="38"/>
-      <x:c r="BC87" s="36"/>
+      <x:c r="AY87" s="38"/>
+      <x:c r="BF87" s="36"/>
     </x:row>
     <x:row r="88">
       <x:c r="C88" s="28"/>
@@ -10143,13 +10424,16 @@
       <x:c r="N88" s="28"/>
       <x:c r="O88" s="28"/>
       <x:c r="AB88" s="30"/>
-      <x:c r="AC88" s="34"/>
-      <x:c r="AD88" s="34"/>
-      <x:c r="AM88" s="38"/>
+      <x:c r="AC88" s="30"/>
+      <x:c r="AD88" s="30"/>
+      <x:c r="AE88" s="30"/>
+      <x:c r="AF88" s="34"/>
+      <x:c r="AG88" s="34"/>
       <x:c r="AP88" s="38"/>
       <x:c r="AS88" s="38"/>
       <x:c r="AV88" s="38"/>
-      <x:c r="BC88" s="36"/>
+      <x:c r="AY88" s="38"/>
+      <x:c r="BF88" s="36"/>
     </x:row>
     <x:row r="89">
       <x:c r="C89" s="28"/>
@@ -10161,13 +10445,16 @@
       <x:c r="N89" s="28"/>
       <x:c r="O89" s="28"/>
       <x:c r="AB89" s="30"/>
-      <x:c r="AC89" s="34"/>
-      <x:c r="AD89" s="34"/>
-      <x:c r="AM89" s="38"/>
+      <x:c r="AC89" s="30"/>
+      <x:c r="AD89" s="30"/>
+      <x:c r="AE89" s="30"/>
+      <x:c r="AF89" s="34"/>
+      <x:c r="AG89" s="34"/>
       <x:c r="AP89" s="38"/>
       <x:c r="AS89" s="38"/>
       <x:c r="AV89" s="38"/>
-      <x:c r="BC89" s="36"/>
+      <x:c r="AY89" s="38"/>
+      <x:c r="BF89" s="36"/>
     </x:row>
     <x:row r="90">
       <x:c r="C90" s="28"/>
@@ -10179,13 +10466,16 @@
       <x:c r="N90" s="28"/>
       <x:c r="O90" s="28"/>
       <x:c r="AB90" s="30"/>
-      <x:c r="AC90" s="34"/>
-      <x:c r="AD90" s="34"/>
-      <x:c r="AM90" s="38"/>
+      <x:c r="AC90" s="30"/>
+      <x:c r="AD90" s="30"/>
+      <x:c r="AE90" s="30"/>
+      <x:c r="AF90" s="34"/>
+      <x:c r="AG90" s="34"/>
       <x:c r="AP90" s="38"/>
       <x:c r="AS90" s="38"/>
       <x:c r="AV90" s="38"/>
-      <x:c r="BC90" s="36"/>
+      <x:c r="AY90" s="38"/>
+      <x:c r="BF90" s="36"/>
     </x:row>
     <x:row r="91">
       <x:c r="C91" s="28"/>
@@ -10197,13 +10487,16 @@
       <x:c r="N91" s="28"/>
       <x:c r="O91" s="28"/>
       <x:c r="AB91" s="30"/>
-      <x:c r="AC91" s="34"/>
-      <x:c r="AD91" s="34"/>
-      <x:c r="AM91" s="38"/>
+      <x:c r="AC91" s="30"/>
+      <x:c r="AD91" s="30"/>
+      <x:c r="AE91" s="30"/>
+      <x:c r="AF91" s="34"/>
+      <x:c r="AG91" s="34"/>
       <x:c r="AP91" s="38"/>
       <x:c r="AS91" s="38"/>
       <x:c r="AV91" s="38"/>
-      <x:c r="BC91" s="36"/>
+      <x:c r="AY91" s="38"/>
+      <x:c r="BF91" s="36"/>
     </x:row>
     <x:row r="92">
       <x:c r="C92" s="28"/>
@@ -10215,13 +10508,16 @@
       <x:c r="N92" s="28"/>
       <x:c r="O92" s="28"/>
       <x:c r="AB92" s="30"/>
-      <x:c r="AC92" s="34"/>
-      <x:c r="AD92" s="34"/>
-      <x:c r="AM92" s="38"/>
+      <x:c r="AC92" s="30"/>
+      <x:c r="AD92" s="30"/>
+      <x:c r="AE92" s="30"/>
+      <x:c r="AF92" s="34"/>
+      <x:c r="AG92" s="34"/>
       <x:c r="AP92" s="38"/>
       <x:c r="AS92" s="38"/>
       <x:c r="AV92" s="38"/>
-      <x:c r="BC92" s="36"/>
+      <x:c r="AY92" s="38"/>
+      <x:c r="BF92" s="36"/>
     </x:row>
     <x:row r="93">
       <x:c r="C93" s="28"/>
@@ -10233,13 +10529,16 @@
       <x:c r="N93" s="28"/>
       <x:c r="O93" s="28"/>
       <x:c r="AB93" s="30"/>
-      <x:c r="AC93" s="34"/>
-      <x:c r="AD93" s="34"/>
-      <x:c r="AM93" s="38"/>
+      <x:c r="AC93" s="30"/>
+      <x:c r="AD93" s="30"/>
+      <x:c r="AE93" s="30"/>
+      <x:c r="AF93" s="34"/>
+      <x:c r="AG93" s="34"/>
       <x:c r="AP93" s="38"/>
       <x:c r="AS93" s="38"/>
       <x:c r="AV93" s="38"/>
-      <x:c r="BC93" s="36"/>
+      <x:c r="AY93" s="38"/>
+      <x:c r="BF93" s="36"/>
     </x:row>
     <x:row r="94">
       <x:c r="C94" s="28"/>
@@ -10251,13 +10550,16 @@
       <x:c r="N94" s="28"/>
       <x:c r="O94" s="28"/>
       <x:c r="AB94" s="30"/>
-      <x:c r="AC94" s="34"/>
-      <x:c r="AD94" s="34"/>
-      <x:c r="AM94" s="38"/>
+      <x:c r="AC94" s="30"/>
+      <x:c r="AD94" s="30"/>
+      <x:c r="AE94" s="30"/>
+      <x:c r="AF94" s="34"/>
+      <x:c r="AG94" s="34"/>
       <x:c r="AP94" s="38"/>
       <x:c r="AS94" s="38"/>
       <x:c r="AV94" s="38"/>
-      <x:c r="BC94" s="36"/>
+      <x:c r="AY94" s="38"/>
+      <x:c r="BF94" s="36"/>
     </x:row>
     <x:row r="95">
       <x:c r="C95" s="28"/>
@@ -10269,13 +10571,16 @@
       <x:c r="N95" s="28"/>
       <x:c r="O95" s="28"/>
       <x:c r="AB95" s="30"/>
-      <x:c r="AC95" s="34"/>
-      <x:c r="AD95" s="34"/>
-      <x:c r="AM95" s="38"/>
+      <x:c r="AC95" s="30"/>
+      <x:c r="AD95" s="30"/>
+      <x:c r="AE95" s="30"/>
+      <x:c r="AF95" s="34"/>
+      <x:c r="AG95" s="34"/>
       <x:c r="AP95" s="38"/>
       <x:c r="AS95" s="38"/>
       <x:c r="AV95" s="38"/>
-      <x:c r="BC95" s="36"/>
+      <x:c r="AY95" s="38"/>
+      <x:c r="BF95" s="36"/>
     </x:row>
     <x:row r="96">
       <x:c r="C96" s="28"/>
@@ -10287,13 +10592,16 @@
       <x:c r="N96" s="28"/>
       <x:c r="O96" s="28"/>
       <x:c r="AB96" s="30"/>
-      <x:c r="AC96" s="34"/>
-      <x:c r="AD96" s="34"/>
-      <x:c r="AM96" s="38"/>
+      <x:c r="AC96" s="30"/>
+      <x:c r="AD96" s="30"/>
+      <x:c r="AE96" s="30"/>
+      <x:c r="AF96" s="34"/>
+      <x:c r="AG96" s="34"/>
       <x:c r="AP96" s="38"/>
       <x:c r="AS96" s="38"/>
       <x:c r="AV96" s="38"/>
-      <x:c r="BC96" s="36"/>
+      <x:c r="AY96" s="38"/>
+      <x:c r="BF96" s="36"/>
     </x:row>
     <x:row r="97">
       <x:c r="C97" s="28"/>
@@ -10305,13 +10613,16 @@
       <x:c r="N97" s="28"/>
       <x:c r="O97" s="28"/>
       <x:c r="AB97" s="30"/>
-      <x:c r="AC97" s="34"/>
-      <x:c r="AD97" s="34"/>
-      <x:c r="AM97" s="38"/>
+      <x:c r="AC97" s="30"/>
+      <x:c r="AD97" s="30"/>
+      <x:c r="AE97" s="30"/>
+      <x:c r="AF97" s="34"/>
+      <x:c r="AG97" s="34"/>
       <x:c r="AP97" s="38"/>
       <x:c r="AS97" s="38"/>
       <x:c r="AV97" s="38"/>
-      <x:c r="BC97" s="36"/>
+      <x:c r="AY97" s="38"/>
+      <x:c r="BF97" s="36"/>
     </x:row>
     <x:row r="98">
       <x:c r="C98" s="28"/>
@@ -10323,13 +10634,16 @@
       <x:c r="N98" s="28"/>
       <x:c r="O98" s="28"/>
       <x:c r="AB98" s="30"/>
-      <x:c r="AC98" s="34"/>
-      <x:c r="AD98" s="34"/>
-      <x:c r="AM98" s="38"/>
+      <x:c r="AC98" s="30"/>
+      <x:c r="AD98" s="30"/>
+      <x:c r="AE98" s="30"/>
+      <x:c r="AF98" s="34"/>
+      <x:c r="AG98" s="34"/>
       <x:c r="AP98" s="38"/>
       <x:c r="AS98" s="38"/>
       <x:c r="AV98" s="38"/>
-      <x:c r="BC98" s="36"/>
+      <x:c r="AY98" s="38"/>
+      <x:c r="BF98" s="36"/>
     </x:row>
     <x:row r="99">
       <x:c r="C99" s="28"/>
@@ -10341,13 +10655,16 @@
       <x:c r="N99" s="28"/>
       <x:c r="O99" s="28"/>
       <x:c r="AB99" s="30"/>
-      <x:c r="AC99" s="34"/>
-      <x:c r="AD99" s="34"/>
-      <x:c r="AM99" s="38"/>
+      <x:c r="AC99" s="30"/>
+      <x:c r="AD99" s="30"/>
+      <x:c r="AE99" s="30"/>
+      <x:c r="AF99" s="34"/>
+      <x:c r="AG99" s="34"/>
       <x:c r="AP99" s="38"/>
       <x:c r="AS99" s="38"/>
       <x:c r="AV99" s="38"/>
-      <x:c r="BC99" s="36"/>
+      <x:c r="AY99" s="38"/>
+      <x:c r="BF99" s="36"/>
     </x:row>
     <x:row r="100">
       <x:c r="C100" s="28"/>
@@ -10359,13 +10676,16 @@
       <x:c r="N100" s="28"/>
       <x:c r="O100" s="28"/>
       <x:c r="AB100" s="30"/>
-      <x:c r="AC100" s="34"/>
-      <x:c r="AD100" s="34"/>
-      <x:c r="AM100" s="38"/>
+      <x:c r="AC100" s="30"/>
+      <x:c r="AD100" s="30"/>
+      <x:c r="AE100" s="30"/>
+      <x:c r="AF100" s="34"/>
+      <x:c r="AG100" s="34"/>
       <x:c r="AP100" s="38"/>
       <x:c r="AS100" s="38"/>
       <x:c r="AV100" s="38"/>
-      <x:c r="BC100" s="36"/>
+      <x:c r="AY100" s="38"/>
+      <x:c r="BF100" s="36"/>
     </x:row>
     <x:row r="101">
       <x:c r="C101" s="28"/>
@@ -10377,13 +10697,16 @@
       <x:c r="N101" s="28"/>
       <x:c r="O101" s="28"/>
       <x:c r="AB101" s="30"/>
-      <x:c r="AC101" s="34"/>
-      <x:c r="AD101" s="34"/>
-      <x:c r="AM101" s="38"/>
+      <x:c r="AC101" s="30"/>
+      <x:c r="AD101" s="30"/>
+      <x:c r="AE101" s="30"/>
+      <x:c r="AF101" s="34"/>
+      <x:c r="AG101" s="34"/>
       <x:c r="AP101" s="38"/>
       <x:c r="AS101" s="38"/>
       <x:c r="AV101" s="38"/>
-      <x:c r="BC101" s="36"/>
+      <x:c r="AY101" s="38"/>
+      <x:c r="BF101" s="36"/>
     </x:row>
     <x:row r="102">
       <x:c r="C102" s="28"/>
@@ -10395,13 +10718,16 @@
       <x:c r="N102" s="28"/>
       <x:c r="O102" s="28"/>
       <x:c r="AB102" s="30"/>
-      <x:c r="AC102" s="34"/>
-      <x:c r="AD102" s="34"/>
-      <x:c r="AM102" s="38"/>
+      <x:c r="AC102" s="30"/>
+      <x:c r="AD102" s="30"/>
+      <x:c r="AE102" s="30"/>
+      <x:c r="AF102" s="34"/>
+      <x:c r="AG102" s="34"/>
       <x:c r="AP102" s="38"/>
       <x:c r="AS102" s="38"/>
       <x:c r="AV102" s="38"/>
-      <x:c r="BC102" s="36"/>
+      <x:c r="AY102" s="38"/>
+      <x:c r="BF102" s="36"/>
     </x:row>
     <x:row r="103">
       <x:c r="C103" s="28"/>
@@ -10413,18 +10739,21 @@
       <x:c r="N103" s="28"/>
       <x:c r="O103" s="28"/>
       <x:c r="AB103" s="30"/>
-      <x:c r="AC103" s="34"/>
-      <x:c r="AD103" s="34"/>
-      <x:c r="AM103" s="38"/>
+      <x:c r="AC103" s="30"/>
+      <x:c r="AD103" s="30"/>
+      <x:c r="AE103" s="30"/>
+      <x:c r="AF103" s="34"/>
+      <x:c r="AG103" s="34"/>
       <x:c r="AP103" s="38"/>
       <x:c r="AS103" s="38"/>
       <x:c r="AV103" s="38"/>
-      <x:c r="BC103" s="36"/>
+      <x:c r="AY103" s="38"/>
+      <x:c r="BF103" s="36"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:BF1"/>
-    <x:mergeCell ref="A2:BF2"/>
+    <x:mergeCell ref="A1:BI1"/>
+    <x:mergeCell ref="A2:BI2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:A103">
     <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="严格合格"/>
@@ -10438,7 +10767,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73ad8797720549ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d8ddaa804124c35"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15233,7 +15562,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R853841a60df64bef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18e07fbc0a624bd0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16099,7 +16428,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree9d3cd8d2d94c9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc2224aa953646d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16944,7 +17273,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3438f1644da34536"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R209a69bfeebd4234"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: 发布多产品选品 Skill v1.2.1
</commit_message>
<xml_diff>
--- a/skills/cross-market-product-selection/assets/通用选品数据库模板.xlsx
+++ b/skills/cross-market-product-selection/assets/通用选品数据库模板.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务说明" sheetId="1" r:id="R970c4048668544a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目标产品" sheetId="2" r:id="R0a796489e12a4468"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="价格基准" sheetId="3" r:id="Rdf9e9a186d394aae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="亚马逊候选" sheetId="4" r:id="R86727b9705334f8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1688候选" sheetId="5" r:id="Raf98f3a3f0a24573"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="货源匹配" sheetId="6" r:id="Ra87d0c801a324add"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="严格结果" sheetId="7" r:id="R453561ab9ad242da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待核验" sheetId="8" r:id="Ree2cbd2e1cd442c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="9" r:id="R436cc4400f96422b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务说明" sheetId="1" r:id="Rad4226eb2f164503"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目标产品" sheetId="2" r:id="Re588a7ff5d304861"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="价格基准" sheetId="3" r:id="R08bc666aeb6943ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="亚马逊候选" sheetId="4" r:id="R0f5413ba13ec4e76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1688候选" sheetId="5" r:id="R9ffe5238489849e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="货源匹配" sheetId="6" r:id="R8410b951ea5a4ce5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="严格结果" sheetId="7" r:id="R086284ad853842d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待核验" sheetId="8" r:id="R3beaf92faf3a4e14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰记录" sheetId="9" r:id="R32989aaa568f4a1f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -523,9 +523,9 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SupplyCandidatesTable" displayName="SupplyCandidatesTable" ref="A3:AY4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A3:AY4"/>
-  <x:tableColumns count="51">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SupplyCandidatesTable" displayName="SupplyCandidatesTable" ref="A3:BB4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:BB4"/>
+  <x:tableColumns count="54">
     <x:tableColumn id="1" name="状态"/>
     <x:tableColumn id="2" name="模式"/>
     <x:tableColumn id="3" name="目标产品ID"/>
@@ -577,15 +577,18 @@
     <x:tableColumn id="49" name="置信度"/>
     <x:tableColumn id="50" name="冲突说明"/>
     <x:tableColumn id="51" name="决策日志引用"/>
+    <x:tableColumn id="52" name="搜索参考价"/>
+    <x:tableColumn id="53" name="报价口径"/>
+    <x:tableColumn id="54" name="补证据动作"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="SourceMatchesTable" displayName="SourceMatchesTable" ref="A3:BI4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A3:BI4"/>
-  <x:tableColumns count="61">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="SourceMatchesTable" displayName="SourceMatchesTable" ref="A3:BL4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:BL4"/>
+  <x:tableColumns count="64">
     <x:tableColumn id="1" name="状态"/>
     <x:tableColumn id="2" name="模式"/>
     <x:tableColumn id="3" name="目标产品ID"/>
@@ -647,6 +650,9 @@
     <x:tableColumn id="59" name="置信度"/>
     <x:tableColumn id="60" name="冲突说明"/>
     <x:tableColumn id="61" name="决策日志引用"/>
+    <x:tableColumn id="62" name="搜索参考价"/>
+    <x:tableColumn id="63" name="报价口径"/>
+    <x:tableColumn id="64" name="补证据动作"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -745,9 +751,9 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PendingAuditTable" displayName="PendingAuditTable" ref="A3:S4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A3:S4"/>
-  <x:tableColumns count="19">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PendingAuditTable" displayName="PendingAuditTable" ref="A3:AA4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:AA4"/>
+  <x:tableColumns count="27">
     <x:tableColumn id="1" name="状态"/>
     <x:tableColumn id="2" name="模式"/>
     <x:tableColumn id="3" name="目标产品ID"/>
@@ -767,6 +773,14 @@
     <x:tableColumn id="17" name="用户保留决定"/>
     <x:tableColumn id="18" name="决策日志引用"/>
     <x:tableColumn id="19" name="更新时间"/>
+    <x:tableColumn id="20" name="Amazon实际售价"/>
+    <x:tableColumn id="21" name="实际单价"/>
+    <x:tableColumn id="22" name="成本币种"/>
+    <x:tableColumn id="23" name="搜索参考价"/>
+    <x:tableColumn id="24" name="报价口径"/>
+    <x:tableColumn id="25" name="外观门槛"/>
+    <x:tableColumn id="26" name="价格/MOQ门槛"/>
+    <x:tableColumn id="27" name="供应商门槛"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1284,7 +1298,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R973be06183c74496"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bc4d7bab3934fa3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2480,7 +2494,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ad32d240e914e85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce6081175eaf4454"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3309,7 +3323,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b253179c58a461c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra45da8ede79c4edd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5539,7 +5553,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1813d6434fdc4cb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a7973fe106f4b08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5599,6 +5613,9 @@
     <x:col min="49" max="49" width="12" hidden="0" customWidth="1"/>
     <x:col min="50" max="50" width="30" hidden="0" customWidth="1"/>
     <x:col min="51" max="51" width="16" hidden="0" customWidth="1"/>
+    <x:col min="52" max="52" width="16" hidden="0" customWidth="1"/>
+    <x:col min="53" max="53" width="16" hidden="0" customWidth="1"/>
+    <x:col min="54" max="54" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -5655,10 +5672,13 @@
       <x:c r="AW1" s="4"/>
       <x:c r="AX1" s="4"/>
       <x:c r="AY1" s="4"/>
+      <x:c r="AZ1" s="4"/>
+      <x:c r="BA1" s="4"/>
+      <x:c r="BB1" s="4"/>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>按目标产品 ID 核验商品与工厂；已知单价越过目标成本带即淘汰，严格行必须绑定 SKU、采购档位、MOQ和阶梯价。</x:v>
+        <x:v>按目标产品 ID 核验商品与工厂；搜索参考价与确认 SKU 单价分开。未知主体写补查动作；严格行绑定 SKU、采购档位、MOQ和阶梯价。</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -5710,6 +5730,9 @@
       <x:c r="AW2" s="8"/>
       <x:c r="AX2" s="8"/>
       <x:c r="AY2" s="8"/>
+      <x:c r="AZ2" s="8"/>
+      <x:c r="BA2" s="8"/>
+      <x:c r="BB2" s="8"/>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="14" t="str">
@@ -5864,6 +5887,15 @@
       </x:c>
       <x:c r="AY3" s="14" t="str">
         <x:v>决策日志引用</x:v>
+      </x:c>
+      <x:c r="AZ3" s="14" t="str">
+        <x:v>搜索参考价</x:v>
+      </x:c>
+      <x:c r="BA3" s="14" t="str">
+        <x:v>报价口径</x:v>
+      </x:c>
+      <x:c r="BB3" s="14" t="str">
+        <x:v>补证据动作</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="100" customHeight="1">
@@ -5926,6 +5958,9 @@
       <x:c r="AW4" s="19"/>
       <x:c r="AX4" s="19"/>
       <x:c r="AY4" s="19"/>
+      <x:c r="AZ4" s="19"/>
+      <x:c r="BA4" s="19"/>
+      <x:c r="BB4" s="19"/>
     </x:row>
     <x:row r="5">
       <x:c r="C5" s="28"/>
@@ -8206,8 +8241,8 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:AY1"/>
-    <x:mergeCell ref="A2:AY2"/>
+    <x:mergeCell ref="A1:BB1"/>
+    <x:mergeCell ref="A2:BB2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:A103">
     <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="严格合格"/>
@@ -8221,7 +8256,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3de49f1eeeb14ff5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd17025c0959142cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8291,6 +8326,9 @@
     <x:col min="59" max="59" width="12" hidden="0" customWidth="1"/>
     <x:col min="60" max="60" width="30" hidden="0" customWidth="1"/>
     <x:col min="61" max="61" width="16" hidden="0" customWidth="1"/>
+    <x:col min="62" max="62" width="16" hidden="0" customWidth="1"/>
+    <x:col min="63" max="63" width="16" hidden="0" customWidth="1"/>
+    <x:col min="64" max="64" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -8357,6 +8395,9 @@
       <x:c r="BG1" s="4"/>
       <x:c r="BH1" s="4"/>
       <x:c r="BI1" s="4"/>
+      <x:c r="BJ1" s="4"/>
+      <x:c r="BK1" s="4"/>
+      <x:c r="BL1" s="4"/>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="8" t="str">
@@ -8422,6 +8463,9 @@
       <x:c r="BG2" s="8"/>
       <x:c r="BH2" s="8"/>
       <x:c r="BI2" s="8"/>
+      <x:c r="BJ2" s="8"/>
+      <x:c r="BK2" s="8"/>
+      <x:c r="BL2" s="8"/>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="14" t="str">
@@ -8606,6 +8650,15 @@
       </x:c>
       <x:c r="BI3" s="14" t="str">
         <x:v>决策日志引用</x:v>
+      </x:c>
+      <x:c r="BJ3" s="14" t="str">
+        <x:v>搜索参考价</x:v>
+      </x:c>
+      <x:c r="BK3" s="14" t="str">
+        <x:v>报价口径</x:v>
+      </x:c>
+      <x:c r="BL3" s="14" t="str">
+        <x:v>补证据动作</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="100" customHeight="1">
@@ -8670,6 +8723,9 @@
       <x:c r="BG4" s="19"/>
       <x:c r="BH4" s="19"/>
       <x:c r="BI4" s="19"/>
+      <x:c r="BJ4" s="19"/>
+      <x:c r="BK4" s="19"/>
+      <x:c r="BL4" s="19"/>
     </x:row>
     <x:row r="5">
       <x:c r="C5" s="28"/>
@@ -10752,8 +10808,8 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:BI1"/>
-    <x:mergeCell ref="A2:BI2"/>
+    <x:mergeCell ref="A1:BL1"/>
+    <x:mergeCell ref="A2:BL2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:A103">
     <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="严格合格"/>
@@ -10767,7 +10823,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d8ddaa804124c35"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a1ad6819b1d4d8e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15562,7 +15618,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18e07fbc0a624bd0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4537624d1cbe4faf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15590,6 +15646,14 @@
     <x:col min="17" max="17" width="16" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="16" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="20" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="16" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="16" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="16" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="16" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="16" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="16" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="16" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -15614,10 +15678,18 @@
       <x:c r="Q1" s="4"/>
       <x:c r="R1" s="4"/>
       <x:c r="S1" s="4"/>
+      <x:c r="T1" s="4"/>
+      <x:c r="U1" s="4"/>
+      <x:c r="V1" s="4"/>
+      <x:c r="W1" s="4"/>
+      <x:c r="X1" s="4"/>
+      <x:c r="Y1" s="4"/>
+      <x:c r="Z1" s="4"/>
+      <x:c r="AA1" s="4"/>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>没有明确失败但缺少可靠硬门槛或评分原始证据的记录放在这里；写清缺口、现有证据与补证据动作。</x:v>
+        <x:v>保留缺证但未明确失败的商品；搜索参考价不得当实际单价，已知价格与门槛不得因转入本表丢失；写清补证据动作。</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -15637,6 +15709,14 @@
       <x:c r="Q2" s="8"/>
       <x:c r="R2" s="8"/>
       <x:c r="S2" s="8"/>
+      <x:c r="T2" s="8"/>
+      <x:c r="U2" s="8"/>
+      <x:c r="V2" s="8"/>
+      <x:c r="W2" s="8"/>
+      <x:c r="X2" s="8"/>
+      <x:c r="Y2" s="8"/>
+      <x:c r="Z2" s="8"/>
+      <x:c r="AA2" s="8"/>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="14" t="str">
@@ -15695,6 +15775,30 @@
       </x:c>
       <x:c r="S3" s="14" t="str">
         <x:v>更新时间</x:v>
+      </x:c>
+      <x:c r="T3" s="14" t="str">
+        <x:v>Amazon实际售价</x:v>
+      </x:c>
+      <x:c r="U3" s="14" t="str">
+        <x:v>实际单价</x:v>
+      </x:c>
+      <x:c r="V3" s="14" t="str">
+        <x:v>成本币种</x:v>
+      </x:c>
+      <x:c r="W3" s="14" t="str">
+        <x:v>搜索参考价</x:v>
+      </x:c>
+      <x:c r="X3" s="14" t="str">
+        <x:v>报价口径</x:v>
+      </x:c>
+      <x:c r="Y3" s="14" t="str">
+        <x:v>外观门槛</x:v>
+      </x:c>
+      <x:c r="Z3" s="14" t="str">
+        <x:v>价格/MOQ门槛</x:v>
+      </x:c>
+      <x:c r="AA3" s="14" t="str">
+        <x:v>供应商门槛</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="100" customHeight="1">
@@ -15717,6 +15821,14 @@
       <x:c r="Q4" s="19"/>
       <x:c r="R4" s="19"/>
       <x:c r="S4" s="35"/>
+      <x:c r="T4" s="29"/>
+      <x:c r="U4" s="29"/>
+      <x:c r="V4" s="29"/>
+      <x:c r="W4" s="19"/>
+      <x:c r="X4" s="19"/>
+      <x:c r="Y4" s="19"/>
+      <x:c r="Z4" s="29"/>
+      <x:c r="AA4" s="19"/>
     </x:row>
     <x:row r="5">
       <x:c r="C5" s="28"/>
@@ -15724,6 +15836,10 @@
       <x:c r="G5" s="28"/>
       <x:c r="H5" s="28"/>
       <x:c r="S5" s="36"/>
+      <x:c r="T5" s="30"/>
+      <x:c r="U5" s="30"/>
+      <x:c r="V5" s="30"/>
+      <x:c r="Z5" s="30"/>
     </x:row>
     <x:row r="6">
       <x:c r="C6" s="28"/>
@@ -15731,6 +15847,10 @@
       <x:c r="G6" s="28"/>
       <x:c r="H6" s="28"/>
       <x:c r="S6" s="36"/>
+      <x:c r="T6" s="30"/>
+      <x:c r="U6" s="30"/>
+      <x:c r="V6" s="30"/>
+      <x:c r="Z6" s="30"/>
     </x:row>
     <x:row r="7">
       <x:c r="C7" s="28"/>
@@ -15738,6 +15858,10 @@
       <x:c r="G7" s="28"/>
       <x:c r="H7" s="28"/>
       <x:c r="S7" s="36"/>
+      <x:c r="T7" s="30"/>
+      <x:c r="U7" s="30"/>
+      <x:c r="V7" s="30"/>
+      <x:c r="Z7" s="30"/>
     </x:row>
     <x:row r="8">
       <x:c r="C8" s="28"/>
@@ -15745,6 +15869,10 @@
       <x:c r="G8" s="28"/>
       <x:c r="H8" s="28"/>
       <x:c r="S8" s="36"/>
+      <x:c r="T8" s="30"/>
+      <x:c r="U8" s="30"/>
+      <x:c r="V8" s="30"/>
+      <x:c r="Z8" s="30"/>
     </x:row>
     <x:row r="9">
       <x:c r="C9" s="28"/>
@@ -15752,6 +15880,10 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="S9" s="36"/>
+      <x:c r="T9" s="30"/>
+      <x:c r="U9" s="30"/>
+      <x:c r="V9" s="30"/>
+      <x:c r="Z9" s="30"/>
     </x:row>
     <x:row r="10">
       <x:c r="C10" s="28"/>
@@ -15759,6 +15891,10 @@
       <x:c r="G10" s="28"/>
       <x:c r="H10" s="28"/>
       <x:c r="S10" s="36"/>
+      <x:c r="T10" s="30"/>
+      <x:c r="U10" s="30"/>
+      <x:c r="V10" s="30"/>
+      <x:c r="Z10" s="30"/>
     </x:row>
     <x:row r="11">
       <x:c r="C11" s="28"/>
@@ -15766,6 +15902,10 @@
       <x:c r="G11" s="28"/>
       <x:c r="H11" s="28"/>
       <x:c r="S11" s="36"/>
+      <x:c r="T11" s="30"/>
+      <x:c r="U11" s="30"/>
+      <x:c r="V11" s="30"/>
+      <x:c r="Z11" s="30"/>
     </x:row>
     <x:row r="12">
       <x:c r="C12" s="28"/>
@@ -15773,6 +15913,10 @@
       <x:c r="G12" s="28"/>
       <x:c r="H12" s="28"/>
       <x:c r="S12" s="36"/>
+      <x:c r="T12" s="30"/>
+      <x:c r="U12" s="30"/>
+      <x:c r="V12" s="30"/>
+      <x:c r="Z12" s="30"/>
     </x:row>
     <x:row r="13">
       <x:c r="C13" s="28"/>
@@ -15780,6 +15924,10 @@
       <x:c r="G13" s="28"/>
       <x:c r="H13" s="28"/>
       <x:c r="S13" s="36"/>
+      <x:c r="T13" s="30"/>
+      <x:c r="U13" s="30"/>
+      <x:c r="V13" s="30"/>
+      <x:c r="Z13" s="30"/>
     </x:row>
     <x:row r="14">
       <x:c r="C14" s="28"/>
@@ -15787,6 +15935,10 @@
       <x:c r="G14" s="28"/>
       <x:c r="H14" s="28"/>
       <x:c r="S14" s="36"/>
+      <x:c r="T14" s="30"/>
+      <x:c r="U14" s="30"/>
+      <x:c r="V14" s="30"/>
+      <x:c r="Z14" s="30"/>
     </x:row>
     <x:row r="15">
       <x:c r="C15" s="28"/>
@@ -15794,6 +15946,10 @@
       <x:c r="G15" s="28"/>
       <x:c r="H15" s="28"/>
       <x:c r="S15" s="36"/>
+      <x:c r="T15" s="30"/>
+      <x:c r="U15" s="30"/>
+      <x:c r="V15" s="30"/>
+      <x:c r="Z15" s="30"/>
     </x:row>
     <x:row r="16">
       <x:c r="C16" s="28"/>
@@ -15801,6 +15957,10 @@
       <x:c r="G16" s="28"/>
       <x:c r="H16" s="28"/>
       <x:c r="S16" s="36"/>
+      <x:c r="T16" s="30"/>
+      <x:c r="U16" s="30"/>
+      <x:c r="V16" s="30"/>
+      <x:c r="Z16" s="30"/>
     </x:row>
     <x:row r="17">
       <x:c r="C17" s="28"/>
@@ -15808,6 +15968,10 @@
       <x:c r="G17" s="28"/>
       <x:c r="H17" s="28"/>
       <x:c r="S17" s="36"/>
+      <x:c r="T17" s="30"/>
+      <x:c r="U17" s="30"/>
+      <x:c r="V17" s="30"/>
+      <x:c r="Z17" s="30"/>
     </x:row>
     <x:row r="18">
       <x:c r="C18" s="28"/>
@@ -15815,6 +15979,10 @@
       <x:c r="G18" s="28"/>
       <x:c r="H18" s="28"/>
       <x:c r="S18" s="36"/>
+      <x:c r="T18" s="30"/>
+      <x:c r="U18" s="30"/>
+      <x:c r="V18" s="30"/>
+      <x:c r="Z18" s="30"/>
     </x:row>
     <x:row r="19">
       <x:c r="C19" s="28"/>
@@ -15822,6 +15990,10 @@
       <x:c r="G19" s="28"/>
       <x:c r="H19" s="28"/>
       <x:c r="S19" s="36"/>
+      <x:c r="T19" s="30"/>
+      <x:c r="U19" s="30"/>
+      <x:c r="V19" s="30"/>
+      <x:c r="Z19" s="30"/>
     </x:row>
     <x:row r="20">
       <x:c r="C20" s="28"/>
@@ -15829,6 +16001,10 @@
       <x:c r="G20" s="28"/>
       <x:c r="H20" s="28"/>
       <x:c r="S20" s="36"/>
+      <x:c r="T20" s="30"/>
+      <x:c r="U20" s="30"/>
+      <x:c r="V20" s="30"/>
+      <x:c r="Z20" s="30"/>
     </x:row>
     <x:row r="21">
       <x:c r="C21" s="28"/>
@@ -15836,6 +16012,10 @@
       <x:c r="G21" s="28"/>
       <x:c r="H21" s="28"/>
       <x:c r="S21" s="36"/>
+      <x:c r="T21" s="30"/>
+      <x:c r="U21" s="30"/>
+      <x:c r="V21" s="30"/>
+      <x:c r="Z21" s="30"/>
     </x:row>
     <x:row r="22">
       <x:c r="C22" s="28"/>
@@ -15843,6 +16023,10 @@
       <x:c r="G22" s="28"/>
       <x:c r="H22" s="28"/>
       <x:c r="S22" s="36"/>
+      <x:c r="T22" s="30"/>
+      <x:c r="U22" s="30"/>
+      <x:c r="V22" s="30"/>
+      <x:c r="Z22" s="30"/>
     </x:row>
     <x:row r="23">
       <x:c r="C23" s="28"/>
@@ -15850,6 +16034,10 @@
       <x:c r="G23" s="28"/>
       <x:c r="H23" s="28"/>
       <x:c r="S23" s="36"/>
+      <x:c r="T23" s="30"/>
+      <x:c r="U23" s="30"/>
+      <x:c r="V23" s="30"/>
+      <x:c r="Z23" s="30"/>
     </x:row>
     <x:row r="24">
       <x:c r="C24" s="28"/>
@@ -15857,6 +16045,10 @@
       <x:c r="G24" s="28"/>
       <x:c r="H24" s="28"/>
       <x:c r="S24" s="36"/>
+      <x:c r="T24" s="30"/>
+      <x:c r="U24" s="30"/>
+      <x:c r="V24" s="30"/>
+      <x:c r="Z24" s="30"/>
     </x:row>
     <x:row r="25">
       <x:c r="C25" s="28"/>
@@ -15864,6 +16056,10 @@
       <x:c r="G25" s="28"/>
       <x:c r="H25" s="28"/>
       <x:c r="S25" s="36"/>
+      <x:c r="T25" s="30"/>
+      <x:c r="U25" s="30"/>
+      <x:c r="V25" s="30"/>
+      <x:c r="Z25" s="30"/>
     </x:row>
     <x:row r="26">
       <x:c r="C26" s="28"/>
@@ -15871,6 +16067,10 @@
       <x:c r="G26" s="28"/>
       <x:c r="H26" s="28"/>
       <x:c r="S26" s="36"/>
+      <x:c r="T26" s="30"/>
+      <x:c r="U26" s="30"/>
+      <x:c r="V26" s="30"/>
+      <x:c r="Z26" s="30"/>
     </x:row>
     <x:row r="27">
       <x:c r="C27" s="28"/>
@@ -15878,6 +16078,10 @@
       <x:c r="G27" s="28"/>
       <x:c r="H27" s="28"/>
       <x:c r="S27" s="36"/>
+      <x:c r="T27" s="30"/>
+      <x:c r="U27" s="30"/>
+      <x:c r="V27" s="30"/>
+      <x:c r="Z27" s="30"/>
     </x:row>
     <x:row r="28">
       <x:c r="C28" s="28"/>
@@ -15885,6 +16089,10 @@
       <x:c r="G28" s="28"/>
       <x:c r="H28" s="28"/>
       <x:c r="S28" s="36"/>
+      <x:c r="T28" s="30"/>
+      <x:c r="U28" s="30"/>
+      <x:c r="V28" s="30"/>
+      <x:c r="Z28" s="30"/>
     </x:row>
     <x:row r="29">
       <x:c r="C29" s="28"/>
@@ -15892,6 +16100,10 @@
       <x:c r="G29" s="28"/>
       <x:c r="H29" s="28"/>
       <x:c r="S29" s="36"/>
+      <x:c r="T29" s="30"/>
+      <x:c r="U29" s="30"/>
+      <x:c r="V29" s="30"/>
+      <x:c r="Z29" s="30"/>
     </x:row>
     <x:row r="30">
       <x:c r="C30" s="28"/>
@@ -15899,6 +16111,10 @@
       <x:c r="G30" s="28"/>
       <x:c r="H30" s="28"/>
       <x:c r="S30" s="36"/>
+      <x:c r="T30" s="30"/>
+      <x:c r="U30" s="30"/>
+      <x:c r="V30" s="30"/>
+      <x:c r="Z30" s="30"/>
     </x:row>
     <x:row r="31">
       <x:c r="C31" s="28"/>
@@ -15906,6 +16122,10 @@
       <x:c r="G31" s="28"/>
       <x:c r="H31" s="28"/>
       <x:c r="S31" s="36"/>
+      <x:c r="T31" s="30"/>
+      <x:c r="U31" s="30"/>
+      <x:c r="V31" s="30"/>
+      <x:c r="Z31" s="30"/>
     </x:row>
     <x:row r="32">
       <x:c r="C32" s="28"/>
@@ -15913,6 +16133,10 @@
       <x:c r="G32" s="28"/>
       <x:c r="H32" s="28"/>
       <x:c r="S32" s="36"/>
+      <x:c r="T32" s="30"/>
+      <x:c r="U32" s="30"/>
+      <x:c r="V32" s="30"/>
+      <x:c r="Z32" s="30"/>
     </x:row>
     <x:row r="33">
       <x:c r="C33" s="28"/>
@@ -15920,6 +16144,10 @@
       <x:c r="G33" s="28"/>
       <x:c r="H33" s="28"/>
       <x:c r="S33" s="36"/>
+      <x:c r="T33" s="30"/>
+      <x:c r="U33" s="30"/>
+      <x:c r="V33" s="30"/>
+      <x:c r="Z33" s="30"/>
     </x:row>
     <x:row r="34">
       <x:c r="C34" s="28"/>
@@ -15927,6 +16155,10 @@
       <x:c r="G34" s="28"/>
       <x:c r="H34" s="28"/>
       <x:c r="S34" s="36"/>
+      <x:c r="T34" s="30"/>
+      <x:c r="U34" s="30"/>
+      <x:c r="V34" s="30"/>
+      <x:c r="Z34" s="30"/>
     </x:row>
     <x:row r="35">
       <x:c r="C35" s="28"/>
@@ -15934,6 +16166,10 @@
       <x:c r="G35" s="28"/>
       <x:c r="H35" s="28"/>
       <x:c r="S35" s="36"/>
+      <x:c r="T35" s="30"/>
+      <x:c r="U35" s="30"/>
+      <x:c r="V35" s="30"/>
+      <x:c r="Z35" s="30"/>
     </x:row>
     <x:row r="36">
       <x:c r="C36" s="28"/>
@@ -15941,6 +16177,10 @@
       <x:c r="G36" s="28"/>
       <x:c r="H36" s="28"/>
       <x:c r="S36" s="36"/>
+      <x:c r="T36" s="30"/>
+      <x:c r="U36" s="30"/>
+      <x:c r="V36" s="30"/>
+      <x:c r="Z36" s="30"/>
     </x:row>
     <x:row r="37">
       <x:c r="C37" s="28"/>
@@ -15948,6 +16188,10 @@
       <x:c r="G37" s="28"/>
       <x:c r="H37" s="28"/>
       <x:c r="S37" s="36"/>
+      <x:c r="T37" s="30"/>
+      <x:c r="U37" s="30"/>
+      <x:c r="V37" s="30"/>
+      <x:c r="Z37" s="30"/>
     </x:row>
     <x:row r="38">
       <x:c r="C38" s="28"/>
@@ -15955,6 +16199,10 @@
       <x:c r="G38" s="28"/>
       <x:c r="H38" s="28"/>
       <x:c r="S38" s="36"/>
+      <x:c r="T38" s="30"/>
+      <x:c r="U38" s="30"/>
+      <x:c r="V38" s="30"/>
+      <x:c r="Z38" s="30"/>
     </x:row>
     <x:row r="39">
       <x:c r="C39" s="28"/>
@@ -15962,6 +16210,10 @@
       <x:c r="G39" s="28"/>
       <x:c r="H39" s="28"/>
       <x:c r="S39" s="36"/>
+      <x:c r="T39" s="30"/>
+      <x:c r="U39" s="30"/>
+      <x:c r="V39" s="30"/>
+      <x:c r="Z39" s="30"/>
     </x:row>
     <x:row r="40">
       <x:c r="C40" s="28"/>
@@ -15969,6 +16221,10 @@
       <x:c r="G40" s="28"/>
       <x:c r="H40" s="28"/>
       <x:c r="S40" s="36"/>
+      <x:c r="T40" s="30"/>
+      <x:c r="U40" s="30"/>
+      <x:c r="V40" s="30"/>
+      <x:c r="Z40" s="30"/>
     </x:row>
     <x:row r="41">
       <x:c r="C41" s="28"/>
@@ -15976,6 +16232,10 @@
       <x:c r="G41" s="28"/>
       <x:c r="H41" s="28"/>
       <x:c r="S41" s="36"/>
+      <x:c r="T41" s="30"/>
+      <x:c r="U41" s="30"/>
+      <x:c r="V41" s="30"/>
+      <x:c r="Z41" s="30"/>
     </x:row>
     <x:row r="42">
       <x:c r="C42" s="28"/>
@@ -15983,6 +16243,10 @@
       <x:c r="G42" s="28"/>
       <x:c r="H42" s="28"/>
       <x:c r="S42" s="36"/>
+      <x:c r="T42" s="30"/>
+      <x:c r="U42" s="30"/>
+      <x:c r="V42" s="30"/>
+      <x:c r="Z42" s="30"/>
     </x:row>
     <x:row r="43">
       <x:c r="C43" s="28"/>
@@ -15990,6 +16254,10 @@
       <x:c r="G43" s="28"/>
       <x:c r="H43" s="28"/>
       <x:c r="S43" s="36"/>
+      <x:c r="T43" s="30"/>
+      <x:c r="U43" s="30"/>
+      <x:c r="V43" s="30"/>
+      <x:c r="Z43" s="30"/>
     </x:row>
     <x:row r="44">
       <x:c r="C44" s="28"/>
@@ -15997,6 +16265,10 @@
       <x:c r="G44" s="28"/>
       <x:c r="H44" s="28"/>
       <x:c r="S44" s="36"/>
+      <x:c r="T44" s="30"/>
+      <x:c r="U44" s="30"/>
+      <x:c r="V44" s="30"/>
+      <x:c r="Z44" s="30"/>
     </x:row>
     <x:row r="45">
       <x:c r="C45" s="28"/>
@@ -16004,6 +16276,10 @@
       <x:c r="G45" s="28"/>
       <x:c r="H45" s="28"/>
       <x:c r="S45" s="36"/>
+      <x:c r="T45" s="30"/>
+      <x:c r="U45" s="30"/>
+      <x:c r="V45" s="30"/>
+      <x:c r="Z45" s="30"/>
     </x:row>
     <x:row r="46">
       <x:c r="C46" s="28"/>
@@ -16011,6 +16287,10 @@
       <x:c r="G46" s="28"/>
       <x:c r="H46" s="28"/>
       <x:c r="S46" s="36"/>
+      <x:c r="T46" s="30"/>
+      <x:c r="U46" s="30"/>
+      <x:c r="V46" s="30"/>
+      <x:c r="Z46" s="30"/>
     </x:row>
     <x:row r="47">
       <x:c r="C47" s="28"/>
@@ -16018,6 +16298,10 @@
       <x:c r="G47" s="28"/>
       <x:c r="H47" s="28"/>
       <x:c r="S47" s="36"/>
+      <x:c r="T47" s="30"/>
+      <x:c r="U47" s="30"/>
+      <x:c r="V47" s="30"/>
+      <x:c r="Z47" s="30"/>
     </x:row>
     <x:row r="48">
       <x:c r="C48" s="28"/>
@@ -16025,6 +16309,10 @@
       <x:c r="G48" s="28"/>
       <x:c r="H48" s="28"/>
       <x:c r="S48" s="36"/>
+      <x:c r="T48" s="30"/>
+      <x:c r="U48" s="30"/>
+      <x:c r="V48" s="30"/>
+      <x:c r="Z48" s="30"/>
     </x:row>
     <x:row r="49">
       <x:c r="C49" s="28"/>
@@ -16032,6 +16320,10 @@
       <x:c r="G49" s="28"/>
       <x:c r="H49" s="28"/>
       <x:c r="S49" s="36"/>
+      <x:c r="T49" s="30"/>
+      <x:c r="U49" s="30"/>
+      <x:c r="V49" s="30"/>
+      <x:c r="Z49" s="30"/>
     </x:row>
     <x:row r="50">
       <x:c r="C50" s="28"/>
@@ -16039,6 +16331,10 @@
       <x:c r="G50" s="28"/>
       <x:c r="H50" s="28"/>
       <x:c r="S50" s="36"/>
+      <x:c r="T50" s="30"/>
+      <x:c r="U50" s="30"/>
+      <x:c r="V50" s="30"/>
+      <x:c r="Z50" s="30"/>
     </x:row>
     <x:row r="51">
       <x:c r="C51" s="28"/>
@@ -16046,6 +16342,10 @@
       <x:c r="G51" s="28"/>
       <x:c r="H51" s="28"/>
       <x:c r="S51" s="36"/>
+      <x:c r="T51" s="30"/>
+      <x:c r="U51" s="30"/>
+      <x:c r="V51" s="30"/>
+      <x:c r="Z51" s="30"/>
     </x:row>
     <x:row r="52">
       <x:c r="C52" s="28"/>
@@ -16053,6 +16353,10 @@
       <x:c r="G52" s="28"/>
       <x:c r="H52" s="28"/>
       <x:c r="S52" s="36"/>
+      <x:c r="T52" s="30"/>
+      <x:c r="U52" s="30"/>
+      <x:c r="V52" s="30"/>
+      <x:c r="Z52" s="30"/>
     </x:row>
     <x:row r="53">
       <x:c r="C53" s="28"/>
@@ -16060,6 +16364,10 @@
       <x:c r="G53" s="28"/>
       <x:c r="H53" s="28"/>
       <x:c r="S53" s="36"/>
+      <x:c r="T53" s="30"/>
+      <x:c r="U53" s="30"/>
+      <x:c r="V53" s="30"/>
+      <x:c r="Z53" s="30"/>
     </x:row>
     <x:row r="54">
       <x:c r="C54" s="28"/>
@@ -16067,6 +16375,10 @@
       <x:c r="G54" s="28"/>
       <x:c r="H54" s="28"/>
       <x:c r="S54" s="36"/>
+      <x:c r="T54" s="30"/>
+      <x:c r="U54" s="30"/>
+      <x:c r="V54" s="30"/>
+      <x:c r="Z54" s="30"/>
     </x:row>
     <x:row r="55">
       <x:c r="C55" s="28"/>
@@ -16074,6 +16386,10 @@
       <x:c r="G55" s="28"/>
       <x:c r="H55" s="28"/>
       <x:c r="S55" s="36"/>
+      <x:c r="T55" s="30"/>
+      <x:c r="U55" s="30"/>
+      <x:c r="V55" s="30"/>
+      <x:c r="Z55" s="30"/>
     </x:row>
     <x:row r="56">
       <x:c r="C56" s="28"/>
@@ -16081,6 +16397,10 @@
       <x:c r="G56" s="28"/>
       <x:c r="H56" s="28"/>
       <x:c r="S56" s="36"/>
+      <x:c r="T56" s="30"/>
+      <x:c r="U56" s="30"/>
+      <x:c r="V56" s="30"/>
+      <x:c r="Z56" s="30"/>
     </x:row>
     <x:row r="57">
       <x:c r="C57" s="28"/>
@@ -16088,6 +16408,10 @@
       <x:c r="G57" s="28"/>
       <x:c r="H57" s="28"/>
       <x:c r="S57" s="36"/>
+      <x:c r="T57" s="30"/>
+      <x:c r="U57" s="30"/>
+      <x:c r="V57" s="30"/>
+      <x:c r="Z57" s="30"/>
     </x:row>
     <x:row r="58">
       <x:c r="C58" s="28"/>
@@ -16095,6 +16419,10 @@
       <x:c r="G58" s="28"/>
       <x:c r="H58" s="28"/>
       <x:c r="S58" s="36"/>
+      <x:c r="T58" s="30"/>
+      <x:c r="U58" s="30"/>
+      <x:c r="V58" s="30"/>
+      <x:c r="Z58" s="30"/>
     </x:row>
     <x:row r="59">
       <x:c r="C59" s="28"/>
@@ -16102,6 +16430,10 @@
       <x:c r="G59" s="28"/>
       <x:c r="H59" s="28"/>
       <x:c r="S59" s="36"/>
+      <x:c r="T59" s="30"/>
+      <x:c r="U59" s="30"/>
+      <x:c r="V59" s="30"/>
+      <x:c r="Z59" s="30"/>
     </x:row>
     <x:row r="60">
       <x:c r="C60" s="28"/>
@@ -16109,6 +16441,10 @@
       <x:c r="G60" s="28"/>
       <x:c r="H60" s="28"/>
       <x:c r="S60" s="36"/>
+      <x:c r="T60" s="30"/>
+      <x:c r="U60" s="30"/>
+      <x:c r="V60" s="30"/>
+      <x:c r="Z60" s="30"/>
     </x:row>
     <x:row r="61">
       <x:c r="C61" s="28"/>
@@ -16116,6 +16452,10 @@
       <x:c r="G61" s="28"/>
       <x:c r="H61" s="28"/>
       <x:c r="S61" s="36"/>
+      <x:c r="T61" s="30"/>
+      <x:c r="U61" s="30"/>
+      <x:c r="V61" s="30"/>
+      <x:c r="Z61" s="30"/>
     </x:row>
     <x:row r="62">
       <x:c r="C62" s="28"/>
@@ -16123,6 +16463,10 @@
       <x:c r="G62" s="28"/>
       <x:c r="H62" s="28"/>
       <x:c r="S62" s="36"/>
+      <x:c r="T62" s="30"/>
+      <x:c r="U62" s="30"/>
+      <x:c r="V62" s="30"/>
+      <x:c r="Z62" s="30"/>
     </x:row>
     <x:row r="63">
       <x:c r="C63" s="28"/>
@@ -16130,6 +16474,10 @@
       <x:c r="G63" s="28"/>
       <x:c r="H63" s="28"/>
       <x:c r="S63" s="36"/>
+      <x:c r="T63" s="30"/>
+      <x:c r="U63" s="30"/>
+      <x:c r="V63" s="30"/>
+      <x:c r="Z63" s="30"/>
     </x:row>
     <x:row r="64">
       <x:c r="C64" s="28"/>
@@ -16137,6 +16485,10 @@
       <x:c r="G64" s="28"/>
       <x:c r="H64" s="28"/>
       <x:c r="S64" s="36"/>
+      <x:c r="T64" s="30"/>
+      <x:c r="U64" s="30"/>
+      <x:c r="V64" s="30"/>
+      <x:c r="Z64" s="30"/>
     </x:row>
     <x:row r="65">
       <x:c r="C65" s="28"/>
@@ -16144,6 +16496,10 @@
       <x:c r="G65" s="28"/>
       <x:c r="H65" s="28"/>
       <x:c r="S65" s="36"/>
+      <x:c r="T65" s="30"/>
+      <x:c r="U65" s="30"/>
+      <x:c r="V65" s="30"/>
+      <x:c r="Z65" s="30"/>
     </x:row>
     <x:row r="66">
       <x:c r="C66" s="28"/>
@@ -16151,6 +16507,10 @@
       <x:c r="G66" s="28"/>
       <x:c r="H66" s="28"/>
       <x:c r="S66" s="36"/>
+      <x:c r="T66" s="30"/>
+      <x:c r="U66" s="30"/>
+      <x:c r="V66" s="30"/>
+      <x:c r="Z66" s="30"/>
     </x:row>
     <x:row r="67">
       <x:c r="C67" s="28"/>
@@ -16158,6 +16518,10 @@
       <x:c r="G67" s="28"/>
       <x:c r="H67" s="28"/>
       <x:c r="S67" s="36"/>
+      <x:c r="T67" s="30"/>
+      <x:c r="U67" s="30"/>
+      <x:c r="V67" s="30"/>
+      <x:c r="Z67" s="30"/>
     </x:row>
     <x:row r="68">
       <x:c r="C68" s="28"/>
@@ -16165,6 +16529,10 @@
       <x:c r="G68" s="28"/>
       <x:c r="H68" s="28"/>
       <x:c r="S68" s="36"/>
+      <x:c r="T68" s="30"/>
+      <x:c r="U68" s="30"/>
+      <x:c r="V68" s="30"/>
+      <x:c r="Z68" s="30"/>
     </x:row>
     <x:row r="69">
       <x:c r="C69" s="28"/>
@@ -16172,6 +16540,10 @@
       <x:c r="G69" s="28"/>
       <x:c r="H69" s="28"/>
       <x:c r="S69" s="36"/>
+      <x:c r="T69" s="30"/>
+      <x:c r="U69" s="30"/>
+      <x:c r="V69" s="30"/>
+      <x:c r="Z69" s="30"/>
     </x:row>
     <x:row r="70">
       <x:c r="C70" s="28"/>
@@ -16179,6 +16551,10 @@
       <x:c r="G70" s="28"/>
       <x:c r="H70" s="28"/>
       <x:c r="S70" s="36"/>
+      <x:c r="T70" s="30"/>
+      <x:c r="U70" s="30"/>
+      <x:c r="V70" s="30"/>
+      <x:c r="Z70" s="30"/>
     </x:row>
     <x:row r="71">
       <x:c r="C71" s="28"/>
@@ -16186,6 +16562,10 @@
       <x:c r="G71" s="28"/>
       <x:c r="H71" s="28"/>
       <x:c r="S71" s="36"/>
+      <x:c r="T71" s="30"/>
+      <x:c r="U71" s="30"/>
+      <x:c r="V71" s="30"/>
+      <x:c r="Z71" s="30"/>
     </x:row>
     <x:row r="72">
       <x:c r="C72" s="28"/>
@@ -16193,6 +16573,10 @@
       <x:c r="G72" s="28"/>
       <x:c r="H72" s="28"/>
       <x:c r="S72" s="36"/>
+      <x:c r="T72" s="30"/>
+      <x:c r="U72" s="30"/>
+      <x:c r="V72" s="30"/>
+      <x:c r="Z72" s="30"/>
     </x:row>
     <x:row r="73">
       <x:c r="C73" s="28"/>
@@ -16200,6 +16584,10 @@
       <x:c r="G73" s="28"/>
       <x:c r="H73" s="28"/>
       <x:c r="S73" s="36"/>
+      <x:c r="T73" s="30"/>
+      <x:c r="U73" s="30"/>
+      <x:c r="V73" s="30"/>
+      <x:c r="Z73" s="30"/>
     </x:row>
     <x:row r="74">
       <x:c r="C74" s="28"/>
@@ -16207,6 +16595,10 @@
       <x:c r="G74" s="28"/>
       <x:c r="H74" s="28"/>
       <x:c r="S74" s="36"/>
+      <x:c r="T74" s="30"/>
+      <x:c r="U74" s="30"/>
+      <x:c r="V74" s="30"/>
+      <x:c r="Z74" s="30"/>
     </x:row>
     <x:row r="75">
       <x:c r="C75" s="28"/>
@@ -16214,6 +16606,10 @@
       <x:c r="G75" s="28"/>
       <x:c r="H75" s="28"/>
       <x:c r="S75" s="36"/>
+      <x:c r="T75" s="30"/>
+      <x:c r="U75" s="30"/>
+      <x:c r="V75" s="30"/>
+      <x:c r="Z75" s="30"/>
     </x:row>
     <x:row r="76">
       <x:c r="C76" s="28"/>
@@ -16221,6 +16617,10 @@
       <x:c r="G76" s="28"/>
       <x:c r="H76" s="28"/>
       <x:c r="S76" s="36"/>
+      <x:c r="T76" s="30"/>
+      <x:c r="U76" s="30"/>
+      <x:c r="V76" s="30"/>
+      <x:c r="Z76" s="30"/>
     </x:row>
     <x:row r="77">
       <x:c r="C77" s="28"/>
@@ -16228,6 +16628,10 @@
       <x:c r="G77" s="28"/>
       <x:c r="H77" s="28"/>
       <x:c r="S77" s="36"/>
+      <x:c r="T77" s="30"/>
+      <x:c r="U77" s="30"/>
+      <x:c r="V77" s="30"/>
+      <x:c r="Z77" s="30"/>
     </x:row>
     <x:row r="78">
       <x:c r="C78" s="28"/>
@@ -16235,6 +16639,10 @@
       <x:c r="G78" s="28"/>
       <x:c r="H78" s="28"/>
       <x:c r="S78" s="36"/>
+      <x:c r="T78" s="30"/>
+      <x:c r="U78" s="30"/>
+      <x:c r="V78" s="30"/>
+      <x:c r="Z78" s="30"/>
     </x:row>
     <x:row r="79">
       <x:c r="C79" s="28"/>
@@ -16242,6 +16650,10 @@
       <x:c r="G79" s="28"/>
       <x:c r="H79" s="28"/>
       <x:c r="S79" s="36"/>
+      <x:c r="T79" s="30"/>
+      <x:c r="U79" s="30"/>
+      <x:c r="V79" s="30"/>
+      <x:c r="Z79" s="30"/>
     </x:row>
     <x:row r="80">
       <x:c r="C80" s="28"/>
@@ -16249,6 +16661,10 @@
       <x:c r="G80" s="28"/>
       <x:c r="H80" s="28"/>
       <x:c r="S80" s="36"/>
+      <x:c r="T80" s="30"/>
+      <x:c r="U80" s="30"/>
+      <x:c r="V80" s="30"/>
+      <x:c r="Z80" s="30"/>
     </x:row>
     <x:row r="81">
       <x:c r="C81" s="28"/>
@@ -16256,6 +16672,10 @@
       <x:c r="G81" s="28"/>
       <x:c r="H81" s="28"/>
       <x:c r="S81" s="36"/>
+      <x:c r="T81" s="30"/>
+      <x:c r="U81" s="30"/>
+      <x:c r="V81" s="30"/>
+      <x:c r="Z81" s="30"/>
     </x:row>
     <x:row r="82">
       <x:c r="C82" s="28"/>
@@ -16263,6 +16683,10 @@
       <x:c r="G82" s="28"/>
       <x:c r="H82" s="28"/>
       <x:c r="S82" s="36"/>
+      <x:c r="T82" s="30"/>
+      <x:c r="U82" s="30"/>
+      <x:c r="V82" s="30"/>
+      <x:c r="Z82" s="30"/>
     </x:row>
     <x:row r="83">
       <x:c r="C83" s="28"/>
@@ -16270,6 +16694,10 @@
       <x:c r="G83" s="28"/>
       <x:c r="H83" s="28"/>
       <x:c r="S83" s="36"/>
+      <x:c r="T83" s="30"/>
+      <x:c r="U83" s="30"/>
+      <x:c r="V83" s="30"/>
+      <x:c r="Z83" s="30"/>
     </x:row>
     <x:row r="84">
       <x:c r="C84" s="28"/>
@@ -16277,6 +16705,10 @@
       <x:c r="G84" s="28"/>
       <x:c r="H84" s="28"/>
       <x:c r="S84" s="36"/>
+      <x:c r="T84" s="30"/>
+      <x:c r="U84" s="30"/>
+      <x:c r="V84" s="30"/>
+      <x:c r="Z84" s="30"/>
     </x:row>
     <x:row r="85">
       <x:c r="C85" s="28"/>
@@ -16284,6 +16716,10 @@
       <x:c r="G85" s="28"/>
       <x:c r="H85" s="28"/>
       <x:c r="S85" s="36"/>
+      <x:c r="T85" s="30"/>
+      <x:c r="U85" s="30"/>
+      <x:c r="V85" s="30"/>
+      <x:c r="Z85" s="30"/>
     </x:row>
     <x:row r="86">
       <x:c r="C86" s="28"/>
@@ -16291,6 +16727,10 @@
       <x:c r="G86" s="28"/>
       <x:c r="H86" s="28"/>
       <x:c r="S86" s="36"/>
+      <x:c r="T86" s="30"/>
+      <x:c r="U86" s="30"/>
+      <x:c r="V86" s="30"/>
+      <x:c r="Z86" s="30"/>
     </x:row>
     <x:row r="87">
       <x:c r="C87" s="28"/>
@@ -16298,6 +16738,10 @@
       <x:c r="G87" s="28"/>
       <x:c r="H87" s="28"/>
       <x:c r="S87" s="36"/>
+      <x:c r="T87" s="30"/>
+      <x:c r="U87" s="30"/>
+      <x:c r="V87" s="30"/>
+      <x:c r="Z87" s="30"/>
     </x:row>
     <x:row r="88">
       <x:c r="C88" s="28"/>
@@ -16305,6 +16749,10 @@
       <x:c r="G88" s="28"/>
       <x:c r="H88" s="28"/>
       <x:c r="S88" s="36"/>
+      <x:c r="T88" s="30"/>
+      <x:c r="U88" s="30"/>
+      <x:c r="V88" s="30"/>
+      <x:c r="Z88" s="30"/>
     </x:row>
     <x:row r="89">
       <x:c r="C89" s="28"/>
@@ -16312,6 +16760,10 @@
       <x:c r="G89" s="28"/>
       <x:c r="H89" s="28"/>
       <x:c r="S89" s="36"/>
+      <x:c r="T89" s="30"/>
+      <x:c r="U89" s="30"/>
+      <x:c r="V89" s="30"/>
+      <x:c r="Z89" s="30"/>
     </x:row>
     <x:row r="90">
       <x:c r="C90" s="28"/>
@@ -16319,6 +16771,10 @@
       <x:c r="G90" s="28"/>
       <x:c r="H90" s="28"/>
       <x:c r="S90" s="36"/>
+      <x:c r="T90" s="30"/>
+      <x:c r="U90" s="30"/>
+      <x:c r="V90" s="30"/>
+      <x:c r="Z90" s="30"/>
     </x:row>
     <x:row r="91">
       <x:c r="C91" s="28"/>
@@ -16326,6 +16782,10 @@
       <x:c r="G91" s="28"/>
       <x:c r="H91" s="28"/>
       <x:c r="S91" s="36"/>
+      <x:c r="T91" s="30"/>
+      <x:c r="U91" s="30"/>
+      <x:c r="V91" s="30"/>
+      <x:c r="Z91" s="30"/>
     </x:row>
     <x:row r="92">
       <x:c r="C92" s="28"/>
@@ -16333,6 +16793,10 @@
       <x:c r="G92" s="28"/>
       <x:c r="H92" s="28"/>
       <x:c r="S92" s="36"/>
+      <x:c r="T92" s="30"/>
+      <x:c r="U92" s="30"/>
+      <x:c r="V92" s="30"/>
+      <x:c r="Z92" s="30"/>
     </x:row>
     <x:row r="93">
       <x:c r="C93" s="28"/>
@@ -16340,6 +16804,10 @@
       <x:c r="G93" s="28"/>
       <x:c r="H93" s="28"/>
       <x:c r="S93" s="36"/>
+      <x:c r="T93" s="30"/>
+      <x:c r="U93" s="30"/>
+      <x:c r="V93" s="30"/>
+      <x:c r="Z93" s="30"/>
     </x:row>
     <x:row r="94">
       <x:c r="C94" s="28"/>
@@ -16347,6 +16815,10 @@
       <x:c r="G94" s="28"/>
       <x:c r="H94" s="28"/>
       <x:c r="S94" s="36"/>
+      <x:c r="T94" s="30"/>
+      <x:c r="U94" s="30"/>
+      <x:c r="V94" s="30"/>
+      <x:c r="Z94" s="30"/>
     </x:row>
     <x:row r="95">
       <x:c r="C95" s="28"/>
@@ -16354,6 +16826,10 @@
       <x:c r="G95" s="28"/>
       <x:c r="H95" s="28"/>
       <x:c r="S95" s="36"/>
+      <x:c r="T95" s="30"/>
+      <x:c r="U95" s="30"/>
+      <x:c r="V95" s="30"/>
+      <x:c r="Z95" s="30"/>
     </x:row>
     <x:row r="96">
       <x:c r="C96" s="28"/>
@@ -16361,6 +16837,10 @@
       <x:c r="G96" s="28"/>
       <x:c r="H96" s="28"/>
       <x:c r="S96" s="36"/>
+      <x:c r="T96" s="30"/>
+      <x:c r="U96" s="30"/>
+      <x:c r="V96" s="30"/>
+      <x:c r="Z96" s="30"/>
     </x:row>
     <x:row r="97">
       <x:c r="C97" s="28"/>
@@ -16368,6 +16848,10 @@
       <x:c r="G97" s="28"/>
       <x:c r="H97" s="28"/>
       <x:c r="S97" s="36"/>
+      <x:c r="T97" s="30"/>
+      <x:c r="U97" s="30"/>
+      <x:c r="V97" s="30"/>
+      <x:c r="Z97" s="30"/>
     </x:row>
     <x:row r="98">
       <x:c r="C98" s="28"/>
@@ -16375,6 +16859,10 @@
       <x:c r="G98" s="28"/>
       <x:c r="H98" s="28"/>
       <x:c r="S98" s="36"/>
+      <x:c r="T98" s="30"/>
+      <x:c r="U98" s="30"/>
+      <x:c r="V98" s="30"/>
+      <x:c r="Z98" s="30"/>
     </x:row>
     <x:row r="99">
       <x:c r="C99" s="28"/>
@@ -16382,6 +16870,10 @@
       <x:c r="G99" s="28"/>
       <x:c r="H99" s="28"/>
       <x:c r="S99" s="36"/>
+      <x:c r="T99" s="30"/>
+      <x:c r="U99" s="30"/>
+      <x:c r="V99" s="30"/>
+      <x:c r="Z99" s="30"/>
     </x:row>
     <x:row r="100">
       <x:c r="C100" s="28"/>
@@ -16389,6 +16881,10 @@
       <x:c r="G100" s="28"/>
       <x:c r="H100" s="28"/>
       <x:c r="S100" s="36"/>
+      <x:c r="T100" s="30"/>
+      <x:c r="U100" s="30"/>
+      <x:c r="V100" s="30"/>
+      <x:c r="Z100" s="30"/>
     </x:row>
     <x:row r="101">
       <x:c r="C101" s="28"/>
@@ -16396,6 +16892,10 @@
       <x:c r="G101" s="28"/>
       <x:c r="H101" s="28"/>
       <x:c r="S101" s="36"/>
+      <x:c r="T101" s="30"/>
+      <x:c r="U101" s="30"/>
+      <x:c r="V101" s="30"/>
+      <x:c r="Z101" s="30"/>
     </x:row>
     <x:row r="102">
       <x:c r="C102" s="28"/>
@@ -16403,6 +16903,10 @@
       <x:c r="G102" s="28"/>
       <x:c r="H102" s="28"/>
       <x:c r="S102" s="36"/>
+      <x:c r="T102" s="30"/>
+      <x:c r="U102" s="30"/>
+      <x:c r="V102" s="30"/>
+      <x:c r="Z102" s="30"/>
     </x:row>
     <x:row r="103">
       <x:c r="C103" s="28"/>
@@ -16410,11 +16914,15 @@
       <x:c r="G103" s="28"/>
       <x:c r="H103" s="28"/>
       <x:c r="S103" s="36"/>
+      <x:c r="T103" s="30"/>
+      <x:c r="U103" s="30"/>
+      <x:c r="V103" s="30"/>
+      <x:c r="Z103" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:S1"/>
-    <x:mergeCell ref="A2:S2"/>
+    <x:mergeCell ref="A1:AA1"/>
+    <x:mergeCell ref="A2:AA2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:A103">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="严格合格"/>
@@ -16428,7 +16936,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc2224aa953646d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R782948ec43cf4d13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17273,7 +17781,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R209a69bfeebd4234"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red416656f75b4361"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>